<commit_message>
small problem with 2023 row in excel
</commit_message>
<xml_diff>
--- a/Manual/MM23_cleaned.xlsx
+++ b/Manual/MM23_cleaned.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/onettperera/Desktop/ADS_Easter/Manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1431497E-338D-8D4C-A679-21A0579E68E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CDD7B3-AF62-0443-8D9E-AC0CF5295008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{B1576BF3-F55A-1D42-85D3-6C766BD046A7}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{B1576BF3-F55A-1D42-85D3-6C766BD046A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly" sheetId="1" r:id="rId1"/>
     <sheet name="Financial Year Averages" sheetId="2" r:id="rId2"/>
+    <sheet name="Financial Year Inflation" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="133">
   <si>
     <t>aggregate number</t>
   </si>
@@ -445,7 +446,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -515,6 +516,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFEAECF0"/>
+      <name val="Courier New"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -767,7 +774,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
@@ -943,6 +950,8 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3"/>
   </cellXfs>
   <cellStyles count="35">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -27585,55 +27594,4579 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FA976F5-DA60-5F43-AF37-C024C9208180}">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:VB25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A1" s="83" t="s">
         <v>132</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="83" t="s">
         <v>118</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="83" t="s">
         <v>119</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="83" t="s">
         <v>120</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="83" t="s">
         <v>121</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="83" t="s">
         <v>122</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="83" t="s">
         <v>123</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="83" t="s">
         <v>124</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="83" t="s">
         <v>125</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="83" t="s">
         <v>126</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="83" t="s">
         <v>128</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="83" t="s">
         <v>129</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="83" t="s">
         <v>130</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="83" t="s">
         <v>131</v>
       </c>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="83"/>
+      <c r="T1" s="83"/>
+      <c r="U1" s="83"/>
+      <c r="V1" s="83"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="83"/>
+      <c r="AF1" s="83"/>
+      <c r="AG1" s="83"/>
+      <c r="AH1" s="83"/>
+    </row>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A2" s="83">
+        <v>2015</v>
+      </c>
+      <c r="B2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!D$4:D$461)</f>
+        <v>100.16549999999999</v>
+      </c>
+      <c r="C2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!E$4:E$461)</f>
+        <v>99.359833333333327</v>
+      </c>
+      <c r="D2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!F$4:F$461)</f>
+        <v>100.27841666666667</v>
+      </c>
+      <c r="E2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!G$4:G$461)</f>
+        <v>100.17075</v>
+      </c>
+      <c r="F2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!H$4:H$461)</f>
+        <v>100.34033333333333</v>
+      </c>
+      <c r="G2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!I$4:I$461)</f>
+        <v>100.0585</v>
+      </c>
+      <c r="H2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!J$4:J$461)</f>
+        <v>100.51175000000002</v>
+      </c>
+      <c r="I2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!K$4:K$461)</f>
+        <v>99.871416666666661</v>
+      </c>
+      <c r="J2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!L$4:L$461)</f>
+        <v>100.47616666666666</v>
+      </c>
+      <c r="K2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!M$4:M$461)</f>
+        <v>99.984166666666681</v>
+      </c>
+      <c r="L2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!N$4:N$461)</f>
+        <v>101.17858333333334</v>
+      </c>
+      <c r="M2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!O$4:O$461)</f>
+        <v>100.46141666666665</v>
+      </c>
+      <c r="N2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!P$4:P$461)</f>
+        <v>100.283</v>
+      </c>
+      <c r="O2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!Q$4:Q$461)</f>
+        <v>100.72233333333334</v>
+      </c>
+      <c r="P2" s="83"/>
+      <c r="Q2" s="83"/>
+      <c r="R2" s="83"/>
+      <c r="S2" s="83"/>
+      <c r="T2" s="83"/>
+      <c r="U2" s="83"/>
+      <c r="V2" s="83"/>
+      <c r="W2" s="83"/>
+      <c r="X2" s="83"/>
+      <c r="Y2" s="83"/>
+      <c r="Z2" s="83"/>
+      <c r="AA2" s="83"/>
+      <c r="AB2" s="83"/>
+      <c r="AC2" s="83"/>
+      <c r="AD2" s="83"/>
+      <c r="AE2" s="83"/>
+      <c r="AF2" s="83"/>
+      <c r="AG2" s="83"/>
+      <c r="AH2" s="83"/>
+    </row>
+    <row r="3" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A3" s="83">
+        <v>2016</v>
+      </c>
+      <c r="B3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!D$4:D$461)</f>
+        <v>101.53616666666665</v>
+      </c>
+      <c r="C3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!E$4:E$461)</f>
+        <v>97.686833333333325</v>
+      </c>
+      <c r="D3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!F$4:F$461)</f>
+        <v>102.32091666666666</v>
+      </c>
+      <c r="E3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!G$4:G$461)</f>
+        <v>100.24566666666668</v>
+      </c>
+      <c r="F3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!H$4:H$461)</f>
+        <v>102.13883333333335</v>
+      </c>
+      <c r="G3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!I$4:I$461)</f>
+        <v>100.10899999999999</v>
+      </c>
+      <c r="H3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!J$4:J$461)</f>
+        <v>102.70283333333333</v>
+      </c>
+      <c r="I3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!K$4:K$461)</f>
+        <v>101.86000000000001</v>
+      </c>
+      <c r="J3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!L$4:L$461)</f>
+        <v>103.35358333333333</v>
+      </c>
+      <c r="K3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!M$4:M$461)</f>
+        <v>100.79616666666668</v>
+      </c>
+      <c r="L3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!N$4:N$461)</f>
+        <v>105.84099999999999</v>
+      </c>
+      <c r="M3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!O$4:O$461)</f>
+        <v>103.16008333333333</v>
+      </c>
+      <c r="N3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!P$4:P$461)</f>
+        <v>101.36708333333333</v>
+      </c>
+      <c r="O3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!Q$4:Q$461)</f>
+        <v>102.063</v>
+      </c>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="83"/>
+      <c r="Z3" s="83"/>
+      <c r="AA3" s="83"/>
+      <c r="AB3" s="83"/>
+      <c r="AC3" s="83"/>
+      <c r="AD3" s="83"/>
+      <c r="AE3" s="83"/>
+      <c r="AF3" s="83"/>
+      <c r="AG3" s="83"/>
+      <c r="AH3" s="83"/>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A4" s="83">
+        <v>2017</v>
+      </c>
+      <c r="B4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!D$4:D$461)</f>
+        <v>104.22325000000001</v>
+      </c>
+      <c r="C4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!E$4:E$461)</f>
+        <v>100.62633333333332</v>
+      </c>
+      <c r="D4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!F$4:F$461)</f>
+        <v>107.18333333333332</v>
+      </c>
+      <c r="E4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!G$4:G$461)</f>
+        <v>103.45533333333333</v>
+      </c>
+      <c r="F4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!H$4:H$461)</f>
+        <v>104.18933333333332</v>
+      </c>
+      <c r="G4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!I$4:I$461)</f>
+        <v>103.22658333333332</v>
+      </c>
+      <c r="H4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!J$4:J$461)</f>
+        <v>105.42900000000002</v>
+      </c>
+      <c r="I4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!K$4:K$461)</f>
+        <v>105.66108333333331</v>
+      </c>
+      <c r="J4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!L$4:L$461)</f>
+        <v>104.62608333333333</v>
+      </c>
+      <c r="K4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!M$4:M$461)</f>
+        <v>103.28841666666666</v>
+      </c>
+      <c r="L4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!N$4:N$461)</f>
+        <v>109.44699999999999</v>
+      </c>
+      <c r="M4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!O$4:O$461)</f>
+        <v>106.31766666666668</v>
+      </c>
+      <c r="N4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!P$4:P$461)</f>
+        <v>102.57616666666667</v>
+      </c>
+      <c r="O4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!Q$4:Q$461)</f>
+        <v>102.80433333333333</v>
+      </c>
+      <c r="P4" s="83"/>
+      <c r="Q4" s="83"/>
+      <c r="R4" s="83"/>
+      <c r="S4" s="83"/>
+      <c r="T4" s="83"/>
+      <c r="U4" s="83"/>
+      <c r="V4" s="83"/>
+      <c r="W4" s="83"/>
+      <c r="X4" s="83"/>
+      <c r="Y4" s="83"/>
+      <c r="Z4" s="83"/>
+      <c r="AA4" s="83"/>
+      <c r="AB4" s="83"/>
+      <c r="AC4" s="83"/>
+      <c r="AD4" s="83"/>
+      <c r="AE4" s="83"/>
+      <c r="AF4" s="83"/>
+      <c r="AG4" s="83"/>
+      <c r="AH4" s="83"/>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A5" s="83">
+        <v>2018</v>
+      </c>
+      <c r="B5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!D$4:D$461)</f>
+        <v>106.42750000000001</v>
+      </c>
+      <c r="C5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!E$4:E$461)</f>
+        <v>102.15249999999999</v>
+      </c>
+      <c r="D5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!F$4:F$461)</f>
+        <v>111.80899999999998</v>
+      </c>
+      <c r="E5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!G$4:G$461)</f>
+        <v>103.06716666666667</v>
+      </c>
+      <c r="F5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!H$4:H$461)</f>
+        <v>106.02291666666669</v>
+      </c>
+      <c r="G5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!I$4:I$461)</f>
+        <v>104.29216666666666</v>
+      </c>
+      <c r="H5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!J$4:J$461)</f>
+        <v>107.94308333333335</v>
+      </c>
+      <c r="I5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!K$4:K$461)</f>
+        <v>110.24416666666667</v>
+      </c>
+      <c r="J5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!L$4:L$461)</f>
+        <v>106.54825000000001</v>
+      </c>
+      <c r="K5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!M$4:M$461)</f>
+        <v>106.36141666666667</v>
+      </c>
+      <c r="L5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!N$4:N$461)</f>
+        <v>112.71508333333334</v>
+      </c>
+      <c r="M5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!O$4:O$461)</f>
+        <v>109.10675000000002</v>
+      </c>
+      <c r="N5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!P$4:P$461)</f>
+        <v>102.5265</v>
+      </c>
+      <c r="O5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!Q$4:Q$461)</f>
+        <v>103.36333333333334</v>
+      </c>
+      <c r="P5" s="83"/>
+      <c r="Q5" s="83"/>
+      <c r="R5" s="83"/>
+      <c r="S5" s="83"/>
+      <c r="T5" s="83"/>
+      <c r="U5" s="83"/>
+      <c r="V5" s="83"/>
+      <c r="W5" s="83"/>
+      <c r="X5" s="83"/>
+      <c r="Y5" s="83"/>
+      <c r="Z5" s="83"/>
+      <c r="AA5" s="83"/>
+      <c r="AB5" s="83"/>
+      <c r="AC5" s="83"/>
+      <c r="AD5" s="83"/>
+      <c r="AE5" s="83"/>
+      <c r="AF5" s="83"/>
+      <c r="AG5" s="83"/>
+      <c r="AH5" s="83"/>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A6" s="83">
+        <v>2019</v>
+      </c>
+      <c r="B6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!D$4:D$461)</f>
+        <v>108.24916666666667</v>
+      </c>
+      <c r="C6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!E$4:E$461)</f>
+        <v>103.64933333333333</v>
+      </c>
+      <c r="D6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!F$4:F$461)</f>
+        <v>114.71591666666666</v>
+      </c>
+      <c r="E6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!G$4:G$461)</f>
+        <v>102.52391666666666</v>
+      </c>
+      <c r="F6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!H$4:H$461)</f>
+        <v>107.88216666666665</v>
+      </c>
+      <c r="G6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!I$4:I$461)</f>
+        <v>105.14791666666667</v>
+      </c>
+      <c r="H6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!J$4:J$461)</f>
+        <v>110.89258333333333</v>
+      </c>
+      <c r="I6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!K$4:K$461)</f>
+        <v>112.05733333333335</v>
+      </c>
+      <c r="J6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!L$4:L$461)</f>
+        <v>110.98208333333332</v>
+      </c>
+      <c r="K6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!M$4:M$461)</f>
+        <v>107.99141666666667</v>
+      </c>
+      <c r="L6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!N$4:N$461)</f>
+        <v>116.03508333333336</v>
+      </c>
+      <c r="M6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!O$4:O$461)</f>
+        <v>111.91091666666665</v>
+      </c>
+      <c r="N6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!P$4:P$461)</f>
+        <v>104.35108333333334</v>
+      </c>
+      <c r="O6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!Q$4:Q$461)</f>
+        <v>104.1439166666667</v>
+      </c>
+      <c r="P6" s="83"/>
+      <c r="Q6" s="83"/>
+      <c r="R6" s="83"/>
+      <c r="S6" s="83"/>
+      <c r="T6" s="83"/>
+      <c r="U6" s="83"/>
+      <c r="V6" s="83"/>
+      <c r="W6" s="83"/>
+      <c r="X6" s="83"/>
+      <c r="Y6" s="83"/>
+      <c r="Z6" s="83"/>
+      <c r="AA6" s="83"/>
+      <c r="AB6" s="83"/>
+      <c r="AC6" s="83"/>
+      <c r="AD6" s="83"/>
+      <c r="AE6" s="83"/>
+      <c r="AF6" s="83"/>
+      <c r="AG6" s="83"/>
+      <c r="AH6" s="83"/>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A7" s="83">
+        <v>2020</v>
+      </c>
+      <c r="B7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!D$4:D$461)</f>
+        <v>109.12025</v>
+      </c>
+      <c r="C7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!E$4:E$461)</f>
+        <v>103.80775000000001</v>
+      </c>
+      <c r="D7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!F$4:F$461)</f>
+        <v>117.58825</v>
+      </c>
+      <c r="E7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!G$4:G$461)</f>
+        <v>100.09300000000002</v>
+      </c>
+      <c r="F7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!H$4:H$461)</f>
+        <v>108.55033333333334</v>
+      </c>
+      <c r="G7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!I$4:I$461)</f>
+        <v>105.38983333333334</v>
+      </c>
+      <c r="H7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!J$4:J$461)</f>
+        <v>112.74474999999997</v>
+      </c>
+      <c r="I7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!K$4:K$461)</f>
+        <v>112.85741666666668</v>
+      </c>
+      <c r="J7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!L$4:L$461)</f>
+        <v>114.63116666666667</v>
+      </c>
+      <c r="K7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!M$4:M$461)</f>
+        <v>110.43516666666665</v>
+      </c>
+      <c r="L7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!N$4:N$461)</f>
+        <v>118.79841666666665</v>
+      </c>
+      <c r="M7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!O$4:O$461)</f>
+        <v>112.60033333333332</v>
+      </c>
+      <c r="N7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!P$4:P$461)</f>
+        <v>105.20324999999998</v>
+      </c>
+      <c r="O7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!Q$4:Q$461)</f>
+        <v>105.88483333333335</v>
+      </c>
+      <c r="P7" s="83"/>
+      <c r="Q7" s="83"/>
+      <c r="R7" s="83"/>
+      <c r="S7" s="83"/>
+      <c r="T7" s="83"/>
+      <c r="U7" s="83"/>
+      <c r="V7" s="83"/>
+      <c r="W7" s="83"/>
+      <c r="X7" s="83"/>
+      <c r="Y7" s="83"/>
+      <c r="Z7" s="83"/>
+      <c r="AA7" s="83"/>
+      <c r="AB7" s="83"/>
+      <c r="AC7" s="83"/>
+      <c r="AD7" s="83"/>
+      <c r="AE7" s="83"/>
+      <c r="AF7" s="83"/>
+      <c r="AG7" s="83"/>
+      <c r="AH7" s="83"/>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A8" s="83">
+        <v>2021</v>
+      </c>
+      <c r="B8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!D$4:D$461)</f>
+        <v>113.12966666666667</v>
+      </c>
+      <c r="C8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!E$4:E$461)</f>
+        <v>105.66408333333332</v>
+      </c>
+      <c r="D8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!F$4:F$461)</f>
+        <v>121.09750000000001</v>
+      </c>
+      <c r="E8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!G$4:G$461)</f>
+        <v>103.44716666666669</v>
+      </c>
+      <c r="F8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!H$4:H$461)</f>
+        <v>111.82508333333332</v>
+      </c>
+      <c r="G8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!I$4:I$461)</f>
+        <v>111.33216666666665</v>
+      </c>
+      <c r="H8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!J$4:J$461)</f>
+        <v>114.81333333333333</v>
+      </c>
+      <c r="I8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!K$4:K$461)</f>
+        <v>123.69483333333334</v>
+      </c>
+      <c r="J8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!L$4:L$461)</f>
+        <v>116.41508333333331</v>
+      </c>
+      <c r="K8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!M$4:M$461)</f>
+        <v>113.33258333333333</v>
+      </c>
+      <c r="L8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!N$4:N$461)</f>
+        <v>122.83691666666664</v>
+      </c>
+      <c r="M8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!O$4:O$461)</f>
+        <v>117.77583333333332</v>
+      </c>
+      <c r="N8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!P$4:P$461)</f>
+        <v>106.59633333333335</v>
+      </c>
+      <c r="O8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!Q$4:Q$461)</f>
+        <v>107.80974999999999</v>
+      </c>
+      <c r="P8" s="83"/>
+      <c r="Q8" s="83"/>
+      <c r="R8" s="83"/>
+      <c r="S8" s="83"/>
+      <c r="T8" s="83"/>
+      <c r="U8" s="83"/>
+      <c r="V8" s="83"/>
+      <c r="W8" s="83"/>
+      <c r="X8" s="83"/>
+      <c r="Y8" s="83"/>
+      <c r="Z8" s="83"/>
+      <c r="AA8" s="83"/>
+      <c r="AB8" s="83"/>
+      <c r="AC8" s="83"/>
+      <c r="AD8" s="83"/>
+      <c r="AE8" s="83"/>
+      <c r="AF8" s="83"/>
+      <c r="AG8" s="83"/>
+      <c r="AH8" s="83"/>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A9" s="83">
+        <v>2022</v>
+      </c>
+      <c r="B9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!D$4:D$461)</f>
+        <v>123.04399999999998</v>
+      </c>
+      <c r="C9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!E$4:E$461)</f>
+        <v>120.66683333333333</v>
+      </c>
+      <c r="D9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!F$4:F$461)</f>
+        <v>127.25466666666669</v>
+      </c>
+      <c r="E9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!G$4:G$461)</f>
+        <v>111.01149999999997</v>
+      </c>
+      <c r="F9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!H$4:H$461)</f>
+        <v>123.4155833333333</v>
+      </c>
+      <c r="G9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!I$4:I$461)</f>
+        <v>122.45841666666666</v>
+      </c>
+      <c r="H9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!J$4:J$461)</f>
+        <v>119.34825000000001</v>
+      </c>
+      <c r="I9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!K$4:K$461)</f>
+        <v>135.10224999999997</v>
+      </c>
+      <c r="J9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!L$4:L$461)</f>
+        <v>119.66116666666669</v>
+      </c>
+      <c r="K9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!M$4:M$461)</f>
+        <v>119.14958333333334</v>
+      </c>
+      <c r="L9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!N$4:N$461)</f>
+        <v>127.50683333333335</v>
+      </c>
+      <c r="M9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!O$4:O$461)</f>
+        <v>129.26033333333331</v>
+      </c>
+      <c r="N9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!P$4:P$461)</f>
+        <v>111.73</v>
+      </c>
+      <c r="O9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!Q$4:Q$461)</f>
+        <v>112.18416666666667</v>
+      </c>
+      <c r="P9" s="83"/>
+      <c r="Q9" s="83"/>
+      <c r="R9" s="83"/>
+      <c r="S9" s="83"/>
+      <c r="T9" s="83"/>
+      <c r="U9" s="83"/>
+      <c r="V9" s="83"/>
+      <c r="W9" s="83"/>
+      <c r="X9" s="83"/>
+      <c r="Y9" s="83"/>
+      <c r="Z9" s="83"/>
+      <c r="AA9" s="83"/>
+      <c r="AB9" s="83"/>
+      <c r="AC9" s="83"/>
+      <c r="AD9" s="83"/>
+      <c r="AE9" s="83"/>
+      <c r="AF9" s="83"/>
+      <c r="AG9" s="83"/>
+      <c r="AH9" s="83"/>
+    </row>
+    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A10" s="83">
+        <v>2023</v>
+      </c>
+      <c r="B10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!D$4:D$461)</f>
+        <v>129.87941666666669</v>
+      </c>
+      <c r="C10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!E$4:E$461)</f>
+        <v>134.33116666666666</v>
+      </c>
+      <c r="D10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!F$4:F$461)</f>
+        <v>140.86641666666665</v>
+      </c>
+      <c r="E10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!G$4:G$461)</f>
+        <v>117.85725000000001</v>
+      </c>
+      <c r="F10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!H$4:H$461)</f>
+        <v>128.80408333333335</v>
+      </c>
+      <c r="G10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!I$4:I$461)</f>
+        <v>126.90808333333332</v>
+      </c>
+      <c r="H10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!J$4:J$461)</f>
+        <v>128.66024999999999</v>
+      </c>
+      <c r="I10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!K$4:K$461)</f>
+        <v>134.63233333333332</v>
+      </c>
+      <c r="J10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!L$4:L$461)</f>
+        <v>129.17991666666668</v>
+      </c>
+      <c r="K10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!M$4:M$461)</f>
+        <v>126.51691666666666</v>
+      </c>
+      <c r="L10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!N$4:N$461)</f>
+        <v>132.48083333333329</v>
+      </c>
+      <c r="M10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!O$4:O$461)</f>
+        <v>139.75333333333336</v>
+      </c>
+      <c r="N10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!P$4:P$461)</f>
+        <v>117.30658333333334</v>
+      </c>
+      <c r="O10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!Q$4:Q$461)</f>
+        <v>119.24366666666664</v>
+      </c>
+      <c r="P10" s="83"/>
+      <c r="Q10" s="83"/>
+      <c r="R10" s="83"/>
+      <c r="S10" s="83"/>
+      <c r="T10" s="83"/>
+      <c r="U10" s="83"/>
+      <c r="V10" s="83"/>
+      <c r="W10" s="83"/>
+      <c r="X10" s="83"/>
+      <c r="Y10" s="83"/>
+      <c r="Z10" s="83"/>
+      <c r="AA10" s="83"/>
+      <c r="AB10" s="83"/>
+      <c r="AC10" s="83"/>
+      <c r="AD10" s="83"/>
+      <c r="AE10" s="83"/>
+      <c r="AF10" s="83"/>
+      <c r="AG10" s="83"/>
+      <c r="AH10" s="83"/>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A11" s="83"/>
+      <c r="B11" s="83"/>
+      <c r="C11" s="83"/>
+      <c r="D11" s="83"/>
+      <c r="E11" s="83"/>
+      <c r="F11" s="83"/>
+      <c r="G11" s="83"/>
+      <c r="H11" s="83"/>
+      <c r="I11" s="83"/>
+      <c r="J11" s="83"/>
+      <c r="K11" s="83"/>
+      <c r="L11" s="83"/>
+      <c r="M11" s="83"/>
+      <c r="N11" s="83"/>
+      <c r="O11" s="83"/>
+      <c r="P11" s="83"/>
+      <c r="Q11" s="83"/>
+      <c r="R11" s="83"/>
+      <c r="S11" s="83"/>
+      <c r="T11" s="83"/>
+      <c r="U11" s="83"/>
+      <c r="V11" s="83"/>
+      <c r="W11" s="83"/>
+      <c r="X11" s="83"/>
+      <c r="Y11" s="83"/>
+      <c r="Z11" s="83"/>
+      <c r="AA11" s="83"/>
+      <c r="AB11" s="83"/>
+      <c r="AC11" s="83"/>
+      <c r="AD11" s="83"/>
+      <c r="AE11" s="83"/>
+      <c r="AF11" s="83"/>
+      <c r="AG11" s="83"/>
+      <c r="AH11" s="83"/>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A12" s="83"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="83"/>
+      <c r="F12" s="83"/>
+      <c r="G12" s="83"/>
+      <c r="H12" s="83"/>
+      <c r="I12" s="83"/>
+      <c r="J12" s="83"/>
+      <c r="K12" s="83"/>
+      <c r="L12" s="83"/>
+      <c r="M12" s="83"/>
+      <c r="N12" s="83"/>
+      <c r="O12" s="83"/>
+      <c r="P12" s="83"/>
+      <c r="Q12" s="83"/>
+      <c r="R12" s="83"/>
+      <c r="S12" s="83"/>
+      <c r="T12" s="83"/>
+      <c r="U12" s="83"/>
+      <c r="V12" s="83"/>
+      <c r="W12" s="83"/>
+      <c r="X12" s="83"/>
+      <c r="Y12" s="83"/>
+      <c r="Z12" s="83"/>
+      <c r="AA12" s="83"/>
+      <c r="AB12" s="83"/>
+      <c r="AC12" s="83"/>
+      <c r="AD12" s="83"/>
+      <c r="AE12" s="83"/>
+      <c r="AF12" s="83"/>
+      <c r="AG12" s="83"/>
+      <c r="AH12" s="83"/>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A13" s="83"/>
+      <c r="B13" s="83"/>
+      <c r="C13" s="83"/>
+      <c r="D13" s="83"/>
+      <c r="E13" s="83"/>
+      <c r="F13" s="83"/>
+      <c r="G13" s="83"/>
+      <c r="H13" s="83"/>
+      <c r="I13" s="83"/>
+      <c r="J13" s="83"/>
+      <c r="K13" s="83"/>
+      <c r="L13" s="83"/>
+      <c r="M13" s="83"/>
+      <c r="N13" s="83"/>
+      <c r="O13" s="83"/>
+      <c r="P13" s="83"/>
+      <c r="Q13" s="83"/>
+      <c r="R13" s="83"/>
+      <c r="S13" s="83"/>
+      <c r="T13" s="83"/>
+      <c r="U13" s="83"/>
+      <c r="V13" s="83"/>
+      <c r="W13" s="83"/>
+      <c r="X13" s="83"/>
+      <c r="Y13" s="83"/>
+      <c r="Z13" s="83"/>
+      <c r="AA13" s="83"/>
+      <c r="AB13" s="83"/>
+      <c r="AC13" s="83"/>
+      <c r="AD13" s="83"/>
+      <c r="AE13" s="83"/>
+      <c r="AF13" s="83"/>
+      <c r="AG13" s="83"/>
+      <c r="AH13" s="83"/>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A14" s="83"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
+      <c r="D14" s="83"/>
+      <c r="E14" s="83"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="83"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="83"/>
+      <c r="J14" s="83"/>
+      <c r="K14" s="83"/>
+      <c r="L14" s="83"/>
+      <c r="M14" s="83"/>
+      <c r="N14" s="83"/>
+      <c r="O14" s="83"/>
+      <c r="P14" s="83"/>
+      <c r="Q14" s="83"/>
+      <c r="R14" s="83"/>
+      <c r="S14" s="83"/>
+      <c r="T14" s="83"/>
+      <c r="U14" s="83"/>
+      <c r="V14" s="83"/>
+      <c r="W14" s="83"/>
+      <c r="X14" s="83"/>
+      <c r="Y14" s="83"/>
+      <c r="Z14" s="83"/>
+      <c r="AA14" s="83"/>
+      <c r="AB14" s="83"/>
+      <c r="AC14" s="83"/>
+      <c r="AD14" s="83"/>
+      <c r="AE14" s="83"/>
+      <c r="AF14" s="83"/>
+      <c r="AG14" s="83"/>
+      <c r="AH14" s="83"/>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A15" s="83"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="83"/>
+      <c r="D15" s="83"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="83"/>
+      <c r="H15" s="83"/>
+      <c r="I15" s="83"/>
+      <c r="J15" s="83"/>
+      <c r="K15" s="83"/>
+      <c r="L15" s="83"/>
+      <c r="M15" s="83"/>
+      <c r="N15" s="83"/>
+      <c r="O15" s="83"/>
+      <c r="P15" s="83"/>
+      <c r="Q15" s="83"/>
+      <c r="R15" s="83"/>
+      <c r="S15" s="83"/>
+      <c r="T15" s="83"/>
+      <c r="U15" s="83"/>
+      <c r="V15" s="83"/>
+      <c r="W15" s="83"/>
+      <c r="X15" s="83"/>
+      <c r="Y15" s="83"/>
+      <c r="Z15" s="83"/>
+      <c r="AA15" s="83"/>
+      <c r="AB15" s="83"/>
+      <c r="AC15" s="83"/>
+      <c r="AD15" s="83"/>
+      <c r="AE15" s="83"/>
+      <c r="AF15" s="83"/>
+      <c r="AG15" s="83"/>
+      <c r="AH15" s="83"/>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A16" s="83"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="83"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="83"/>
+      <c r="G16" s="83"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="83"/>
+      <c r="J16" s="83"/>
+      <c r="K16" s="83"/>
+      <c r="L16" s="83"/>
+      <c r="M16" s="83"/>
+      <c r="N16" s="83"/>
+      <c r="O16" s="83"/>
+      <c r="P16" s="83"/>
+      <c r="Q16" s="83"/>
+      <c r="R16" s="83"/>
+      <c r="S16" s="83"/>
+      <c r="T16" s="83"/>
+      <c r="U16" s="83"/>
+      <c r="V16" s="83"/>
+      <c r="W16" s="83"/>
+      <c r="X16" s="83"/>
+      <c r="Y16" s="83"/>
+      <c r="Z16" s="83"/>
+      <c r="AA16" s="83"/>
+      <c r="AB16" s="83"/>
+      <c r="AC16" s="83"/>
+      <c r="AD16" s="83"/>
+      <c r="AE16" s="83"/>
+      <c r="AF16" s="83"/>
+      <c r="AG16" s="83"/>
+      <c r="AH16" s="83"/>
+    </row>
+    <row r="17" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A17" s="83"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="E17" s="83"/>
+      <c r="F17" s="83"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="83"/>
+      <c r="I17" s="83"/>
+      <c r="J17" s="83"/>
+      <c r="K17" s="83"/>
+      <c r="L17" s="83"/>
+      <c r="M17" s="83"/>
+      <c r="N17" s="83"/>
+      <c r="O17" s="83"/>
+      <c r="P17" s="83"/>
+      <c r="Q17" s="83"/>
+      <c r="R17" s="83"/>
+      <c r="S17" s="83"/>
+      <c r="T17" s="83"/>
+      <c r="U17" s="83"/>
+      <c r="V17" s="83"/>
+      <c r="W17" s="83"/>
+      <c r="X17" s="83"/>
+      <c r="Y17" s="83"/>
+      <c r="Z17" s="83"/>
+      <c r="AA17" s="83"/>
+      <c r="AB17" s="83"/>
+      <c r="AC17" s="83"/>
+      <c r="AD17" s="83"/>
+      <c r="AE17" s="83"/>
+      <c r="AF17" s="83"/>
+      <c r="AG17" s="83"/>
+      <c r="AH17" s="83"/>
+    </row>
+    <row r="18" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A18" s="83"/>
+      <c r="B18" s="83"/>
+      <c r="C18" s="83"/>
+      <c r="D18" s="83"/>
+      <c r="E18" s="83"/>
+      <c r="F18" s="83"/>
+      <c r="G18" s="83"/>
+      <c r="H18" s="83"/>
+      <c r="I18" s="83"/>
+      <c r="J18" s="83"/>
+      <c r="K18" s="83"/>
+      <c r="L18" s="83"/>
+      <c r="M18" s="83"/>
+      <c r="N18" s="83"/>
+      <c r="O18" s="83"/>
+      <c r="P18" s="83"/>
+      <c r="Q18" s="83"/>
+      <c r="R18" s="83"/>
+      <c r="S18" s="83"/>
+      <c r="T18" s="83"/>
+      <c r="U18" s="83"/>
+      <c r="V18" s="83"/>
+      <c r="W18" s="83"/>
+      <c r="X18" s="83"/>
+      <c r="Y18" s="83"/>
+      <c r="Z18" s="83"/>
+      <c r="AA18" s="83"/>
+      <c r="AB18" s="83"/>
+      <c r="AC18" s="83"/>
+      <c r="AD18" s="83"/>
+      <c r="AE18" s="83"/>
+      <c r="AF18" s="83"/>
+      <c r="AG18" s="83"/>
+      <c r="AH18" s="83"/>
+    </row>
+    <row r="19" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A19" s="83"/>
+      <c r="B19" s="83"/>
+      <c r="C19" s="83"/>
+      <c r="D19" s="83"/>
+      <c r="E19" s="83"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="83"/>
+      <c r="H19" s="83"/>
+      <c r="I19" s="83"/>
+      <c r="J19" s="83"/>
+      <c r="K19" s="83"/>
+      <c r="L19" s="83"/>
+      <c r="M19" s="83"/>
+      <c r="N19" s="83"/>
+      <c r="O19" s="83"/>
+      <c r="P19" s="83"/>
+      <c r="Q19" s="83"/>
+      <c r="R19" s="83"/>
+      <c r="S19" s="83"/>
+      <c r="T19" s="83"/>
+      <c r="U19" s="83"/>
+      <c r="V19" s="83"/>
+      <c r="W19" s="83"/>
+      <c r="X19" s="83"/>
+      <c r="Y19" s="83"/>
+      <c r="Z19" s="83"/>
+      <c r="AA19" s="83"/>
+      <c r="AB19" s="83"/>
+      <c r="AC19" s="83"/>
+      <c r="AD19" s="83"/>
+      <c r="AE19" s="83"/>
+      <c r="AF19" s="83"/>
+      <c r="AG19" s="83"/>
+      <c r="AH19" s="83"/>
+    </row>
+    <row r="20" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A20" s="83"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="83"/>
+      <c r="D20" s="83"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="83"/>
+      <c r="G20" s="83"/>
+      <c r="H20" s="83"/>
+      <c r="I20" s="83"/>
+      <c r="J20" s="83"/>
+      <c r="K20" s="83"/>
+      <c r="L20" s="83"/>
+      <c r="M20" s="83"/>
+      <c r="N20" s="83"/>
+      <c r="O20" s="83"/>
+      <c r="P20" s="83"/>
+      <c r="Q20" s="83"/>
+      <c r="R20" s="83"/>
+      <c r="S20" s="83"/>
+      <c r="T20" s="83"/>
+      <c r="U20" s="83"/>
+      <c r="V20" s="83"/>
+      <c r="W20" s="83"/>
+      <c r="X20" s="83"/>
+      <c r="Y20" s="83"/>
+      <c r="Z20" s="83"/>
+      <c r="AA20" s="83"/>
+      <c r="AB20" s="83"/>
+      <c r="AC20" s="83"/>
+      <c r="AD20" s="83"/>
+      <c r="AE20" s="83"/>
+      <c r="AF20" s="83"/>
+      <c r="AG20" s="83"/>
+      <c r="AH20" s="83"/>
+    </row>
+    <row r="21" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A21" s="83"/>
+      <c r="B21" s="83"/>
+      <c r="C21" s="83"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="83"/>
+      <c r="J21" s="83"/>
+      <c r="K21" s="83"/>
+      <c r="L21" s="83"/>
+      <c r="M21" s="83"/>
+      <c r="N21" s="83"/>
+      <c r="O21" s="83"/>
+      <c r="P21" s="83"/>
+      <c r="Q21" s="83"/>
+      <c r="R21" s="83"/>
+      <c r="S21" s="83"/>
+      <c r="T21" s="83"/>
+      <c r="U21" s="83"/>
+      <c r="V21" s="83"/>
+      <c r="W21" s="83"/>
+      <c r="X21" s="83"/>
+      <c r="Y21" s="83"/>
+      <c r="Z21" s="83"/>
+      <c r="AA21" s="83"/>
+      <c r="AB21" s="83"/>
+      <c r="AC21" s="83"/>
+      <c r="AD21" s="83"/>
+      <c r="AE21" s="83"/>
+      <c r="AF21" s="83"/>
+      <c r="AG21" s="83"/>
+      <c r="AH21" s="83"/>
+    </row>
+    <row r="22" spans="1:574" ht="17" x14ac:dyDescent="0.25">
+      <c r="A22" s="83"/>
+      <c r="B22" s="83"/>
+      <c r="C22" s="83"/>
+      <c r="D22" s="83"/>
+      <c r="E22" s="83"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="83"/>
+      <c r="H22" s="83"/>
+      <c r="I22" s="83"/>
+      <c r="J22" s="83"/>
+      <c r="K22" s="83"/>
+      <c r="L22" s="83"/>
+      <c r="M22" s="83"/>
+      <c r="N22" s="83"/>
+      <c r="O22" s="83"/>
+      <c r="P22" s="83"/>
+      <c r="Q22" s="83"/>
+      <c r="R22" s="83"/>
+      <c r="S22" s="83"/>
+      <c r="T22" s="83"/>
+      <c r="U22" s="83"/>
+      <c r="V22" s="83"/>
+      <c r="W22" s="83"/>
+      <c r="X22" s="83"/>
+      <c r="Y22" s="83"/>
+      <c r="Z22" s="83"/>
+      <c r="AA22" s="83"/>
+      <c r="AB22" s="83"/>
+      <c r="AC22" s="83"/>
+      <c r="AD22" s="83"/>
+      <c r="AE22" s="83"/>
+      <c r="AF22" s="83"/>
+      <c r="AG22" s="83"/>
+      <c r="AH22" s="83"/>
+      <c r="VB22" s="82">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!D$4:D$461)</f>
+        <v>100.16549999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A23" s="83"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="83"/>
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="83"/>
+      <c r="H23" s="83"/>
+      <c r="I23" s="83"/>
+      <c r="J23" s="83"/>
+      <c r="K23" s="83"/>
+      <c r="L23" s="83"/>
+      <c r="M23" s="83"/>
+      <c r="N23" s="83"/>
+      <c r="O23" s="83"/>
+      <c r="P23" s="83"/>
+      <c r="Q23" s="83"/>
+      <c r="R23" s="83"/>
+      <c r="S23" s="83"/>
+      <c r="T23" s="83"/>
+      <c r="U23" s="83"/>
+      <c r="V23" s="83"/>
+      <c r="W23" s="83"/>
+      <c r="X23" s="83"/>
+      <c r="Y23" s="83"/>
+      <c r="Z23" s="83"/>
+      <c r="AA23" s="83"/>
+      <c r="AB23" s="83"/>
+      <c r="AC23" s="83"/>
+      <c r="AD23" s="83"/>
+      <c r="AE23" s="83"/>
+      <c r="AF23" s="83"/>
+      <c r="AG23" s="83"/>
+      <c r="AH23" s="83"/>
+    </row>
+    <row r="24" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A24" s="83"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="83"/>
+      <c r="E24" s="83"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="83"/>
+      <c r="H24" s="83"/>
+      <c r="I24" s="83"/>
+      <c r="J24" s="83"/>
+      <c r="K24" s="83"/>
+      <c r="L24" s="83"/>
+      <c r="M24" s="83"/>
+      <c r="N24" s="83"/>
+      <c r="O24" s="83"/>
+      <c r="P24" s="83"/>
+      <c r="Q24" s="83"/>
+      <c r="R24" s="83"/>
+      <c r="S24" s="83"/>
+      <c r="T24" s="83"/>
+      <c r="U24" s="83"/>
+      <c r="V24" s="83"/>
+      <c r="W24" s="83"/>
+      <c r="X24" s="83"/>
+      <c r="Y24" s="83"/>
+      <c r="Z24" s="83"/>
+      <c r="AA24" s="83"/>
+      <c r="AB24" s="83"/>
+      <c r="AC24" s="83"/>
+      <c r="AD24" s="83"/>
+      <c r="AE24" s="83"/>
+      <c r="AF24" s="83"/>
+      <c r="AG24" s="83"/>
+      <c r="AH24" s="83"/>
+    </row>
+    <row r="25" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="A25" s="83"/>
+      <c r="B25" s="83"/>
+      <c r="C25" s="83"/>
+      <c r="D25" s="83"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="83"/>
+      <c r="H25" s="83"/>
+      <c r="I25" s="83"/>
+      <c r="J25" s="83"/>
+      <c r="K25" s="83"/>
+      <c r="L25" s="83"/>
+      <c r="M25" s="83"/>
+      <c r="N25" s="83"/>
+      <c r="O25" s="83"/>
+      <c r="P25" s="83"/>
+      <c r="Q25" s="83"/>
+      <c r="R25" s="83"/>
+      <c r="S25" s="83"/>
+      <c r="T25" s="83"/>
+      <c r="U25" s="83"/>
+      <c r="V25" s="83"/>
+      <c r="W25" s="83"/>
+      <c r="X25" s="83"/>
+      <c r="Y25" s="83"/>
+      <c r="Z25" s="83"/>
+      <c r="AA25" s="83"/>
+      <c r="AB25" s="83"/>
+      <c r="AC25" s="83"/>
+      <c r="AD25" s="83"/>
+      <c r="AE25" s="83"/>
+      <c r="AF25" s="83"/>
+      <c r="AG25" s="83"/>
+      <c r="AH25" s="83"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21DB90F7-3BE6-A64F-8333-62671F03D732}">
+  <dimension ref="A1:AE85"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A1" s="83" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="83" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="83" t="s">
+        <v>119</v>
+      </c>
+      <c r="D1" s="83" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="83" t="s">
+        <v>121</v>
+      </c>
+      <c r="F1" s="83" t="s">
+        <v>122</v>
+      </c>
+      <c r="G1" s="83" t="s">
+        <v>123</v>
+      </c>
+      <c r="H1" s="83" t="s">
+        <v>124</v>
+      </c>
+      <c r="I1" s="83" t="s">
+        <v>125</v>
+      </c>
+      <c r="J1" s="83" t="s">
+        <v>126</v>
+      </c>
+      <c r="K1" s="83" t="s">
+        <v>127</v>
+      </c>
+      <c r="L1" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="M1" s="83" t="s">
+        <v>129</v>
+      </c>
+      <c r="N1" s="83" t="s">
+        <v>130</v>
+      </c>
+      <c r="O1" s="83" t="s">
+        <v>131</v>
+      </c>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="83"/>
+      <c r="T1" s="83"/>
+      <c r="U1" s="83"/>
+      <c r="V1" s="83"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="83"/>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A2" s="83">
+        <v>2015</v>
+      </c>
+      <c r="B2" s="83">
+        <f>('Financial Year Averages'!B3-'Financial Year Averages'!B2)/'Financial Year Averages'!B2*100</f>
+        <v>1.3684019614204999</v>
+      </c>
+      <c r="C2" s="83">
+        <f>('Financial Year Averages'!C3-'Financial Year Averages'!C2)/'Financial Year Averages'!C2*100</f>
+        <v>-1.6837789918461368</v>
+      </c>
+      <c r="D2" s="83">
+        <f>('Financial Year Averages'!D3-'Financial Year Averages'!D2)/'Financial Year Averages'!D2*100</f>
+        <v>2.0368291282354609</v>
+      </c>
+      <c r="E2" s="83">
+        <f>('Financial Year Averages'!E3-'Financial Year Averages'!E2)/'Financial Year Averages'!E2*100</f>
+        <v>7.4788964509780509E-2</v>
+      </c>
+      <c r="F2" s="83">
+        <f>('Financial Year Averages'!F3-'Financial Year Averages'!F2)/'Financial Year Averages'!F2*100</f>
+        <v>1.7923998657901126</v>
+      </c>
+      <c r="G2" s="83">
+        <f>('Financial Year Averages'!G3-'Financial Year Averages'!G2)/'Financial Year Averages'!G2*100</f>
+        <v>5.047047477225778E-2</v>
+      </c>
+      <c r="H2" s="83">
+        <f>('Financial Year Averages'!H3-'Financial Year Averages'!H2)/'Financial Year Averages'!H2*100</f>
+        <v>2.1799275540753293</v>
+      </c>
+      <c r="I2" s="83">
+        <f>('Financial Year Averages'!I3-'Financial Year Averages'!I2)/'Financial Year Averages'!I2*100</f>
+        <v>1.9911436121613231</v>
+      </c>
+      <c r="J2" s="83">
+        <f>('Financial Year Averages'!J3-'Financial Year Averages'!J2)/'Financial Year Averages'!J2*100</f>
+        <v>2.8637802994740142</v>
+      </c>
+      <c r="K2" s="83">
+        <f>('Financial Year Averages'!K3-'Financial Year Averages'!K2)/'Financial Year Averages'!K2*100</f>
+        <v>0.81212858702627666</v>
+      </c>
+      <c r="L2" s="83">
+        <f>('Financial Year Averages'!L3-'Financial Year Averages'!L2)/'Financial Year Averages'!L2*100</f>
+        <v>4.6081062939044157</v>
+      </c>
+      <c r="M2" s="83">
+        <f>('Financial Year Averages'!M3-'Financial Year Averages'!M2)/'Financial Year Averages'!M2*100</f>
+        <v>2.686271761049241</v>
+      </c>
+      <c r="N2" s="83">
+        <f>('Financial Year Averages'!N3-'Financial Year Averages'!N2)/'Financial Year Averages'!N2*100</f>
+        <v>1.0810240353133882</v>
+      </c>
+      <c r="O2" s="83">
+        <f>('Financial Year Averages'!O3-'Financial Year Averages'!O2)/'Financial Year Averages'!O2*100</f>
+        <v>1.3310520341400587</v>
+      </c>
+      <c r="P2" s="83"/>
+      <c r="Q2" s="83"/>
+      <c r="R2" s="83"/>
+      <c r="S2" s="83"/>
+      <c r="T2" s="83"/>
+      <c r="U2" s="83"/>
+      <c r="V2" s="83"/>
+      <c r="W2" s="83"/>
+      <c r="X2" s="83"/>
+      <c r="Y2" s="83"/>
+      <c r="Z2" s="83"/>
+      <c r="AA2" s="83"/>
+      <c r="AB2" s="83"/>
+      <c r="AC2" s="83"/>
+      <c r="AD2" s="83"/>
+      <c r="AE2" s="83"/>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A3" s="83">
+        <v>2016</v>
+      </c>
+      <c r="B3" s="83">
+        <f>('Financial Year Averages'!B4-'Financial Year Averages'!B3)/'Financial Year Averages'!B3*100</f>
+        <v>2.6464297614807495</v>
+      </c>
+      <c r="C3" s="83">
+        <f>('Financial Year Averages'!C4-'Financial Year Averages'!C3)/'Financial Year Averages'!C3*100</f>
+        <v>3.0091056283600102</v>
+      </c>
+      <c r="D3" s="83">
+        <f>('Financial Year Averages'!D4-'Financial Year Averages'!D3)/'Financial Year Averages'!D3*100</f>
+        <v>4.7521238326148643</v>
+      </c>
+      <c r="E3" s="83">
+        <f>('Financial Year Averages'!E4-'Financial Year Averages'!E3)/'Financial Year Averages'!E3*100</f>
+        <v>3.2018009090999602</v>
+      </c>
+      <c r="F3" s="83">
+        <f>('Financial Year Averages'!F4-'Financial Year Averages'!F3)/'Financial Year Averages'!F3*100</f>
+        <v>2.0075616032426167</v>
+      </c>
+      <c r="G3" s="83">
+        <f>('Financial Year Averages'!G4-'Financial Year Averages'!G3)/'Financial Year Averages'!G3*100</f>
+        <v>3.1141888674677891</v>
+      </c>
+      <c r="H3" s="83">
+        <f>('Financial Year Averages'!H4-'Financial Year Averages'!H3)/'Financial Year Averages'!H3*100</f>
+        <v>2.6544220623579218</v>
+      </c>
+      <c r="I3" s="83">
+        <f>('Financial Year Averages'!I4-'Financial Year Averages'!I3)/'Financial Year Averages'!I3*100</f>
+        <v>3.7316741933372226</v>
+      </c>
+      <c r="J3" s="83">
+        <f>('Financial Year Averages'!J4-'Financial Year Averages'!J3)/'Financial Year Averages'!J3*100</f>
+        <v>1.231210335393945</v>
+      </c>
+      <c r="K3" s="83">
+        <f>('Financial Year Averages'!K4-'Financial Year Averages'!K3)/'Financial Year Averages'!K3*100</f>
+        <v>2.4725642674903154</v>
+      </c>
+      <c r="L3" s="83">
+        <f>('Financial Year Averages'!L4-'Financial Year Averages'!L3)/'Financial Year Averages'!L3*100</f>
+        <v>3.4069972883854036</v>
+      </c>
+      <c r="M3" s="83">
+        <f>('Financial Year Averages'!M4-'Financial Year Averages'!M3)/'Financial Year Averages'!M3*100</f>
+        <v>3.0608576799327412</v>
+      </c>
+      <c r="N3" s="83">
+        <f>('Financial Year Averages'!N4-'Financial Year Averages'!N3)/'Financial Year Averages'!N3*100</f>
+        <v>1.1927770767137649</v>
+      </c>
+      <c r="O3" s="83">
+        <f>('Financial Year Averages'!O4-'Financial Year Averages'!O3)/'Financial Year Averages'!O3*100</f>
+        <v>0.72634875844657687</v>
+      </c>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="83"/>
+      <c r="Z3" s="83"/>
+      <c r="AA3" s="83"/>
+      <c r="AB3" s="83"/>
+      <c r="AC3" s="83"/>
+      <c r="AD3" s="83"/>
+      <c r="AE3" s="83"/>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A4" s="83">
+        <v>2017</v>
+      </c>
+      <c r="B4" s="83">
+        <f>('Financial Year Averages'!B5-'Financial Year Averages'!B4)/'Financial Year Averages'!B4*100</f>
+        <v>2.1149311693887896</v>
+      </c>
+      <c r="C4" s="83">
+        <f>('Financial Year Averages'!C5-'Financial Year Averages'!C4)/'Financial Year Averages'!C4*100</f>
+        <v>1.5166672739740115</v>
+      </c>
+      <c r="D4" s="83">
+        <f>('Financial Year Averages'!D5-'Financial Year Averages'!D4)/'Financial Year Averages'!D4*100</f>
+        <v>4.3156585290001503</v>
+      </c>
+      <c r="E4" s="83">
+        <f>('Financial Year Averages'!E5-'Financial Year Averages'!E4)/'Financial Year Averages'!E4*100</f>
+        <v>-0.37520218065122785</v>
+      </c>
+      <c r="F4" s="83">
+        <f>('Financial Year Averages'!F5-'Financial Year Averages'!F4)/'Financial Year Averages'!F4*100</f>
+        <v>1.7598570551048403</v>
+      </c>
+      <c r="G4" s="83">
+        <f>('Financial Year Averages'!G5-'Financial Year Averages'!G4)/'Financial Year Averages'!G4*100</f>
+        <v>1.0322760852138406</v>
+      </c>
+      <c r="H4" s="83">
+        <f>('Financial Year Averages'!H5-'Financial Year Averages'!H4)/'Financial Year Averages'!H4*100</f>
+        <v>2.3846221943993888</v>
+      </c>
+      <c r="I4" s="83">
+        <f>('Financial Year Averages'!I5-'Financial Year Averages'!I4)/'Financial Year Averages'!I4*100</f>
+        <v>4.3375320304779796</v>
+      </c>
+      <c r="J4" s="83">
+        <f>('Financial Year Averages'!J5-'Financial Year Averages'!J4)/'Financial Year Averages'!J4*100</f>
+        <v>1.8371773131779761</v>
+      </c>
+      <c r="K4" s="83">
+        <f>('Financial Year Averages'!K5-'Financial Year Averages'!K4)/'Financial Year Averages'!K4*100</f>
+        <v>2.9751642044404858</v>
+      </c>
+      <c r="L4" s="83">
+        <f>('Financial Year Averages'!L5-'Financial Year Averages'!L4)/'Financial Year Averages'!L4*100</f>
+        <v>2.985996266077052</v>
+      </c>
+      <c r="M4" s="83">
+        <f>('Financial Year Averages'!M5-'Financial Year Averages'!M4)/'Financial Year Averages'!M4*100</f>
+        <v>2.6233488946647348</v>
+      </c>
+      <c r="N4" s="83">
+        <f>('Financial Year Averages'!N5-'Financial Year Averages'!N4)/'Financial Year Averages'!N4*100</f>
+        <v>-4.8419304679287394E-2</v>
+      </c>
+      <c r="O4" s="83">
+        <f>('Financial Year Averages'!O5-'Financial Year Averages'!O4)/'Financial Year Averages'!O4*100</f>
+        <v>0.54375139828737284</v>
+      </c>
+      <c r="P4" s="83"/>
+      <c r="Q4" s="83"/>
+      <c r="R4" s="83"/>
+      <c r="S4" s="83"/>
+      <c r="T4" s="83"/>
+      <c r="U4" s="83"/>
+      <c r="V4" s="83"/>
+      <c r="W4" s="83"/>
+      <c r="X4" s="83"/>
+      <c r="Y4" s="83"/>
+      <c r="Z4" s="83"/>
+      <c r="AA4" s="83"/>
+      <c r="AB4" s="83"/>
+      <c r="AC4" s="83"/>
+      <c r="AD4" s="83"/>
+      <c r="AE4" s="83"/>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A5" s="83">
+        <v>2018</v>
+      </c>
+      <c r="B5" s="83">
+        <f>('Financial Year Averages'!B6-'Financial Year Averages'!B5)/'Financial Year Averages'!B5*100</f>
+        <v>1.7116503409989505</v>
+      </c>
+      <c r="C5" s="83">
+        <f>('Financial Year Averages'!C6-'Financial Year Averages'!C5)/'Financial Year Averages'!C5*100</f>
+        <v>1.4652929035837028</v>
+      </c>
+      <c r="D5" s="83">
+        <f>('Financial Year Averages'!D6-'Financial Year Averages'!D5)/'Financial Year Averages'!D5*100</f>
+        <v>2.5998950591335892</v>
+      </c>
+      <c r="E5" s="83">
+        <f>('Financial Year Averages'!E6-'Financial Year Averages'!E5)/'Financial Year Averages'!E5*100</f>
+        <v>-0.52708347145793322</v>
+      </c>
+      <c r="F5" s="83">
+        <f>('Financial Year Averages'!F6-'Financial Year Averages'!F5)/'Financial Year Averages'!F5*100</f>
+        <v>1.7536303079129529</v>
+      </c>
+      <c r="G5" s="83">
+        <f>('Financial Year Averages'!G6-'Financial Year Averages'!G5)/'Financial Year Averages'!G5*100</f>
+        <v>0.82053142374069132</v>
+      </c>
+      <c r="H5" s="83">
+        <f>('Financial Year Averages'!H6-'Financial Year Averages'!H5)/'Financial Year Averages'!H5*100</f>
+        <v>2.7324585410366597</v>
+      </c>
+      <c r="I5" s="83">
+        <f>('Financial Year Averages'!I6-'Financial Year Averages'!I5)/'Financial Year Averages'!I5*100</f>
+        <v>1.6446826362694997</v>
+      </c>
+      <c r="J5" s="83">
+        <f>('Financial Year Averages'!J6-'Financial Year Averages'!J5)/'Financial Year Averages'!J5*100</f>
+        <v>4.1613384859284981</v>
+      </c>
+      <c r="K5" s="83">
+        <f>('Financial Year Averages'!K6-'Financial Year Averages'!K5)/'Financial Year Averages'!K5*100</f>
+        <v>1.5325106143596829</v>
+      </c>
+      <c r="L5" s="83">
+        <f>('Financial Year Averages'!L6-'Financial Year Averages'!L5)/'Financial Year Averages'!L5*100</f>
+        <v>2.9454797901197973</v>
+      </c>
+      <c r="M5" s="83">
+        <f>('Financial Year Averages'!M6-'Financial Year Averages'!M5)/'Financial Year Averages'!M5*100</f>
+        <v>2.5701129092990405</v>
+      </c>
+      <c r="N5" s="83">
+        <f>('Financial Year Averages'!N6-'Financial Year Averages'!N5)/'Financial Year Averages'!N5*100</f>
+        <v>1.7796212036237817</v>
+      </c>
+      <c r="O5" s="83">
+        <f>('Financial Year Averages'!O6-'Financial Year Averages'!O5)/'Financial Year Averages'!O5*100</f>
+        <v>0.75518397884487132</v>
+      </c>
+      <c r="P5" s="83"/>
+      <c r="Q5" s="83"/>
+      <c r="R5" s="83"/>
+      <c r="S5" s="83"/>
+      <c r="T5" s="83"/>
+      <c r="U5" s="83"/>
+      <c r="V5" s="83"/>
+      <c r="W5" s="83"/>
+      <c r="X5" s="83"/>
+      <c r="Y5" s="83"/>
+      <c r="Z5" s="83"/>
+      <c r="AA5" s="83"/>
+      <c r="AB5" s="83"/>
+      <c r="AC5" s="83"/>
+      <c r="AD5" s="83"/>
+      <c r="AE5" s="83"/>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A6" s="83">
+        <v>2019</v>
+      </c>
+      <c r="B6" s="83">
+        <f>('Financial Year Averages'!B7-'Financial Year Averages'!B6)/'Financial Year Averages'!B6*100</f>
+        <v>0.80470211471989572</v>
+      </c>
+      <c r="C6" s="83">
+        <f>('Financial Year Averages'!C7-'Financial Year Averages'!C6)/'Financial Year Averages'!C6*100</f>
+        <v>0.15283905990713728</v>
+      </c>
+      <c r="D6" s="83">
+        <f>('Financial Year Averages'!D7-'Financial Year Averages'!D6)/'Financial Year Averages'!D6*100</f>
+        <v>2.5038664352738129</v>
+      </c>
+      <c r="E6" s="83">
+        <f>('Financial Year Averages'!E7-'Financial Year Averages'!E6)/'Financial Year Averages'!E6*100</f>
+        <v>-2.3710727659480892</v>
+      </c>
+      <c r="F6" s="83">
+        <f>('Financial Year Averages'!F7-'Financial Year Averages'!F6)/'Financial Year Averages'!F6*100</f>
+        <v>0.61934857939142818</v>
+      </c>
+      <c r="G6" s="83">
+        <f>('Financial Year Averages'!G7-'Financial Year Averages'!G6)/'Financial Year Averages'!G6*100</f>
+        <v>0.23007271502447105</v>
+      </c>
+      <c r="H6" s="83">
+        <f>('Financial Year Averages'!H7-'Financial Year Averages'!H6)/'Financial Year Averages'!H6*100</f>
+        <v>1.6702349345575112</v>
+      </c>
+      <c r="I6" s="83">
+        <f>('Financial Year Averages'!I7-'Financial Year Averages'!I6)/'Financial Year Averages'!I6*100</f>
+        <v>0.7139946218007448</v>
+      </c>
+      <c r="J6" s="83">
+        <f>('Financial Year Averages'!J7-'Financial Year Averages'!J6)/'Financial Year Averages'!J6*100</f>
+        <v>3.28799318208271</v>
+      </c>
+      <c r="K6" s="83">
+        <f>('Financial Year Averages'!K7-'Financial Year Averages'!K6)/'Financial Year Averages'!K6*100</f>
+        <v>2.2629113270576102</v>
+      </c>
+      <c r="L6" s="83">
+        <f>('Financial Year Averages'!L7-'Financial Year Averages'!L6)/'Financial Year Averages'!L6*100</f>
+        <v>2.3814636521568913</v>
+      </c>
+      <c r="M6" s="83">
+        <f>('Financial Year Averages'!M7-'Financial Year Averages'!M6)/'Financial Year Averages'!M6*100</f>
+        <v>0.61604058585289057</v>
+      </c>
+      <c r="N6" s="83">
+        <f>('Financial Year Averages'!N7-'Financial Year Averages'!N6)/'Financial Year Averages'!N6*100</f>
+        <v>0.81663423075784802</v>
+      </c>
+      <c r="O6" s="83">
+        <f>('Financial Year Averages'!O7-'Financial Year Averages'!O6)/'Financial Year Averages'!O6*100</f>
+        <v>1.6716450872870463</v>
+      </c>
+      <c r="P6" s="83"/>
+      <c r="Q6" s="83"/>
+      <c r="R6" s="83"/>
+      <c r="S6" s="83"/>
+      <c r="T6" s="83"/>
+      <c r="U6" s="83"/>
+      <c r="V6" s="83"/>
+      <c r="W6" s="83"/>
+      <c r="X6" s="83"/>
+      <c r="Y6" s="83"/>
+      <c r="Z6" s="83"/>
+      <c r="AA6" s="83"/>
+      <c r="AB6" s="83"/>
+      <c r="AC6" s="83"/>
+      <c r="AD6" s="83"/>
+      <c r="AE6" s="83"/>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A7" s="83">
+        <v>2020</v>
+      </c>
+      <c r="B7" s="83">
+        <f>('Financial Year Averages'!B8-'Financial Year Averages'!B7)/'Financial Year Averages'!B7*100</f>
+        <v>3.674310374716578</v>
+      </c>
+      <c r="C7" s="83">
+        <f>('Financial Year Averages'!C8-'Financial Year Averages'!C7)/'Financial Year Averages'!C7*100</f>
+        <v>1.7882415651368131</v>
+      </c>
+      <c r="D7" s="83">
+        <f>('Financial Year Averages'!D8-'Financial Year Averages'!D7)/'Financial Year Averages'!D7*100</f>
+        <v>2.9843543041077734</v>
+      </c>
+      <c r="E7" s="83">
+        <f>('Financial Year Averages'!E8-'Financial Year Averages'!E7)/'Financial Year Averages'!E7*100</f>
+        <v>3.3510501899899801</v>
+      </c>
+      <c r="F7" s="83">
+        <f>('Financial Year Averages'!F8-'Financial Year Averages'!F7)/'Financial Year Averages'!F7*100</f>
+        <v>3.0168032648448642</v>
+      </c>
+      <c r="G7" s="83">
+        <f>('Financial Year Averages'!G8-'Financial Year Averages'!G7)/'Financial Year Averages'!G7*100</f>
+        <v>5.6384312844850388</v>
+      </c>
+      <c r="H7" s="83">
+        <f>('Financial Year Averages'!H8-'Financial Year Averages'!H7)/'Financial Year Averages'!H7*100</f>
+        <v>1.8347491420517277</v>
+      </c>
+      <c r="I7" s="83">
+        <f>('Financial Year Averages'!I8-'Financial Year Averages'!I7)/'Financial Year Averages'!I7*100</f>
+        <v>9.6027509637898447</v>
+      </c>
+      <c r="J7" s="83">
+        <f>('Financial Year Averages'!J8-'Financial Year Averages'!J7)/'Financial Year Averages'!J7*100</f>
+        <v>1.5562230748763568</v>
+      </c>
+      <c r="K7" s="83">
+        <f>('Financial Year Averages'!K8-'Financial Year Averages'!K7)/'Financial Year Averages'!K7*100</f>
+        <v>2.623635888930326</v>
+      </c>
+      <c r="L7" s="83">
+        <f>('Financial Year Averages'!L8-'Financial Year Averages'!L7)/'Financial Year Averages'!L7*100</f>
+        <v>3.3994560814152139</v>
+      </c>
+      <c r="M7" s="83">
+        <f>('Financial Year Averages'!M8-'Financial Year Averages'!M7)/'Financial Year Averages'!M7*100</f>
+        <v>4.5963451854790245</v>
+      </c>
+      <c r="N7" s="83">
+        <f>('Financial Year Averages'!N8-'Financial Year Averages'!N7)/'Financial Year Averages'!N7*100</f>
+        <v>1.3241827921983071</v>
+      </c>
+      <c r="O7" s="83">
+        <f>('Financial Year Averages'!O8-'Financial Year Averages'!O7)/'Financial Year Averages'!O7*100</f>
+        <v>1.8179342650584014</v>
+      </c>
+      <c r="P7" s="83"/>
+      <c r="Q7" s="83"/>
+      <c r="R7" s="83"/>
+      <c r="S7" s="83"/>
+      <c r="T7" s="83"/>
+      <c r="U7" s="83"/>
+      <c r="V7" s="83"/>
+      <c r="W7" s="83"/>
+      <c r="X7" s="83"/>
+      <c r="Y7" s="83"/>
+      <c r="Z7" s="83"/>
+      <c r="AA7" s="83"/>
+      <c r="AB7" s="83"/>
+      <c r="AC7" s="83"/>
+      <c r="AD7" s="83"/>
+      <c r="AE7" s="83"/>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A8" s="83">
+        <v>2021</v>
+      </c>
+      <c r="B8" s="83">
+        <f>('Financial Year Averages'!B9-'Financial Year Averages'!B8)/'Financial Year Averages'!B8*100</f>
+        <v>8.7636900429890048</v>
+      </c>
+      <c r="C8" s="83">
+        <f>('Financial Year Averages'!C9-'Financial Year Averages'!C8)/'Financial Year Averages'!C8*100</f>
+        <v>14.198533244897952</v>
+      </c>
+      <c r="D8" s="83">
+        <f>('Financial Year Averages'!D9-'Financial Year Averages'!D8)/'Financial Year Averages'!D8*100</f>
+        <v>5.0844705024188626</v>
+      </c>
+      <c r="E8" s="83">
+        <f>('Financial Year Averages'!E9-'Financial Year Averages'!E8)/'Financial Year Averages'!E8*100</f>
+        <v>7.3122672926436971</v>
+      </c>
+      <c r="F8" s="83">
+        <f>('Financial Year Averages'!F9-'Financial Year Averages'!F8)/'Financial Year Averages'!F8*100</f>
+        <v>10.364848077466201</v>
+      </c>
+      <c r="G8" s="83">
+        <f>('Financial Year Averages'!G9-'Financial Year Averages'!G8)/'Financial Year Averages'!G8*100</f>
+        <v>9.9937424493969385</v>
+      </c>
+      <c r="H8" s="83">
+        <f>('Financial Year Averages'!H9-'Financial Year Averages'!H8)/'Financial Year Averages'!H8*100</f>
+        <v>3.9498170944141284</v>
+      </c>
+      <c r="I8" s="83">
+        <f>('Financial Year Averages'!I9-'Financial Year Averages'!I8)/'Financial Year Averages'!I8*100</f>
+        <v>9.2222256655828794</v>
+      </c>
+      <c r="J8" s="83">
+        <f>('Financial Year Averages'!J9-'Financial Year Averages'!J8)/'Financial Year Averages'!J8*100</f>
+        <v>2.7883700637303219</v>
+      </c>
+      <c r="K8" s="83">
+        <f>('Financial Year Averages'!K9-'Financial Year Averages'!K8)/'Financial Year Averages'!K8*100</f>
+        <v>5.1326810250950254</v>
+      </c>
+      <c r="L8" s="83">
+        <f>('Financial Year Averages'!L9-'Financial Year Averages'!L8)/'Financial Year Averages'!L8*100</f>
+        <v>3.801720845321372</v>
+      </c>
+      <c r="M8" s="83">
+        <f>('Financial Year Averages'!M9-'Financial Year Averages'!M8)/'Financial Year Averages'!M8*100</f>
+        <v>9.7511515520303274</v>
+      </c>
+      <c r="N8" s="83">
+        <f>('Financial Year Averages'!N9-'Financial Year Averages'!N8)/'Financial Year Averages'!N8*100</f>
+        <v>4.8159880421152588</v>
+      </c>
+      <c r="O8" s="83">
+        <f>('Financial Year Averages'!O9-'Financial Year Averages'!O8)/'Financial Year Averages'!O8*100</f>
+        <v>4.0575334481961756</v>
+      </c>
+      <c r="P8" s="83"/>
+      <c r="Q8" s="83"/>
+      <c r="R8" s="83"/>
+      <c r="S8" s="83"/>
+      <c r="T8" s="83"/>
+      <c r="U8" s="83"/>
+      <c r="V8" s="83"/>
+      <c r="W8" s="83"/>
+      <c r="X8" s="83"/>
+      <c r="Y8" s="83"/>
+      <c r="Z8" s="83"/>
+      <c r="AA8" s="83"/>
+      <c r="AB8" s="83"/>
+      <c r="AC8" s="83"/>
+      <c r="AD8" s="83"/>
+      <c r="AE8" s="83"/>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A9" s="83">
+        <v>2022</v>
+      </c>
+      <c r="B9" s="83">
+        <f>('Financial Year Averages'!B10-'Financial Year Averages'!B9)/'Financial Year Averages'!B9*100</f>
+        <v>5.5552620742715639</v>
+      </c>
+      <c r="C9" s="83">
+        <f>('Financial Year Averages'!C10-'Financial Year Averages'!C9)/'Financial Year Averages'!C9*100</f>
+        <v>11.324017508263109</v>
+      </c>
+      <c r="D9" s="83">
+        <f>('Financial Year Averages'!D10-'Financial Year Averages'!D9)/'Financial Year Averages'!D9*100</f>
+        <v>10.696464307792214</v>
+      </c>
+      <c r="E9" s="83">
+        <f>('Financial Year Averages'!E10-'Financial Year Averages'!E9)/'Financial Year Averages'!E9*100</f>
+        <v>6.1667034496426405</v>
+      </c>
+      <c r="F9" s="83">
+        <f>('Financial Year Averages'!F10-'Financial Year Averages'!F9)/'Financial Year Averages'!F9*100</f>
+        <v>4.3661423091492786</v>
+      </c>
+      <c r="G9" s="83">
+        <f>('Financial Year Averages'!G10-'Financial Year Averages'!G9)/'Financial Year Averages'!G9*100</f>
+        <v>3.6336144038010119</v>
+      </c>
+      <c r="H9" s="83">
+        <f>('Financial Year Averages'!H10-'Financial Year Averages'!H9)/'Financial Year Averages'!H9*100</f>
+        <v>7.8023766582249703</v>
+      </c>
+      <c r="I9" s="83">
+        <f>('Financial Year Averages'!I10-'Financial Year Averages'!I9)/'Financial Year Averages'!I9*100</f>
+        <v>-0.34782297605454288</v>
+      </c>
+      <c r="J9" s="83">
+        <f>('Financial Year Averages'!J10-'Financial Year Averages'!J9)/'Financial Year Averages'!J9*100</f>
+        <v>7.9547527950448931</v>
+      </c>
+      <c r="K9" s="83">
+        <f>('Financial Year Averages'!K10-'Financial Year Averages'!K9)/'Financial Year Averages'!K9*100</f>
+        <v>6.1832640343545648</v>
+      </c>
+      <c r="L9" s="83">
+        <f>('Financial Year Averages'!L10-'Financial Year Averages'!L9)/'Financial Year Averages'!L9*100</f>
+        <v>3.9009673991328144</v>
+      </c>
+      <c r="M9" s="83">
+        <f>('Financial Year Averages'!M10-'Financial Year Averages'!M9)/'Financial Year Averages'!M9*100</f>
+        <v>8.1177262423894323</v>
+      </c>
+      <c r="N9" s="83">
+        <f>('Financial Year Averages'!N10-'Financial Year Averages'!N9)/'Financial Year Averages'!N9*100</f>
+        <v>4.9911244368865404</v>
+      </c>
+      <c r="O9" s="83">
+        <f>('Financial Year Averages'!O10-'Financial Year Averages'!O9)/'Financial Year Averages'!O9*100</f>
+        <v>6.2927775012813489</v>
+      </c>
+      <c r="P9" s="83"/>
+      <c r="Q9" s="83"/>
+      <c r="R9" s="83"/>
+      <c r="S9" s="83"/>
+      <c r="T9" s="83"/>
+      <c r="U9" s="83"/>
+      <c r="V9" s="83"/>
+      <c r="W9" s="83"/>
+      <c r="X9" s="83"/>
+      <c r="Y9" s="83"/>
+      <c r="Z9" s="83"/>
+      <c r="AA9" s="83"/>
+      <c r="AB9" s="83"/>
+      <c r="AC9" s="83"/>
+      <c r="AD9" s="83"/>
+      <c r="AE9" s="83"/>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A10" s="83">
+        <v>2023</v>
+      </c>
+      <c r="B10" s="83">
+        <f>('Financial Year Averages'!B11-'Financial Year Averages'!B10)/'Financial Year Averages'!B10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="C10" s="83">
+        <f>('Financial Year Averages'!C11-'Financial Year Averages'!C10)/'Financial Year Averages'!C10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="D10" s="83">
+        <f>('Financial Year Averages'!D11-'Financial Year Averages'!D10)/'Financial Year Averages'!D10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="E10" s="83">
+        <f>('Financial Year Averages'!E11-'Financial Year Averages'!E10)/'Financial Year Averages'!E10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="F10" s="83">
+        <f>('Financial Year Averages'!F11-'Financial Year Averages'!F10)/'Financial Year Averages'!F10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="G10" s="83">
+        <f>('Financial Year Averages'!G11-'Financial Year Averages'!G10)/'Financial Year Averages'!G10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="H10" s="83">
+        <f>('Financial Year Averages'!H11-'Financial Year Averages'!H10)/'Financial Year Averages'!H10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="I10" s="83">
+        <f>('Financial Year Averages'!I11-'Financial Year Averages'!I10)/'Financial Year Averages'!I10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="J10" s="83">
+        <f>('Financial Year Averages'!J11-'Financial Year Averages'!J10)/'Financial Year Averages'!J10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="K10" s="83">
+        <f>('Financial Year Averages'!K11-'Financial Year Averages'!K10)/'Financial Year Averages'!K10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="L10" s="83">
+        <f>('Financial Year Averages'!L11-'Financial Year Averages'!L10)/'Financial Year Averages'!L10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="M10" s="83">
+        <f>('Financial Year Averages'!M11-'Financial Year Averages'!M10)/'Financial Year Averages'!M10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="N10" s="83">
+        <f>('Financial Year Averages'!N11-'Financial Year Averages'!N10)/'Financial Year Averages'!N10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="O10" s="83">
+        <f>('Financial Year Averages'!O11-'Financial Year Averages'!O10)/'Financial Year Averages'!O10*100</f>
+        <v>-100</v>
+      </c>
+      <c r="P10" s="83"/>
+      <c r="Q10" s="83"/>
+      <c r="R10" s="83"/>
+      <c r="S10" s="83"/>
+      <c r="T10" s="83"/>
+      <c r="U10" s="83"/>
+      <c r="V10" s="83"/>
+      <c r="W10" s="83"/>
+      <c r="X10" s="83"/>
+      <c r="Y10" s="83"/>
+      <c r="Z10" s="83"/>
+      <c r="AA10" s="83"/>
+      <c r="AB10" s="83"/>
+      <c r="AC10" s="83"/>
+      <c r="AD10" s="83"/>
+      <c r="AE10" s="83"/>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A11" s="83"/>
+      <c r="B11" s="83"/>
+      <c r="C11" s="83"/>
+      <c r="D11" s="83"/>
+      <c r="E11" s="83"/>
+      <c r="F11" s="83"/>
+      <c r="G11" s="83"/>
+      <c r="H11" s="83"/>
+      <c r="I11" s="83"/>
+      <c r="J11" s="83"/>
+      <c r="K11" s="83"/>
+      <c r="L11" s="83"/>
+      <c r="M11" s="83"/>
+      <c r="N11" s="83"/>
+      <c r="O11" s="83"/>
+      <c r="P11" s="83"/>
+      <c r="Q11" s="83"/>
+      <c r="R11" s="83"/>
+      <c r="S11" s="83"/>
+      <c r="T11" s="83"/>
+      <c r="U11" s="83"/>
+      <c r="V11" s="83"/>
+      <c r="W11" s="83"/>
+      <c r="X11" s="83"/>
+      <c r="Y11" s="83"/>
+      <c r="Z11" s="83"/>
+      <c r="AA11" s="83"/>
+      <c r="AB11" s="83"/>
+      <c r="AC11" s="83"/>
+      <c r="AD11" s="83"/>
+      <c r="AE11" s="83"/>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A12" s="83"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="83"/>
+      <c r="F12" s="83"/>
+      <c r="G12" s="83"/>
+      <c r="H12" s="83"/>
+      <c r="I12" s="83"/>
+      <c r="J12" s="83"/>
+      <c r="K12" s="83"/>
+      <c r="L12" s="83"/>
+      <c r="M12" s="83"/>
+      <c r="N12" s="83"/>
+      <c r="O12" s="83"/>
+      <c r="P12" s="83"/>
+      <c r="Q12" s="83"/>
+      <c r="R12" s="83"/>
+      <c r="S12" s="83"/>
+      <c r="T12" s="83"/>
+      <c r="U12" s="83"/>
+      <c r="V12" s="83"/>
+      <c r="W12" s="83"/>
+      <c r="X12" s="83"/>
+      <c r="Y12" s="83"/>
+      <c r="Z12" s="83"/>
+      <c r="AA12" s="83"/>
+      <c r="AB12" s="83"/>
+      <c r="AC12" s="83"/>
+      <c r="AD12" s="83"/>
+      <c r="AE12" s="83"/>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A13" s="83"/>
+      <c r="B13" s="83"/>
+      <c r="C13" s="83"/>
+      <c r="D13" s="83"/>
+      <c r="E13" s="83"/>
+      <c r="F13" s="83"/>
+      <c r="G13" s="83"/>
+      <c r="H13" s="83"/>
+      <c r="I13" s="83"/>
+      <c r="J13" s="83"/>
+      <c r="K13" s="83"/>
+      <c r="L13" s="83"/>
+      <c r="M13" s="83"/>
+      <c r="N13" s="83"/>
+      <c r="O13" s="83"/>
+      <c r="P13" s="83"/>
+      <c r="Q13" s="83"/>
+      <c r="R13" s="83"/>
+      <c r="S13" s="83"/>
+      <c r="T13" s="83"/>
+      <c r="U13" s="83"/>
+      <c r="V13" s="83"/>
+      <c r="W13" s="83"/>
+      <c r="X13" s="83"/>
+      <c r="Y13" s="83"/>
+      <c r="Z13" s="83"/>
+      <c r="AA13" s="83"/>
+      <c r="AB13" s="83"/>
+      <c r="AC13" s="83"/>
+      <c r="AD13" s="83"/>
+      <c r="AE13" s="83"/>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A14" s="83"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
+      <c r="D14" s="83"/>
+      <c r="E14" s="83"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="83"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="83"/>
+      <c r="J14" s="83"/>
+      <c r="K14" s="83"/>
+      <c r="L14" s="83"/>
+      <c r="M14" s="83"/>
+      <c r="N14" s="83"/>
+      <c r="O14" s="83"/>
+      <c r="P14" s="83"/>
+      <c r="Q14" s="83"/>
+      <c r="R14" s="83"/>
+      <c r="S14" s="83"/>
+      <c r="T14" s="83"/>
+      <c r="U14" s="83"/>
+      <c r="V14" s="83"/>
+      <c r="W14" s="83"/>
+      <c r="X14" s="83"/>
+      <c r="Y14" s="83"/>
+      <c r="Z14" s="83"/>
+      <c r="AA14" s="83"/>
+      <c r="AB14" s="83"/>
+      <c r="AC14" s="83"/>
+      <c r="AD14" s="83"/>
+      <c r="AE14" s="83"/>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A15" s="83"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="83"/>
+      <c r="D15" s="83"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="83"/>
+      <c r="H15" s="83"/>
+      <c r="I15" s="83"/>
+      <c r="J15" s="83"/>
+      <c r="K15" s="83"/>
+      <c r="L15" s="83"/>
+      <c r="M15" s="83"/>
+      <c r="N15" s="83"/>
+      <c r="O15" s="83"/>
+      <c r="P15" s="83"/>
+      <c r="Q15" s="83"/>
+      <c r="R15" s="83"/>
+      <c r="S15" s="83"/>
+      <c r="T15" s="83"/>
+      <c r="U15" s="83"/>
+      <c r="V15" s="83"/>
+      <c r="W15" s="83"/>
+      <c r="X15" s="83"/>
+      <c r="Y15" s="83"/>
+      <c r="Z15" s="83"/>
+      <c r="AA15" s="83"/>
+      <c r="AB15" s="83"/>
+      <c r="AC15" s="83"/>
+      <c r="AD15" s="83"/>
+      <c r="AE15" s="83"/>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A16" s="83"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="83"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="83"/>
+      <c r="G16" s="83"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="83"/>
+      <c r="J16" s="83"/>
+      <c r="K16" s="83"/>
+      <c r="L16" s="83"/>
+      <c r="M16" s="83"/>
+      <c r="N16" s="83"/>
+      <c r="O16" s="83"/>
+      <c r="P16" s="83"/>
+      <c r="Q16" s="83"/>
+      <c r="R16" s="83"/>
+      <c r="S16" s="83"/>
+      <c r="T16" s="83"/>
+      <c r="U16" s="83"/>
+      <c r="V16" s="83"/>
+      <c r="W16" s="83"/>
+      <c r="X16" s="83"/>
+      <c r="Y16" s="83"/>
+      <c r="Z16" s="83"/>
+      <c r="AA16" s="83"/>
+      <c r="AB16" s="83"/>
+      <c r="AC16" s="83"/>
+      <c r="AD16" s="83"/>
+      <c r="AE16" s="83"/>
+    </row>
+    <row r="17" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A17" s="83"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="E17" s="83"/>
+      <c r="F17" s="83"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="83"/>
+      <c r="I17" s="83"/>
+      <c r="J17" s="83"/>
+      <c r="K17" s="83"/>
+      <c r="L17" s="83"/>
+      <c r="M17" s="83"/>
+      <c r="N17" s="83"/>
+      <c r="O17" s="83"/>
+      <c r="P17" s="83"/>
+      <c r="Q17" s="83"/>
+      <c r="R17" s="83"/>
+      <c r="S17" s="83"/>
+      <c r="T17" s="83"/>
+      <c r="U17" s="83"/>
+      <c r="V17" s="83"/>
+      <c r="W17" s="83"/>
+      <c r="X17" s="83"/>
+      <c r="Y17" s="83"/>
+      <c r="Z17" s="83"/>
+      <c r="AA17" s="83"/>
+      <c r="AB17" s="83"/>
+      <c r="AC17" s="83"/>
+      <c r="AD17" s="83"/>
+      <c r="AE17" s="83"/>
+    </row>
+    <row r="18" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A18" s="83"/>
+      <c r="B18" s="83"/>
+      <c r="C18" s="83"/>
+      <c r="D18" s="83"/>
+      <c r="E18" s="83"/>
+      <c r="F18" s="83"/>
+      <c r="G18" s="83"/>
+      <c r="H18" s="83"/>
+      <c r="I18" s="83"/>
+      <c r="J18" s="83"/>
+      <c r="K18" s="83"/>
+      <c r="L18" s="83"/>
+      <c r="M18" s="83"/>
+      <c r="N18" s="83"/>
+      <c r="O18" s="83"/>
+      <c r="P18" s="83"/>
+      <c r="Q18" s="83"/>
+      <c r="R18" s="83"/>
+      <c r="S18" s="83"/>
+      <c r="T18" s="83"/>
+      <c r="U18" s="83"/>
+      <c r="V18" s="83"/>
+      <c r="W18" s="83"/>
+      <c r="X18" s="83"/>
+      <c r="Y18" s="83"/>
+      <c r="Z18" s="83"/>
+      <c r="AA18" s="83"/>
+      <c r="AB18" s="83"/>
+      <c r="AC18" s="83"/>
+      <c r="AD18" s="83"/>
+      <c r="AE18" s="83"/>
+    </row>
+    <row r="19" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A19" s="83"/>
+      <c r="B19" s="83"/>
+      <c r="C19" s="83"/>
+      <c r="D19" s="83"/>
+      <c r="E19" s="83"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="83"/>
+      <c r="H19" s="83"/>
+      <c r="I19" s="83"/>
+      <c r="J19" s="83"/>
+      <c r="K19" s="83"/>
+      <c r="L19" s="83"/>
+      <c r="M19" s="83"/>
+      <c r="N19" s="83"/>
+      <c r="O19" s="83"/>
+      <c r="P19" s="83"/>
+      <c r="Q19" s="83"/>
+      <c r="R19" s="83"/>
+      <c r="S19" s="83"/>
+      <c r="T19" s="83"/>
+      <c r="U19" s="83"/>
+      <c r="V19" s="83"/>
+      <c r="W19" s="83"/>
+      <c r="X19" s="83"/>
+      <c r="Y19" s="83"/>
+      <c r="Z19" s="83"/>
+      <c r="AA19" s="83"/>
+      <c r="AB19" s="83"/>
+      <c r="AC19" s="83"/>
+      <c r="AD19" s="83"/>
+      <c r="AE19" s="83"/>
+    </row>
+    <row r="20" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A20" s="83"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="83"/>
+      <c r="D20" s="83"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="83"/>
+      <c r="G20" s="83"/>
+      <c r="H20" s="83"/>
+      <c r="I20" s="83"/>
+      <c r="J20" s="83"/>
+      <c r="K20" s="83"/>
+      <c r="L20" s="83"/>
+      <c r="M20" s="83"/>
+      <c r="N20" s="83"/>
+      <c r="O20" s="83"/>
+      <c r="P20" s="83"/>
+      <c r="Q20" s="83"/>
+      <c r="R20" s="83"/>
+      <c r="S20" s="83"/>
+      <c r="T20" s="83"/>
+      <c r="U20" s="83"/>
+      <c r="V20" s="83"/>
+      <c r="W20" s="83"/>
+      <c r="X20" s="83"/>
+      <c r="Y20" s="83"/>
+      <c r="Z20" s="83"/>
+      <c r="AA20" s="83"/>
+      <c r="AB20" s="83"/>
+      <c r="AC20" s="83"/>
+      <c r="AD20" s="83"/>
+      <c r="AE20" s="83"/>
+    </row>
+    <row r="21" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A21" s="83"/>
+      <c r="B21" s="83"/>
+      <c r="C21" s="83"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="83"/>
+      <c r="J21" s="83"/>
+      <c r="K21" s="83"/>
+      <c r="L21" s="83"/>
+      <c r="M21" s="83"/>
+      <c r="N21" s="83"/>
+      <c r="O21" s="83"/>
+      <c r="P21" s="83"/>
+      <c r="Q21" s="83"/>
+      <c r="R21" s="83"/>
+      <c r="S21" s="83"/>
+      <c r="T21" s="83"/>
+      <c r="U21" s="83"/>
+      <c r="V21" s="83"/>
+      <c r="W21" s="83"/>
+      <c r="X21" s="83"/>
+      <c r="Y21" s="83"/>
+      <c r="Z21" s="83"/>
+      <c r="AA21" s="83"/>
+      <c r="AB21" s="83"/>
+      <c r="AC21" s="83"/>
+      <c r="AD21" s="83"/>
+      <c r="AE21" s="83"/>
+    </row>
+    <row r="22" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A22" s="83"/>
+      <c r="B22" s="83"/>
+      <c r="C22" s="83"/>
+      <c r="D22" s="83"/>
+      <c r="E22" s="83"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="83"/>
+      <c r="H22" s="83"/>
+      <c r="I22" s="83"/>
+      <c r="J22" s="83"/>
+      <c r="K22" s="83"/>
+      <c r="L22" s="83"/>
+      <c r="M22" s="83"/>
+      <c r="N22" s="83"/>
+      <c r="O22" s="83"/>
+      <c r="P22" s="83"/>
+      <c r="Q22" s="83"/>
+      <c r="R22" s="83"/>
+      <c r="S22" s="83"/>
+      <c r="T22" s="83"/>
+      <c r="U22" s="83"/>
+      <c r="V22" s="83"/>
+      <c r="W22" s="83"/>
+      <c r="X22" s="83"/>
+      <c r="Y22" s="83"/>
+      <c r="Z22" s="83"/>
+      <c r="AA22" s="83"/>
+      <c r="AB22" s="83"/>
+      <c r="AC22" s="83"/>
+      <c r="AD22" s="83"/>
+      <c r="AE22" s="83"/>
+    </row>
+    <row r="23" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A23" s="83"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="83"/>
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="83"/>
+      <c r="H23" s="83"/>
+      <c r="I23" s="83"/>
+      <c r="J23" s="83"/>
+      <c r="K23" s="83"/>
+      <c r="L23" s="83"/>
+      <c r="M23" s="83"/>
+      <c r="N23" s="83"/>
+      <c r="O23" s="83"/>
+      <c r="P23" s="83"/>
+      <c r="Q23" s="83"/>
+      <c r="R23" s="83"/>
+      <c r="S23" s="83"/>
+      <c r="T23" s="83"/>
+      <c r="U23" s="83"/>
+      <c r="V23" s="83"/>
+      <c r="W23" s="83"/>
+      <c r="X23" s="83"/>
+      <c r="Y23" s="83"/>
+      <c r="Z23" s="83"/>
+      <c r="AA23" s="83"/>
+      <c r="AB23" s="83"/>
+      <c r="AC23" s="83"/>
+      <c r="AD23" s="83"/>
+      <c r="AE23" s="83"/>
+    </row>
+    <row r="24" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A24" s="83"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="83"/>
+      <c r="E24" s="83"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="83"/>
+      <c r="H24" s="83"/>
+      <c r="I24" s="83"/>
+      <c r="J24" s="83"/>
+      <c r="K24" s="83"/>
+      <c r="L24" s="83"/>
+      <c r="M24" s="83"/>
+      <c r="N24" s="83"/>
+      <c r="O24" s="83"/>
+      <c r="P24" s="83"/>
+      <c r="Q24" s="83"/>
+      <c r="R24" s="83"/>
+      <c r="S24" s="83"/>
+      <c r="T24" s="83"/>
+      <c r="U24" s="83"/>
+      <c r="V24" s="83"/>
+      <c r="W24" s="83"/>
+      <c r="X24" s="83"/>
+      <c r="Y24" s="83"/>
+      <c r="Z24" s="83"/>
+      <c r="AA24" s="83"/>
+      <c r="AB24" s="83"/>
+      <c r="AC24" s="83"/>
+      <c r="AD24" s="83"/>
+      <c r="AE24" s="83"/>
+    </row>
+    <row r="25" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A25" s="83"/>
+      <c r="B25" s="83"/>
+      <c r="C25" s="83"/>
+      <c r="D25" s="83"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="83"/>
+      <c r="H25" s="83"/>
+      <c r="I25" s="83"/>
+      <c r="J25" s="83"/>
+      <c r="K25" s="83"/>
+      <c r="L25" s="83"/>
+      <c r="M25" s="83"/>
+      <c r="N25" s="83"/>
+      <c r="O25" s="83"/>
+      <c r="P25" s="83"/>
+      <c r="Q25" s="83"/>
+      <c r="R25" s="83"/>
+      <c r="S25" s="83"/>
+      <c r="T25" s="83"/>
+      <c r="U25" s="83"/>
+      <c r="V25" s="83"/>
+      <c r="W25" s="83"/>
+      <c r="X25" s="83"/>
+      <c r="Y25" s="83"/>
+      <c r="Z25" s="83"/>
+      <c r="AA25" s="83"/>
+      <c r="AB25" s="83"/>
+      <c r="AC25" s="83"/>
+      <c r="AD25" s="83"/>
+      <c r="AE25" s="83"/>
+    </row>
+    <row r="26" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A26" s="83"/>
+      <c r="B26" s="83"/>
+      <c r="C26" s="83"/>
+      <c r="D26" s="83"/>
+      <c r="E26" s="83"/>
+      <c r="F26" s="83"/>
+      <c r="G26" s="83"/>
+      <c r="H26" s="83"/>
+      <c r="I26" s="83"/>
+      <c r="J26" s="83"/>
+      <c r="K26" s="83"/>
+      <c r="L26" s="83"/>
+      <c r="M26" s="83"/>
+      <c r="N26" s="83"/>
+      <c r="O26" s="83"/>
+      <c r="P26" s="83"/>
+      <c r="Q26" s="83"/>
+      <c r="R26" s="83"/>
+      <c r="S26" s="83"/>
+      <c r="T26" s="83"/>
+      <c r="U26" s="83"/>
+      <c r="V26" s="83"/>
+      <c r="W26" s="83"/>
+      <c r="X26" s="83"/>
+      <c r="Y26" s="83"/>
+      <c r="Z26" s="83"/>
+      <c r="AA26" s="83"/>
+      <c r="AB26" s="83"/>
+      <c r="AC26" s="83"/>
+      <c r="AD26" s="83"/>
+      <c r="AE26" s="83"/>
+    </row>
+    <row r="27" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A27" s="83"/>
+      <c r="B27" s="83"/>
+      <c r="C27" s="83"/>
+      <c r="D27" s="83"/>
+      <c r="E27" s="83"/>
+      <c r="F27" s="83"/>
+      <c r="G27" s="83"/>
+      <c r="H27" s="83"/>
+      <c r="I27" s="83"/>
+      <c r="J27" s="83"/>
+      <c r="K27" s="83"/>
+      <c r="L27" s="83"/>
+      <c r="M27" s="83"/>
+      <c r="N27" s="83"/>
+      <c r="O27" s="83"/>
+      <c r="P27" s="83"/>
+      <c r="Q27" s="83"/>
+      <c r="R27" s="83"/>
+      <c r="S27" s="83"/>
+      <c r="T27" s="83"/>
+      <c r="U27" s="83"/>
+      <c r="V27" s="83"/>
+      <c r="W27" s="83"/>
+      <c r="X27" s="83"/>
+      <c r="Y27" s="83"/>
+      <c r="Z27" s="83"/>
+      <c r="AA27" s="83"/>
+      <c r="AB27" s="83"/>
+      <c r="AC27" s="83"/>
+      <c r="AD27" s="83"/>
+      <c r="AE27" s="83"/>
+    </row>
+    <row r="28" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A28" s="83"/>
+      <c r="B28" s="83"/>
+      <c r="C28" s="83"/>
+      <c r="D28" s="83"/>
+      <c r="E28" s="83"/>
+      <c r="F28" s="83"/>
+      <c r="G28" s="83"/>
+      <c r="H28" s="83"/>
+      <c r="I28" s="83"/>
+      <c r="J28" s="83"/>
+      <c r="K28" s="83"/>
+      <c r="L28" s="83"/>
+      <c r="M28" s="83"/>
+      <c r="N28" s="83"/>
+      <c r="O28" s="83"/>
+      <c r="P28" s="83"/>
+      <c r="Q28" s="83"/>
+      <c r="R28" s="83"/>
+      <c r="S28" s="83"/>
+      <c r="T28" s="83"/>
+      <c r="U28" s="83"/>
+      <c r="V28" s="83"/>
+      <c r="W28" s="83"/>
+      <c r="X28" s="83"/>
+      <c r="Y28" s="83"/>
+      <c r="Z28" s="83"/>
+      <c r="AA28" s="83"/>
+      <c r="AB28" s="83"/>
+      <c r="AC28" s="83"/>
+      <c r="AD28" s="83"/>
+      <c r="AE28" s="83"/>
+    </row>
+    <row r="29" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A29" s="83"/>
+      <c r="B29" s="83"/>
+      <c r="C29" s="83"/>
+      <c r="D29" s="83"/>
+      <c r="E29" s="83"/>
+      <c r="F29" s="83"/>
+      <c r="G29" s="83"/>
+      <c r="H29" s="83"/>
+      <c r="I29" s="83"/>
+      <c r="J29" s="83"/>
+      <c r="K29" s="83"/>
+      <c r="L29" s="83"/>
+      <c r="M29" s="83"/>
+      <c r="N29" s="83"/>
+      <c r="O29" s="83"/>
+      <c r="P29" s="83"/>
+      <c r="Q29" s="83"/>
+      <c r="R29" s="83"/>
+      <c r="S29" s="83"/>
+      <c r="T29" s="83"/>
+      <c r="U29" s="83"/>
+      <c r="V29" s="83"/>
+      <c r="W29" s="83"/>
+      <c r="X29" s="83"/>
+      <c r="Y29" s="83"/>
+      <c r="Z29" s="83"/>
+      <c r="AA29" s="83"/>
+      <c r="AB29" s="83"/>
+      <c r="AC29" s="83"/>
+      <c r="AD29" s="83"/>
+      <c r="AE29" s="83"/>
+    </row>
+    <row r="30" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A30" s="83"/>
+      <c r="B30" s="83"/>
+      <c r="C30" s="83"/>
+      <c r="D30" s="83"/>
+      <c r="E30" s="83"/>
+      <c r="F30" s="83"/>
+      <c r="G30" s="83"/>
+      <c r="H30" s="83"/>
+      <c r="I30" s="83"/>
+      <c r="J30" s="83"/>
+      <c r="K30" s="83"/>
+      <c r="L30" s="83"/>
+      <c r="M30" s="83"/>
+      <c r="N30" s="83"/>
+      <c r="O30" s="83"/>
+      <c r="P30" s="83"/>
+      <c r="Q30" s="83"/>
+      <c r="R30" s="83"/>
+      <c r="S30" s="83"/>
+      <c r="T30" s="83"/>
+      <c r="U30" s="83"/>
+      <c r="V30" s="83"/>
+      <c r="W30" s="83"/>
+      <c r="X30" s="83"/>
+      <c r="Y30" s="83"/>
+      <c r="Z30" s="83"/>
+      <c r="AA30" s="83"/>
+      <c r="AB30" s="83"/>
+      <c r="AC30" s="83"/>
+      <c r="AD30" s="83"/>
+      <c r="AE30" s="83"/>
+    </row>
+    <row r="31" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A31" s="83"/>
+      <c r="B31" s="83"/>
+      <c r="C31" s="83"/>
+      <c r="D31" s="83"/>
+      <c r="E31" s="83"/>
+      <c r="F31" s="83"/>
+      <c r="G31" s="83"/>
+      <c r="H31" s="83"/>
+      <c r="I31" s="83"/>
+      <c r="J31" s="83"/>
+      <c r="K31" s="83"/>
+      <c r="L31" s="83"/>
+      <c r="M31" s="83"/>
+      <c r="N31" s="83"/>
+      <c r="O31" s="83"/>
+      <c r="P31" s="83"/>
+      <c r="Q31" s="83"/>
+      <c r="R31" s="83"/>
+      <c r="S31" s="83"/>
+      <c r="T31" s="83"/>
+      <c r="U31" s="83"/>
+      <c r="V31" s="83"/>
+      <c r="W31" s="83"/>
+      <c r="X31" s="83"/>
+      <c r="Y31" s="83"/>
+      <c r="Z31" s="83"/>
+      <c r="AA31" s="83"/>
+      <c r="AB31" s="83"/>
+      <c r="AC31" s="83"/>
+      <c r="AD31" s="83"/>
+      <c r="AE31" s="83"/>
+    </row>
+    <row r="32" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A32" s="83"/>
+      <c r="B32" s="83"/>
+      <c r="C32" s="83"/>
+      <c r="D32" s="83"/>
+      <c r="E32" s="83"/>
+      <c r="F32" s="83"/>
+      <c r="G32" s="83"/>
+      <c r="H32" s="83"/>
+      <c r="I32" s="83"/>
+      <c r="J32" s="83"/>
+      <c r="K32" s="83"/>
+      <c r="L32" s="83"/>
+      <c r="M32" s="83"/>
+      <c r="N32" s="83"/>
+      <c r="O32" s="83"/>
+      <c r="P32" s="83"/>
+      <c r="Q32" s="83"/>
+      <c r="R32" s="83"/>
+      <c r="S32" s="83"/>
+      <c r="T32" s="83"/>
+      <c r="U32" s="83"/>
+      <c r="V32" s="83"/>
+      <c r="W32" s="83"/>
+      <c r="X32" s="83"/>
+      <c r="Y32" s="83"/>
+      <c r="Z32" s="83"/>
+      <c r="AA32" s="83"/>
+      <c r="AB32" s="83"/>
+      <c r="AC32" s="83"/>
+      <c r="AD32" s="83"/>
+      <c r="AE32" s="83"/>
+    </row>
+    <row r="33" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A33" s="83"/>
+      <c r="B33" s="83"/>
+      <c r="C33" s="83"/>
+      <c r="D33" s="83"/>
+      <c r="E33" s="83"/>
+      <c r="F33" s="83"/>
+      <c r="G33" s="83"/>
+      <c r="H33" s="83"/>
+      <c r="I33" s="83"/>
+      <c r="J33" s="83"/>
+      <c r="K33" s="83"/>
+      <c r="L33" s="83"/>
+      <c r="M33" s="83"/>
+      <c r="N33" s="83"/>
+      <c r="O33" s="83"/>
+      <c r="P33" s="83"/>
+      <c r="Q33" s="83"/>
+      <c r="R33" s="83"/>
+      <c r="S33" s="83"/>
+      <c r="T33" s="83"/>
+      <c r="U33" s="83"/>
+      <c r="V33" s="83"/>
+      <c r="W33" s="83"/>
+      <c r="X33" s="83"/>
+      <c r="Y33" s="83"/>
+      <c r="Z33" s="83"/>
+      <c r="AA33" s="83"/>
+      <c r="AB33" s="83"/>
+      <c r="AC33" s="83"/>
+      <c r="AD33" s="83"/>
+      <c r="AE33" s="83"/>
+    </row>
+    <row r="34" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A34" s="83"/>
+      <c r="B34" s="83"/>
+      <c r="C34" s="83"/>
+      <c r="D34" s="83"/>
+      <c r="E34" s="83"/>
+      <c r="F34" s="83"/>
+      <c r="G34" s="83"/>
+      <c r="H34" s="83"/>
+      <c r="I34" s="83"/>
+      <c r="J34" s="83"/>
+      <c r="K34" s="83"/>
+      <c r="L34" s="83"/>
+      <c r="M34" s="83"/>
+      <c r="N34" s="83"/>
+      <c r="O34" s="83"/>
+      <c r="P34" s="83"/>
+      <c r="Q34" s="83"/>
+      <c r="R34" s="83"/>
+      <c r="S34" s="83"/>
+      <c r="T34" s="83"/>
+      <c r="U34" s="83"/>
+      <c r="V34" s="83"/>
+      <c r="W34" s="83"/>
+      <c r="X34" s="83"/>
+      <c r="Y34" s="83"/>
+      <c r="Z34" s="83"/>
+      <c r="AA34" s="83"/>
+      <c r="AB34" s="83"/>
+      <c r="AC34" s="83"/>
+      <c r="AD34" s="83"/>
+      <c r="AE34" s="83"/>
+    </row>
+    <row r="35" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A35" s="83"/>
+      <c r="B35" s="83"/>
+      <c r="C35" s="83"/>
+      <c r="D35" s="83"/>
+      <c r="E35" s="83"/>
+      <c r="F35" s="83"/>
+      <c r="G35" s="83"/>
+      <c r="H35" s="83"/>
+      <c r="I35" s="83"/>
+      <c r="J35" s="83"/>
+      <c r="K35" s="83"/>
+      <c r="L35" s="83"/>
+      <c r="M35" s="83"/>
+      <c r="N35" s="83"/>
+      <c r="O35" s="83"/>
+      <c r="P35" s="83"/>
+      <c r="Q35" s="83"/>
+      <c r="R35" s="83"/>
+      <c r="S35" s="83"/>
+      <c r="T35" s="83"/>
+      <c r="U35" s="83"/>
+      <c r="V35" s="83"/>
+      <c r="W35" s="83"/>
+      <c r="X35" s="83"/>
+      <c r="Y35" s="83"/>
+      <c r="Z35" s="83"/>
+      <c r="AA35" s="83"/>
+      <c r="AB35" s="83"/>
+      <c r="AC35" s="83"/>
+      <c r="AD35" s="83"/>
+      <c r="AE35" s="83"/>
+    </row>
+    <row r="36" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A36" s="83"/>
+      <c r="B36" s="83"/>
+      <c r="C36" s="83"/>
+      <c r="D36" s="83"/>
+      <c r="E36" s="83"/>
+      <c r="F36" s="83"/>
+      <c r="G36" s="83"/>
+      <c r="H36" s="83"/>
+      <c r="I36" s="83"/>
+      <c r="J36" s="83"/>
+      <c r="K36" s="83"/>
+      <c r="L36" s="83"/>
+      <c r="M36" s="83"/>
+      <c r="N36" s="83"/>
+      <c r="O36" s="83"/>
+      <c r="P36" s="83"/>
+      <c r="Q36" s="83"/>
+      <c r="R36" s="83"/>
+      <c r="S36" s="83"/>
+      <c r="T36" s="83"/>
+      <c r="U36" s="83"/>
+      <c r="V36" s="83"/>
+      <c r="W36" s="83"/>
+      <c r="X36" s="83"/>
+      <c r="Y36" s="83"/>
+      <c r="Z36" s="83"/>
+      <c r="AA36" s="83"/>
+      <c r="AB36" s="83"/>
+      <c r="AC36" s="83"/>
+      <c r="AD36" s="83"/>
+      <c r="AE36" s="83"/>
+    </row>
+    <row r="37" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A37" s="83"/>
+      <c r="B37" s="83"/>
+      <c r="C37" s="83"/>
+      <c r="D37" s="83"/>
+      <c r="E37" s="83"/>
+      <c r="F37" s="83"/>
+      <c r="G37" s="83"/>
+      <c r="H37" s="83"/>
+      <c r="I37" s="83"/>
+      <c r="J37" s="83"/>
+      <c r="K37" s="83"/>
+      <c r="L37" s="83"/>
+      <c r="M37" s="83"/>
+      <c r="N37" s="83"/>
+      <c r="O37" s="83"/>
+      <c r="P37" s="83"/>
+      <c r="Q37" s="83"/>
+      <c r="R37" s="83"/>
+      <c r="S37" s="83"/>
+      <c r="T37" s="83"/>
+      <c r="U37" s="83"/>
+      <c r="V37" s="83"/>
+      <c r="W37" s="83"/>
+      <c r="X37" s="83"/>
+      <c r="Y37" s="83"/>
+      <c r="Z37" s="83"/>
+      <c r="AA37" s="83"/>
+      <c r="AB37" s="83"/>
+      <c r="AC37" s="83"/>
+      <c r="AD37" s="83"/>
+      <c r="AE37" s="83"/>
+    </row>
+    <row r="38" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A38" s="83"/>
+      <c r="B38" s="83"/>
+      <c r="C38" s="83"/>
+      <c r="D38" s="83"/>
+      <c r="E38" s="83"/>
+      <c r="F38" s="83"/>
+      <c r="G38" s="83"/>
+      <c r="H38" s="83"/>
+      <c r="I38" s="83"/>
+      <c r="J38" s="83"/>
+      <c r="K38" s="83"/>
+      <c r="L38" s="83"/>
+      <c r="M38" s="83"/>
+      <c r="N38" s="83"/>
+      <c r="O38" s="83"/>
+      <c r="P38" s="83"/>
+      <c r="Q38" s="83"/>
+      <c r="R38" s="83"/>
+      <c r="S38" s="83"/>
+      <c r="T38" s="83"/>
+      <c r="U38" s="83"/>
+      <c r="V38" s="83"/>
+      <c r="W38" s="83"/>
+      <c r="X38" s="83"/>
+      <c r="Y38" s="83"/>
+      <c r="Z38" s="83"/>
+      <c r="AA38" s="83"/>
+      <c r="AB38" s="83"/>
+      <c r="AC38" s="83"/>
+      <c r="AD38" s="83"/>
+      <c r="AE38" s="83"/>
+    </row>
+    <row r="39" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A39" s="83"/>
+      <c r="B39" s="83"/>
+      <c r="C39" s="83"/>
+      <c r="D39" s="83"/>
+      <c r="E39" s="83"/>
+      <c r="F39" s="83"/>
+      <c r="G39" s="83"/>
+      <c r="H39" s="83"/>
+      <c r="I39" s="83"/>
+      <c r="J39" s="83"/>
+      <c r="K39" s="83"/>
+      <c r="L39" s="83"/>
+      <c r="M39" s="83"/>
+      <c r="N39" s="83"/>
+      <c r="O39" s="83"/>
+      <c r="P39" s="83"/>
+      <c r="Q39" s="83"/>
+      <c r="R39" s="83"/>
+      <c r="S39" s="83"/>
+      <c r="T39" s="83"/>
+      <c r="U39" s="83"/>
+      <c r="V39" s="83"/>
+      <c r="W39" s="83"/>
+      <c r="X39" s="83"/>
+      <c r="Y39" s="83"/>
+      <c r="Z39" s="83"/>
+      <c r="AA39" s="83"/>
+      <c r="AB39" s="83"/>
+      <c r="AC39" s="83"/>
+      <c r="AD39" s="83"/>
+      <c r="AE39" s="83"/>
+    </row>
+    <row r="40" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A40" s="83"/>
+      <c r="B40" s="83"/>
+      <c r="C40" s="83"/>
+      <c r="D40" s="83"/>
+      <c r="E40" s="83"/>
+      <c r="F40" s="83"/>
+      <c r="G40" s="83"/>
+      <c r="H40" s="83"/>
+      <c r="I40" s="83"/>
+      <c r="J40" s="83"/>
+      <c r="K40" s="83"/>
+      <c r="L40" s="83"/>
+      <c r="M40" s="83"/>
+      <c r="N40" s="83"/>
+      <c r="O40" s="83"/>
+      <c r="P40" s="83"/>
+      <c r="Q40" s="83"/>
+      <c r="R40" s="83"/>
+      <c r="S40" s="83"/>
+      <c r="T40" s="83"/>
+      <c r="U40" s="83"/>
+      <c r="V40" s="83"/>
+      <c r="W40" s="83"/>
+      <c r="X40" s="83"/>
+      <c r="Y40" s="83"/>
+      <c r="Z40" s="83"/>
+      <c r="AA40" s="83"/>
+      <c r="AB40" s="83"/>
+      <c r="AC40" s="83"/>
+      <c r="AD40" s="83"/>
+      <c r="AE40" s="83"/>
+    </row>
+    <row r="41" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A41" s="83"/>
+      <c r="B41" s="83"/>
+      <c r="C41" s="83"/>
+      <c r="D41" s="83"/>
+      <c r="E41" s="83"/>
+      <c r="F41" s="83"/>
+      <c r="G41" s="83"/>
+      <c r="H41" s="83"/>
+      <c r="I41" s="83"/>
+      <c r="J41" s="83"/>
+      <c r="K41" s="83"/>
+      <c r="L41" s="83"/>
+      <c r="M41" s="83"/>
+      <c r="N41" s="83"/>
+      <c r="O41" s="83"/>
+      <c r="P41" s="83"/>
+      <c r="Q41" s="83"/>
+      <c r="R41" s="83"/>
+      <c r="S41" s="83"/>
+      <c r="T41" s="83"/>
+      <c r="U41" s="83"/>
+      <c r="V41" s="83"/>
+      <c r="W41" s="83"/>
+      <c r="X41" s="83"/>
+      <c r="Y41" s="83"/>
+      <c r="Z41" s="83"/>
+      <c r="AA41" s="83"/>
+      <c r="AB41" s="83"/>
+      <c r="AC41" s="83"/>
+      <c r="AD41" s="83"/>
+      <c r="AE41" s="83"/>
+    </row>
+    <row r="42" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A42" s="83"/>
+      <c r="B42" s="83"/>
+      <c r="C42" s="83"/>
+      <c r="D42" s="83"/>
+      <c r="E42" s="83"/>
+      <c r="F42" s="83"/>
+      <c r="G42" s="83"/>
+      <c r="H42" s="83"/>
+      <c r="I42" s="83"/>
+      <c r="J42" s="83"/>
+      <c r="K42" s="83"/>
+      <c r="L42" s="83"/>
+      <c r="M42" s="83"/>
+      <c r="N42" s="83"/>
+      <c r="O42" s="83"/>
+      <c r="P42" s="83"/>
+      <c r="Q42" s="83"/>
+      <c r="R42" s="83"/>
+      <c r="S42" s="83"/>
+      <c r="T42" s="83"/>
+      <c r="U42" s="83"/>
+      <c r="V42" s="83"/>
+      <c r="W42" s="83"/>
+      <c r="X42" s="83"/>
+      <c r="Y42" s="83"/>
+      <c r="Z42" s="83"/>
+      <c r="AA42" s="83"/>
+      <c r="AB42" s="83"/>
+      <c r="AC42" s="83"/>
+      <c r="AD42" s="83"/>
+      <c r="AE42" s="83"/>
+    </row>
+    <row r="43" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A43" s="83"/>
+      <c r="B43" s="83"/>
+      <c r="C43" s="83"/>
+      <c r="D43" s="83"/>
+      <c r="E43" s="83"/>
+      <c r="F43" s="83"/>
+      <c r="G43" s="83"/>
+      <c r="H43" s="83"/>
+      <c r="I43" s="83"/>
+      <c r="J43" s="83"/>
+      <c r="K43" s="83"/>
+      <c r="L43" s="83"/>
+      <c r="M43" s="83"/>
+      <c r="N43" s="83"/>
+      <c r="O43" s="83"/>
+      <c r="P43" s="83"/>
+      <c r="Q43" s="83"/>
+      <c r="R43" s="83"/>
+      <c r="S43" s="83"/>
+      <c r="T43" s="83"/>
+      <c r="U43" s="83"/>
+      <c r="V43" s="83"/>
+      <c r="W43" s="83"/>
+      <c r="X43" s="83"/>
+      <c r="Y43" s="83"/>
+      <c r="Z43" s="83"/>
+      <c r="AA43" s="83"/>
+      <c r="AB43" s="83"/>
+      <c r="AC43" s="83"/>
+      <c r="AD43" s="83"/>
+      <c r="AE43" s="83"/>
+    </row>
+    <row r="44" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A44" s="83"/>
+      <c r="B44" s="83"/>
+      <c r="C44" s="83"/>
+      <c r="D44" s="83"/>
+      <c r="E44" s="83"/>
+      <c r="F44" s="83"/>
+      <c r="G44" s="83"/>
+      <c r="H44" s="83"/>
+      <c r="I44" s="83"/>
+      <c r="J44" s="83"/>
+      <c r="K44" s="83"/>
+      <c r="L44" s="83"/>
+      <c r="M44" s="83"/>
+      <c r="N44" s="83"/>
+      <c r="O44" s="83"/>
+      <c r="P44" s="83"/>
+      <c r="Q44" s="83"/>
+      <c r="R44" s="83"/>
+      <c r="S44" s="83"/>
+      <c r="T44" s="83"/>
+      <c r="U44" s="83"/>
+      <c r="V44" s="83"/>
+      <c r="W44" s="83"/>
+      <c r="X44" s="83"/>
+      <c r="Y44" s="83"/>
+      <c r="Z44" s="83"/>
+      <c r="AA44" s="83"/>
+      <c r="AB44" s="83"/>
+      <c r="AC44" s="83"/>
+      <c r="AD44" s="83"/>
+      <c r="AE44" s="83"/>
+    </row>
+    <row r="45" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A45" s="83"/>
+      <c r="B45" s="83"/>
+      <c r="C45" s="83"/>
+      <c r="D45" s="83"/>
+      <c r="E45" s="83"/>
+      <c r="F45" s="83"/>
+      <c r="G45" s="83"/>
+      <c r="H45" s="83"/>
+      <c r="I45" s="83"/>
+      <c r="J45" s="83"/>
+      <c r="K45" s="83"/>
+      <c r="L45" s="83"/>
+      <c r="M45" s="83"/>
+      <c r="N45" s="83"/>
+      <c r="O45" s="83"/>
+      <c r="P45" s="83"/>
+      <c r="Q45" s="83"/>
+      <c r="R45" s="83"/>
+      <c r="S45" s="83"/>
+      <c r="T45" s="83"/>
+      <c r="U45" s="83"/>
+      <c r="V45" s="83"/>
+      <c r="W45" s="83"/>
+      <c r="X45" s="83"/>
+      <c r="Y45" s="83"/>
+      <c r="Z45" s="83"/>
+      <c r="AA45" s="83"/>
+      <c r="AB45" s="83"/>
+      <c r="AC45" s="83"/>
+      <c r="AD45" s="83"/>
+      <c r="AE45" s="83"/>
+    </row>
+    <row r="46" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A46" s="83"/>
+      <c r="B46" s="83"/>
+      <c r="C46" s="83"/>
+      <c r="D46" s="83"/>
+      <c r="E46" s="83"/>
+      <c r="F46" s="83"/>
+      <c r="G46" s="83"/>
+      <c r="H46" s="83"/>
+      <c r="I46" s="83"/>
+      <c r="J46" s="83"/>
+      <c r="K46" s="83"/>
+      <c r="L46" s="83"/>
+      <c r="M46" s="83"/>
+      <c r="N46" s="83"/>
+      <c r="O46" s="83"/>
+      <c r="P46" s="83"/>
+      <c r="Q46" s="83"/>
+      <c r="R46" s="83"/>
+      <c r="S46" s="83"/>
+      <c r="T46" s="83"/>
+      <c r="U46" s="83"/>
+      <c r="V46" s="83"/>
+      <c r="W46" s="83"/>
+      <c r="X46" s="83"/>
+      <c r="Y46" s="83"/>
+      <c r="Z46" s="83"/>
+      <c r="AA46" s="83"/>
+      <c r="AB46" s="83"/>
+      <c r="AC46" s="83"/>
+      <c r="AD46" s="83"/>
+      <c r="AE46" s="83"/>
+    </row>
+    <row r="47" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A47" s="83"/>
+      <c r="B47" s="83"/>
+      <c r="C47" s="83"/>
+      <c r="D47" s="83"/>
+      <c r="E47" s="83"/>
+      <c r="F47" s="83"/>
+      <c r="G47" s="83"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="83"/>
+      <c r="J47" s="83"/>
+      <c r="K47" s="83"/>
+      <c r="L47" s="83"/>
+      <c r="M47" s="83"/>
+      <c r="N47" s="83"/>
+      <c r="O47" s="83"/>
+      <c r="P47" s="83"/>
+      <c r="Q47" s="83"/>
+      <c r="R47" s="83"/>
+      <c r="S47" s="83"/>
+      <c r="T47" s="83"/>
+      <c r="U47" s="83"/>
+      <c r="V47" s="83"/>
+      <c r="W47" s="83"/>
+      <c r="X47" s="83"/>
+      <c r="Y47" s="83"/>
+      <c r="Z47" s="83"/>
+      <c r="AA47" s="83"/>
+      <c r="AB47" s="83"/>
+      <c r="AC47" s="83"/>
+      <c r="AD47" s="83"/>
+      <c r="AE47" s="83"/>
+    </row>
+    <row r="48" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A48" s="83"/>
+      <c r="B48" s="83"/>
+      <c r="C48" s="83"/>
+      <c r="D48" s="83"/>
+      <c r="E48" s="83"/>
+      <c r="F48" s="83"/>
+      <c r="G48" s="83"/>
+      <c r="H48" s="83"/>
+      <c r="I48" s="83"/>
+      <c r="J48" s="83"/>
+      <c r="K48" s="83"/>
+      <c r="L48" s="83"/>
+      <c r="M48" s="83"/>
+      <c r="N48" s="83"/>
+      <c r="O48" s="83"/>
+      <c r="P48" s="83"/>
+      <c r="Q48" s="83"/>
+      <c r="R48" s="83"/>
+      <c r="S48" s="83"/>
+      <c r="T48" s="83"/>
+      <c r="U48" s="83"/>
+      <c r="V48" s="83"/>
+      <c r="W48" s="83"/>
+      <c r="X48" s="83"/>
+      <c r="Y48" s="83"/>
+      <c r="Z48" s="83"/>
+      <c r="AA48" s="83"/>
+      <c r="AB48" s="83"/>
+      <c r="AC48" s="83"/>
+      <c r="AD48" s="83"/>
+      <c r="AE48" s="83"/>
+    </row>
+    <row r="49" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A49" s="83"/>
+      <c r="B49" s="83"/>
+      <c r="C49" s="83"/>
+      <c r="D49" s="83"/>
+      <c r="E49" s="83"/>
+      <c r="F49" s="83"/>
+      <c r="G49" s="83"/>
+      <c r="H49" s="83"/>
+      <c r="I49" s="83"/>
+      <c r="J49" s="83"/>
+      <c r="K49" s="83"/>
+      <c r="L49" s="83"/>
+      <c r="M49" s="83"/>
+      <c r="N49" s="83"/>
+      <c r="O49" s="83"/>
+      <c r="P49" s="83"/>
+      <c r="Q49" s="83"/>
+      <c r="R49" s="83"/>
+      <c r="S49" s="83"/>
+      <c r="T49" s="83"/>
+      <c r="U49" s="83"/>
+      <c r="V49" s="83"/>
+      <c r="W49" s="83"/>
+      <c r="X49" s="83"/>
+      <c r="Y49" s="83"/>
+      <c r="Z49" s="83"/>
+      <c r="AA49" s="83"/>
+      <c r="AB49" s="83"/>
+      <c r="AC49" s="83"/>
+      <c r="AD49" s="83"/>
+      <c r="AE49" s="83"/>
+    </row>
+    <row r="50" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A50" s="83"/>
+      <c r="B50" s="83"/>
+      <c r="C50" s="83"/>
+      <c r="D50" s="83"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="83"/>
+      <c r="J50" s="83"/>
+      <c r="K50" s="83"/>
+      <c r="L50" s="83"/>
+      <c r="M50" s="83"/>
+      <c r="N50" s="83"/>
+      <c r="O50" s="83"/>
+      <c r="P50" s="83"/>
+      <c r="Q50" s="83"/>
+      <c r="R50" s="83"/>
+      <c r="S50" s="83"/>
+      <c r="T50" s="83"/>
+      <c r="U50" s="83"/>
+      <c r="V50" s="83"/>
+      <c r="W50" s="83"/>
+      <c r="X50" s="83"/>
+      <c r="Y50" s="83"/>
+      <c r="Z50" s="83"/>
+      <c r="AA50" s="83"/>
+      <c r="AB50" s="83"/>
+      <c r="AC50" s="83"/>
+      <c r="AD50" s="83"/>
+      <c r="AE50" s="83"/>
+    </row>
+    <row r="51" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A51" s="83"/>
+      <c r="B51" s="83"/>
+      <c r="C51" s="83"/>
+      <c r="D51" s="83"/>
+      <c r="E51" s="83"/>
+      <c r="F51" s="83"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="83"/>
+      <c r="J51" s="83"/>
+      <c r="K51" s="83"/>
+      <c r="L51" s="83"/>
+      <c r="M51" s="83"/>
+      <c r="N51" s="83"/>
+      <c r="O51" s="83"/>
+      <c r="P51" s="83"/>
+      <c r="Q51" s="83"/>
+      <c r="R51" s="83"/>
+      <c r="S51" s="83"/>
+      <c r="T51" s="83"/>
+      <c r="U51" s="83"/>
+      <c r="V51" s="83"/>
+      <c r="W51" s="83"/>
+      <c r="X51" s="83"/>
+      <c r="Y51" s="83"/>
+      <c r="Z51" s="83"/>
+      <c r="AA51" s="83"/>
+      <c r="AB51" s="83"/>
+      <c r="AC51" s="83"/>
+      <c r="AD51" s="83"/>
+      <c r="AE51" s="83"/>
+    </row>
+    <row r="52" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A52" s="83"/>
+      <c r="B52" s="83"/>
+      <c r="C52" s="83"/>
+      <c r="D52" s="83"/>
+      <c r="E52" s="83"/>
+      <c r="F52" s="83"/>
+      <c r="G52" s="83"/>
+      <c r="H52" s="83"/>
+      <c r="I52" s="83"/>
+      <c r="J52" s="83"/>
+      <c r="K52" s="83"/>
+      <c r="L52" s="83"/>
+      <c r="M52" s="83"/>
+      <c r="N52" s="83"/>
+      <c r="O52" s="83"/>
+      <c r="P52" s="83"/>
+      <c r="Q52" s="83"/>
+      <c r="R52" s="83"/>
+      <c r="S52" s="83"/>
+      <c r="T52" s="83"/>
+      <c r="U52" s="83"/>
+      <c r="V52" s="83"/>
+      <c r="W52" s="83"/>
+      <c r="X52" s="83"/>
+      <c r="Y52" s="83"/>
+      <c r="Z52" s="83"/>
+      <c r="AA52" s="83"/>
+      <c r="AB52" s="83"/>
+      <c r="AC52" s="83"/>
+      <c r="AD52" s="83"/>
+      <c r="AE52" s="83"/>
+    </row>
+    <row r="53" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A53" s="83"/>
+      <c r="B53" s="83"/>
+      <c r="C53" s="83"/>
+      <c r="D53" s="83"/>
+      <c r="E53" s="83"/>
+      <c r="F53" s="83"/>
+      <c r="G53" s="83"/>
+      <c r="H53" s="83"/>
+      <c r="I53" s="83"/>
+      <c r="J53" s="83"/>
+      <c r="K53" s="83"/>
+      <c r="L53" s="83"/>
+      <c r="M53" s="83"/>
+      <c r="N53" s="83"/>
+      <c r="O53" s="83"/>
+      <c r="P53" s="83"/>
+      <c r="Q53" s="83"/>
+      <c r="R53" s="83"/>
+      <c r="S53" s="83"/>
+      <c r="T53" s="83"/>
+      <c r="U53" s="83"/>
+      <c r="V53" s="83"/>
+      <c r="W53" s="83"/>
+      <c r="X53" s="83"/>
+      <c r="Y53" s="83"/>
+      <c r="Z53" s="83"/>
+      <c r="AA53" s="83"/>
+      <c r="AB53" s="83"/>
+      <c r="AC53" s="83"/>
+      <c r="AD53" s="83"/>
+      <c r="AE53" s="83"/>
+    </row>
+    <row r="54" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A54" s="83"/>
+      <c r="B54" s="83"/>
+      <c r="C54" s="83"/>
+      <c r="D54" s="83"/>
+      <c r="E54" s="83"/>
+      <c r="F54" s="83"/>
+      <c r="G54" s="83"/>
+      <c r="H54" s="83"/>
+      <c r="I54" s="83"/>
+      <c r="J54" s="83"/>
+      <c r="K54" s="83"/>
+      <c r="L54" s="83"/>
+      <c r="M54" s="83"/>
+      <c r="N54" s="83"/>
+      <c r="O54" s="83"/>
+      <c r="P54" s="83"/>
+      <c r="Q54" s="83"/>
+      <c r="R54" s="83"/>
+      <c r="S54" s="83"/>
+      <c r="T54" s="83"/>
+      <c r="U54" s="83"/>
+      <c r="V54" s="83"/>
+      <c r="W54" s="83"/>
+      <c r="X54" s="83"/>
+      <c r="Y54" s="83"/>
+      <c r="Z54" s="83"/>
+      <c r="AA54" s="83"/>
+      <c r="AB54" s="83"/>
+      <c r="AC54" s="83"/>
+      <c r="AD54" s="83"/>
+      <c r="AE54" s="83"/>
+    </row>
+    <row r="55" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A55" s="83"/>
+      <c r="B55" s="83"/>
+      <c r="C55" s="83"/>
+      <c r="D55" s="83"/>
+      <c r="E55" s="83"/>
+      <c r="F55" s="83"/>
+      <c r="G55" s="83"/>
+      <c r="H55" s="83"/>
+      <c r="I55" s="83"/>
+      <c r="J55" s="83"/>
+      <c r="K55" s="83"/>
+      <c r="L55" s="83"/>
+      <c r="M55" s="83"/>
+      <c r="N55" s="83"/>
+      <c r="O55" s="83"/>
+      <c r="P55" s="83"/>
+      <c r="Q55" s="83"/>
+      <c r="R55" s="83"/>
+      <c r="S55" s="83"/>
+      <c r="T55" s="83"/>
+      <c r="U55" s="83"/>
+      <c r="V55" s="83"/>
+      <c r="W55" s="83"/>
+      <c r="X55" s="83"/>
+      <c r="Y55" s="83"/>
+      <c r="Z55" s="83"/>
+      <c r="AA55" s="83"/>
+      <c r="AB55" s="83"/>
+      <c r="AC55" s="83"/>
+      <c r="AD55" s="83"/>
+      <c r="AE55" s="83"/>
+    </row>
+    <row r="56" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A56" s="83"/>
+      <c r="B56" s="83"/>
+      <c r="C56" s="83"/>
+      <c r="D56" s="83"/>
+      <c r="E56" s="83"/>
+      <c r="F56" s="83"/>
+      <c r="G56" s="83"/>
+      <c r="H56" s="83"/>
+      <c r="I56" s="83"/>
+      <c r="J56" s="83"/>
+      <c r="K56" s="83"/>
+      <c r="L56" s="83"/>
+      <c r="M56" s="83"/>
+      <c r="N56" s="83"/>
+      <c r="O56" s="83"/>
+      <c r="P56" s="83"/>
+      <c r="Q56" s="83"/>
+      <c r="R56" s="83"/>
+      <c r="S56" s="83"/>
+      <c r="T56" s="83"/>
+      <c r="U56" s="83"/>
+      <c r="V56" s="83"/>
+      <c r="W56" s="83"/>
+      <c r="X56" s="83"/>
+      <c r="Y56" s="83"/>
+      <c r="Z56" s="83"/>
+      <c r="AA56" s="83"/>
+      <c r="AB56" s="83"/>
+      <c r="AC56" s="83"/>
+      <c r="AD56" s="83"/>
+      <c r="AE56" s="83"/>
+    </row>
+    <row r="57" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A57" s="83"/>
+      <c r="B57" s="83"/>
+      <c r="C57" s="83"/>
+      <c r="D57" s="83"/>
+      <c r="E57" s="83"/>
+      <c r="F57" s="83"/>
+      <c r="G57" s="83"/>
+      <c r="H57" s="83"/>
+      <c r="I57" s="83"/>
+      <c r="J57" s="83"/>
+      <c r="K57" s="83"/>
+      <c r="L57" s="83"/>
+      <c r="M57" s="83"/>
+      <c r="N57" s="83"/>
+      <c r="O57" s="83"/>
+      <c r="P57" s="83"/>
+      <c r="Q57" s="83"/>
+      <c r="R57" s="83"/>
+      <c r="S57" s="83"/>
+      <c r="T57" s="83"/>
+      <c r="U57" s="83"/>
+      <c r="V57" s="83"/>
+      <c r="W57" s="83"/>
+      <c r="X57" s="83"/>
+      <c r="Y57" s="83"/>
+      <c r="Z57" s="83"/>
+      <c r="AA57" s="83"/>
+      <c r="AB57" s="83"/>
+      <c r="AC57" s="83"/>
+      <c r="AD57" s="83"/>
+      <c r="AE57" s="83"/>
+    </row>
+    <row r="58" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A58" s="83"/>
+      <c r="B58" s="83"/>
+      <c r="C58" s="83"/>
+      <c r="D58" s="83"/>
+      <c r="E58" s="83"/>
+      <c r="F58" s="83"/>
+      <c r="G58" s="83"/>
+      <c r="H58" s="83"/>
+      <c r="I58" s="83"/>
+      <c r="J58" s="83"/>
+      <c r="K58" s="83"/>
+      <c r="L58" s="83"/>
+      <c r="M58" s="83"/>
+      <c r="N58" s="83"/>
+      <c r="O58" s="83"/>
+      <c r="P58" s="83"/>
+      <c r="Q58" s="83"/>
+      <c r="R58" s="83"/>
+      <c r="S58" s="83"/>
+      <c r="T58" s="83"/>
+      <c r="U58" s="83"/>
+      <c r="V58" s="83"/>
+      <c r="W58" s="83"/>
+      <c r="X58" s="83"/>
+      <c r="Y58" s="83"/>
+      <c r="Z58" s="83"/>
+      <c r="AA58" s="83"/>
+      <c r="AB58" s="83"/>
+      <c r="AC58" s="83"/>
+      <c r="AD58" s="83"/>
+      <c r="AE58" s="83"/>
+    </row>
+    <row r="59" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A59" s="83"/>
+      <c r="B59" s="83"/>
+      <c r="C59" s="83"/>
+      <c r="D59" s="83"/>
+      <c r="E59" s="83"/>
+      <c r="F59" s="83"/>
+      <c r="G59" s="83"/>
+      <c r="H59" s="83"/>
+      <c r="I59" s="83"/>
+      <c r="J59" s="83"/>
+      <c r="K59" s="83"/>
+      <c r="L59" s="83"/>
+      <c r="M59" s="83"/>
+      <c r="N59" s="83"/>
+      <c r="O59" s="83"/>
+      <c r="P59" s="83"/>
+      <c r="Q59" s="83"/>
+      <c r="R59" s="83"/>
+      <c r="S59" s="83"/>
+      <c r="T59" s="83"/>
+      <c r="U59" s="83"/>
+      <c r="V59" s="83"/>
+      <c r="W59" s="83"/>
+      <c r="X59" s="83"/>
+      <c r="Y59" s="83"/>
+      <c r="Z59" s="83"/>
+      <c r="AA59" s="83"/>
+      <c r="AB59" s="83"/>
+      <c r="AC59" s="83"/>
+      <c r="AD59" s="83"/>
+      <c r="AE59" s="83"/>
+    </row>
+    <row r="60" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A60" s="83"/>
+      <c r="B60" s="83"/>
+      <c r="C60" s="83"/>
+      <c r="D60" s="83"/>
+      <c r="E60" s="83"/>
+      <c r="F60" s="83"/>
+      <c r="G60" s="83"/>
+      <c r="H60" s="83"/>
+      <c r="I60" s="83"/>
+      <c r="J60" s="83"/>
+      <c r="K60" s="83"/>
+      <c r="L60" s="83"/>
+      <c r="M60" s="83"/>
+      <c r="N60" s="83"/>
+      <c r="O60" s="83"/>
+      <c r="P60" s="83"/>
+      <c r="Q60" s="83"/>
+      <c r="R60" s="83"/>
+      <c r="S60" s="83"/>
+      <c r="T60" s="83"/>
+      <c r="U60" s="83"/>
+      <c r="V60" s="83"/>
+      <c r="W60" s="83"/>
+      <c r="X60" s="83"/>
+      <c r="Y60" s="83"/>
+      <c r="Z60" s="83"/>
+      <c r="AA60" s="83"/>
+      <c r="AB60" s="83"/>
+      <c r="AC60" s="83"/>
+      <c r="AD60" s="83"/>
+      <c r="AE60" s="83"/>
+    </row>
+    <row r="61" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A61" s="83"/>
+      <c r="B61" s="83"/>
+      <c r="C61" s="83"/>
+      <c r="D61" s="83"/>
+      <c r="E61" s="83"/>
+      <c r="F61" s="83"/>
+      <c r="G61" s="83"/>
+      <c r="H61" s="83"/>
+      <c r="I61" s="83"/>
+      <c r="J61" s="83"/>
+      <c r="K61" s="83"/>
+      <c r="L61" s="83"/>
+      <c r="M61" s="83"/>
+      <c r="N61" s="83"/>
+      <c r="O61" s="83"/>
+      <c r="P61" s="83"/>
+      <c r="Q61" s="83"/>
+      <c r="R61" s="83"/>
+      <c r="S61" s="83"/>
+      <c r="T61" s="83"/>
+      <c r="U61" s="83"/>
+      <c r="V61" s="83"/>
+      <c r="W61" s="83"/>
+      <c r="X61" s="83"/>
+      <c r="Y61" s="83"/>
+      <c r="Z61" s="83"/>
+      <c r="AA61" s="83"/>
+      <c r="AB61" s="83"/>
+      <c r="AC61" s="83"/>
+      <c r="AD61" s="83"/>
+      <c r="AE61" s="83"/>
+    </row>
+    <row r="62" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A62" s="83"/>
+      <c r="B62" s="83"/>
+      <c r="C62" s="83"/>
+      <c r="D62" s="83"/>
+      <c r="E62" s="83"/>
+      <c r="F62" s="83"/>
+      <c r="G62" s="83"/>
+      <c r="H62" s="83"/>
+      <c r="I62" s="83"/>
+      <c r="J62" s="83"/>
+      <c r="K62" s="83"/>
+      <c r="L62" s="83"/>
+      <c r="M62" s="83"/>
+      <c r="N62" s="83"/>
+      <c r="O62" s="83"/>
+      <c r="P62" s="83"/>
+      <c r="Q62" s="83"/>
+      <c r="R62" s="83"/>
+      <c r="S62" s="83"/>
+      <c r="T62" s="83"/>
+      <c r="U62" s="83"/>
+      <c r="V62" s="83"/>
+      <c r="W62" s="83"/>
+      <c r="X62" s="83"/>
+      <c r="Y62" s="83"/>
+      <c r="Z62" s="83"/>
+      <c r="AA62" s="83"/>
+      <c r="AB62" s="83"/>
+      <c r="AC62" s="83"/>
+      <c r="AD62" s="83"/>
+      <c r="AE62" s="83"/>
+    </row>
+    <row r="63" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A63" s="83"/>
+      <c r="B63" s="83"/>
+      <c r="C63" s="83"/>
+      <c r="D63" s="83"/>
+      <c r="E63" s="83"/>
+      <c r="F63" s="83"/>
+      <c r="G63" s="83"/>
+      <c r="H63" s="83"/>
+      <c r="I63" s="83"/>
+      <c r="J63" s="83"/>
+      <c r="K63" s="83"/>
+      <c r="L63" s="83"/>
+      <c r="M63" s="83"/>
+      <c r="N63" s="83"/>
+      <c r="O63" s="83"/>
+      <c r="P63" s="83"/>
+      <c r="Q63" s="83"/>
+      <c r="R63" s="83"/>
+      <c r="S63" s="83"/>
+      <c r="T63" s="83"/>
+      <c r="U63" s="83"/>
+      <c r="V63" s="83"/>
+      <c r="W63" s="83"/>
+      <c r="X63" s="83"/>
+      <c r="Y63" s="83"/>
+      <c r="Z63" s="83"/>
+      <c r="AA63" s="83"/>
+      <c r="AB63" s="83"/>
+      <c r="AC63" s="83"/>
+      <c r="AD63" s="83"/>
+      <c r="AE63" s="83"/>
+    </row>
+    <row r="64" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A64" s="83"/>
+      <c r="B64" s="83"/>
+      <c r="C64" s="83"/>
+      <c r="D64" s="83"/>
+      <c r="E64" s="83"/>
+      <c r="F64" s="83"/>
+      <c r="G64" s="83"/>
+      <c r="H64" s="83"/>
+      <c r="I64" s="83"/>
+      <c r="J64" s="83"/>
+      <c r="K64" s="83"/>
+      <c r="L64" s="83"/>
+      <c r="M64" s="83"/>
+      <c r="N64" s="83"/>
+      <c r="O64" s="83"/>
+      <c r="P64" s="83"/>
+      <c r="Q64" s="83"/>
+      <c r="R64" s="83"/>
+      <c r="S64" s="83"/>
+      <c r="T64" s="83"/>
+      <c r="U64" s="83"/>
+      <c r="V64" s="83"/>
+      <c r="W64" s="83"/>
+      <c r="X64" s="83"/>
+      <c r="Y64" s="83"/>
+      <c r="Z64" s="83"/>
+      <c r="AA64" s="83"/>
+      <c r="AB64" s="83"/>
+      <c r="AC64" s="83"/>
+      <c r="AD64" s="83"/>
+      <c r="AE64" s="83"/>
+    </row>
+    <row r="65" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A65" s="83"/>
+      <c r="B65" s="83"/>
+      <c r="C65" s="83"/>
+      <c r="D65" s="83"/>
+      <c r="E65" s="83"/>
+      <c r="F65" s="83"/>
+      <c r="G65" s="83"/>
+      <c r="H65" s="83"/>
+      <c r="I65" s="83"/>
+      <c r="J65" s="83"/>
+      <c r="K65" s="83"/>
+      <c r="L65" s="83"/>
+      <c r="M65" s="83"/>
+      <c r="N65" s="83"/>
+      <c r="O65" s="83"/>
+      <c r="P65" s="83"/>
+      <c r="Q65" s="83"/>
+      <c r="R65" s="83"/>
+      <c r="S65" s="83"/>
+      <c r="T65" s="83"/>
+      <c r="U65" s="83"/>
+      <c r="V65" s="83"/>
+      <c r="W65" s="83"/>
+      <c r="X65" s="83"/>
+      <c r="Y65" s="83"/>
+      <c r="Z65" s="83"/>
+      <c r="AA65" s="83"/>
+      <c r="AB65" s="83"/>
+      <c r="AC65" s="83"/>
+      <c r="AD65" s="83"/>
+      <c r="AE65" s="83"/>
+    </row>
+    <row r="66" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A66" s="83"/>
+      <c r="B66" s="83"/>
+      <c r="C66" s="83"/>
+      <c r="D66" s="83"/>
+      <c r="E66" s="83"/>
+      <c r="F66" s="83"/>
+      <c r="G66" s="83"/>
+      <c r="H66" s="83"/>
+      <c r="I66" s="83"/>
+      <c r="J66" s="83"/>
+      <c r="K66" s="83"/>
+      <c r="L66" s="83"/>
+      <c r="M66" s="83"/>
+      <c r="N66" s="83"/>
+      <c r="O66" s="83"/>
+      <c r="P66" s="83"/>
+      <c r="Q66" s="83"/>
+      <c r="R66" s="83"/>
+      <c r="S66" s="83"/>
+      <c r="T66" s="83"/>
+      <c r="U66" s="83"/>
+      <c r="V66" s="83"/>
+      <c r="W66" s="83"/>
+      <c r="X66" s="83"/>
+      <c r="Y66" s="83"/>
+      <c r="Z66" s="83"/>
+      <c r="AA66" s="83"/>
+      <c r="AB66" s="83"/>
+      <c r="AC66" s="83"/>
+      <c r="AD66" s="83"/>
+      <c r="AE66" s="83"/>
+    </row>
+    <row r="67" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A67" s="83"/>
+      <c r="B67" s="83"/>
+      <c r="C67" s="83"/>
+      <c r="D67" s="83"/>
+      <c r="E67" s="83"/>
+      <c r="F67" s="83"/>
+      <c r="G67" s="83"/>
+      <c r="H67" s="83"/>
+      <c r="I67" s="83"/>
+      <c r="J67" s="83"/>
+      <c r="K67" s="83"/>
+      <c r="L67" s="83"/>
+      <c r="M67" s="83"/>
+      <c r="N67" s="83"/>
+      <c r="O67" s="83"/>
+      <c r="P67" s="83"/>
+      <c r="Q67" s="83"/>
+      <c r="R67" s="83"/>
+      <c r="S67" s="83"/>
+      <c r="T67" s="83"/>
+      <c r="U67" s="83"/>
+      <c r="V67" s="83"/>
+      <c r="W67" s="83"/>
+      <c r="X67" s="83"/>
+      <c r="Y67" s="83"/>
+      <c r="Z67" s="83"/>
+      <c r="AA67" s="83"/>
+      <c r="AB67" s="83"/>
+      <c r="AC67" s="83"/>
+      <c r="AD67" s="83"/>
+      <c r="AE67" s="83"/>
+    </row>
+    <row r="68" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A68" s="83"/>
+      <c r="B68" s="83"/>
+      <c r="C68" s="83"/>
+      <c r="D68" s="83"/>
+      <c r="E68" s="83"/>
+      <c r="F68" s="83"/>
+      <c r="G68" s="83"/>
+      <c r="H68" s="83"/>
+      <c r="I68" s="83"/>
+      <c r="J68" s="83"/>
+      <c r="K68" s="83"/>
+      <c r="L68" s="83"/>
+      <c r="M68" s="83"/>
+      <c r="N68" s="83"/>
+      <c r="O68" s="83"/>
+      <c r="P68" s="83"/>
+      <c r="Q68" s="83"/>
+      <c r="R68" s="83"/>
+      <c r="S68" s="83"/>
+      <c r="T68" s="83"/>
+      <c r="U68" s="83"/>
+      <c r="V68" s="83"/>
+      <c r="W68" s="83"/>
+      <c r="X68" s="83"/>
+      <c r="Y68" s="83"/>
+      <c r="Z68" s="83"/>
+      <c r="AA68" s="83"/>
+      <c r="AB68" s="83"/>
+      <c r="AC68" s="83"/>
+      <c r="AD68" s="83"/>
+      <c r="AE68" s="83"/>
+    </row>
+    <row r="69" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A69" s="83"/>
+      <c r="B69" s="83"/>
+      <c r="C69" s="83"/>
+      <c r="D69" s="83"/>
+      <c r="E69" s="83"/>
+      <c r="F69" s="83"/>
+      <c r="G69" s="83"/>
+      <c r="H69" s="83"/>
+      <c r="I69" s="83"/>
+      <c r="J69" s="83"/>
+      <c r="K69" s="83"/>
+      <c r="L69" s="83"/>
+      <c r="M69" s="83"/>
+      <c r="N69" s="83"/>
+      <c r="O69" s="83"/>
+      <c r="P69" s="83"/>
+      <c r="Q69" s="83"/>
+      <c r="R69" s="83"/>
+      <c r="S69" s="83"/>
+      <c r="T69" s="83"/>
+      <c r="U69" s="83"/>
+      <c r="V69" s="83"/>
+      <c r="W69" s="83"/>
+      <c r="X69" s="83"/>
+      <c r="Y69" s="83"/>
+      <c r="Z69" s="83"/>
+      <c r="AA69" s="83"/>
+      <c r="AB69" s="83"/>
+      <c r="AC69" s="83"/>
+      <c r="AD69" s="83"/>
+      <c r="AE69" s="83"/>
+    </row>
+    <row r="70" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A70" s="83"/>
+      <c r="B70" s="83"/>
+      <c r="C70" s="83"/>
+      <c r="D70" s="83"/>
+      <c r="E70" s="83"/>
+      <c r="F70" s="83"/>
+      <c r="G70" s="83"/>
+      <c r="H70" s="83"/>
+      <c r="I70" s="83"/>
+      <c r="J70" s="83"/>
+      <c r="K70" s="83"/>
+      <c r="L70" s="83"/>
+      <c r="M70" s="83"/>
+      <c r="N70" s="83"/>
+      <c r="O70" s="83"/>
+      <c r="P70" s="83"/>
+      <c r="Q70" s="83"/>
+      <c r="R70" s="83"/>
+      <c r="S70" s="83"/>
+      <c r="T70" s="83"/>
+      <c r="U70" s="83"/>
+      <c r="V70" s="83"/>
+      <c r="W70" s="83"/>
+      <c r="X70" s="83"/>
+      <c r="Y70" s="83"/>
+      <c r="Z70" s="83"/>
+      <c r="AA70" s="83"/>
+      <c r="AB70" s="83"/>
+      <c r="AC70" s="83"/>
+      <c r="AD70" s="83"/>
+      <c r="AE70" s="83"/>
+    </row>
+    <row r="71" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A71" s="83"/>
+      <c r="B71" s="83"/>
+      <c r="C71" s="83"/>
+      <c r="D71" s="83"/>
+      <c r="E71" s="83"/>
+      <c r="F71" s="83"/>
+      <c r="G71" s="83"/>
+      <c r="H71" s="83"/>
+      <c r="I71" s="83"/>
+      <c r="J71" s="83"/>
+      <c r="K71" s="83"/>
+      <c r="L71" s="83"/>
+      <c r="M71" s="83"/>
+      <c r="N71" s="83"/>
+      <c r="O71" s="83"/>
+      <c r="P71" s="83"/>
+      <c r="Q71" s="83"/>
+      <c r="R71" s="83"/>
+      <c r="S71" s="83"/>
+      <c r="T71" s="83"/>
+      <c r="U71" s="83"/>
+      <c r="V71" s="83"/>
+      <c r="W71" s="83"/>
+      <c r="X71" s="83"/>
+      <c r="Y71" s="83"/>
+      <c r="Z71" s="83"/>
+      <c r="AA71" s="83"/>
+      <c r="AB71" s="83"/>
+      <c r="AC71" s="83"/>
+      <c r="AD71" s="83"/>
+      <c r="AE71" s="83"/>
+    </row>
+    <row r="72" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A72" s="83"/>
+      <c r="B72" s="83"/>
+      <c r="C72" s="83"/>
+      <c r="D72" s="83"/>
+      <c r="E72" s="83"/>
+      <c r="F72" s="83"/>
+      <c r="G72" s="83"/>
+      <c r="H72" s="83"/>
+      <c r="I72" s="83"/>
+      <c r="J72" s="83"/>
+      <c r="K72" s="83"/>
+      <c r="L72" s="83"/>
+      <c r="M72" s="83"/>
+      <c r="N72" s="83"/>
+      <c r="O72" s="83"/>
+      <c r="P72" s="83"/>
+      <c r="Q72" s="83"/>
+      <c r="R72" s="83"/>
+      <c r="S72" s="83"/>
+      <c r="T72" s="83"/>
+      <c r="U72" s="83"/>
+      <c r="V72" s="83"/>
+      <c r="W72" s="83"/>
+      <c r="X72" s="83"/>
+      <c r="Y72" s="83"/>
+      <c r="Z72" s="83"/>
+      <c r="AA72" s="83"/>
+      <c r="AB72" s="83"/>
+      <c r="AC72" s="83"/>
+      <c r="AD72" s="83"/>
+      <c r="AE72" s="83"/>
+    </row>
+    <row r="73" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A73" s="83"/>
+      <c r="B73" s="83"/>
+      <c r="C73" s="83"/>
+      <c r="D73" s="83"/>
+      <c r="E73" s="83"/>
+      <c r="F73" s="83"/>
+      <c r="G73" s="83"/>
+      <c r="H73" s="83"/>
+      <c r="I73" s="83"/>
+      <c r="J73" s="83"/>
+      <c r="K73" s="83"/>
+      <c r="L73" s="83"/>
+      <c r="M73" s="83"/>
+      <c r="N73" s="83"/>
+      <c r="O73" s="83"/>
+      <c r="P73" s="83"/>
+      <c r="Q73" s="83"/>
+      <c r="R73" s="83"/>
+      <c r="S73" s="83"/>
+      <c r="T73" s="83"/>
+      <c r="U73" s="83"/>
+      <c r="V73" s="83"/>
+      <c r="W73" s="83"/>
+      <c r="X73" s="83"/>
+      <c r="Y73" s="83"/>
+      <c r="Z73" s="83"/>
+      <c r="AA73" s="83"/>
+      <c r="AB73" s="83"/>
+      <c r="AC73" s="83"/>
+      <c r="AD73" s="83"/>
+      <c r="AE73" s="83"/>
+    </row>
+    <row r="74" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A74" s="83"/>
+      <c r="B74" s="83"/>
+      <c r="C74" s="83"/>
+      <c r="D74" s="83"/>
+      <c r="E74" s="83"/>
+      <c r="F74" s="83"/>
+      <c r="G74" s="83"/>
+      <c r="H74" s="83"/>
+      <c r="I74" s="83"/>
+      <c r="J74" s="83"/>
+      <c r="K74" s="83"/>
+      <c r="L74" s="83"/>
+      <c r="M74" s="83"/>
+      <c r="N74" s="83"/>
+      <c r="O74" s="83"/>
+      <c r="P74" s="83"/>
+      <c r="Q74" s="83"/>
+      <c r="R74" s="83"/>
+      <c r="S74" s="83"/>
+      <c r="T74" s="83"/>
+      <c r="U74" s="83"/>
+      <c r="V74" s="83"/>
+      <c r="W74" s="83"/>
+      <c r="X74" s="83"/>
+      <c r="Y74" s="83"/>
+      <c r="Z74" s="83"/>
+      <c r="AA74" s="83"/>
+      <c r="AB74" s="83"/>
+      <c r="AC74" s="83"/>
+      <c r="AD74" s="83"/>
+      <c r="AE74" s="83"/>
+    </row>
+    <row r="75" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A75" s="83"/>
+      <c r="B75" s="83"/>
+      <c r="C75" s="83"/>
+      <c r="D75" s="83"/>
+      <c r="E75" s="83"/>
+      <c r="F75" s="83"/>
+      <c r="G75" s="83"/>
+      <c r="H75" s="83"/>
+      <c r="I75" s="83"/>
+      <c r="J75" s="83"/>
+      <c r="K75" s="83"/>
+      <c r="L75" s="83"/>
+      <c r="M75" s="83"/>
+      <c r="N75" s="83"/>
+      <c r="O75" s="83"/>
+      <c r="P75" s="83"/>
+      <c r="Q75" s="83"/>
+      <c r="R75" s="83"/>
+      <c r="S75" s="83"/>
+      <c r="T75" s="83"/>
+      <c r="U75" s="83"/>
+      <c r="V75" s="83"/>
+      <c r="W75" s="83"/>
+      <c r="X75" s="83"/>
+      <c r="Y75" s="83"/>
+      <c r="Z75" s="83"/>
+      <c r="AA75" s="83"/>
+      <c r="AB75" s="83"/>
+      <c r="AC75" s="83"/>
+      <c r="AD75" s="83"/>
+      <c r="AE75" s="83"/>
+    </row>
+    <row r="76" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A76" s="83"/>
+      <c r="B76" s="83"/>
+      <c r="C76" s="83"/>
+      <c r="D76" s="83"/>
+      <c r="E76" s="83"/>
+      <c r="F76" s="83"/>
+      <c r="G76" s="83"/>
+      <c r="H76" s="83"/>
+      <c r="I76" s="83"/>
+      <c r="J76" s="83"/>
+      <c r="K76" s="83"/>
+      <c r="L76" s="83"/>
+      <c r="M76" s="83"/>
+      <c r="N76" s="83"/>
+      <c r="O76" s="83"/>
+      <c r="P76" s="83"/>
+      <c r="Q76" s="83"/>
+      <c r="R76" s="83"/>
+      <c r="S76" s="83"/>
+      <c r="T76" s="83"/>
+      <c r="U76" s="83"/>
+      <c r="V76" s="83"/>
+      <c r="W76" s="83"/>
+      <c r="X76" s="83"/>
+      <c r="Y76" s="83"/>
+      <c r="Z76" s="83"/>
+      <c r="AA76" s="83"/>
+      <c r="AB76" s="83"/>
+      <c r="AC76" s="83"/>
+      <c r="AD76" s="83"/>
+      <c r="AE76" s="83"/>
+    </row>
+    <row r="77" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A77" s="83"/>
+      <c r="B77" s="83"/>
+      <c r="C77" s="83"/>
+      <c r="D77" s="83"/>
+      <c r="E77" s="83"/>
+      <c r="F77" s="83"/>
+      <c r="G77" s="83"/>
+      <c r="H77" s="83"/>
+      <c r="I77" s="83"/>
+      <c r="J77" s="83"/>
+      <c r="K77" s="83"/>
+      <c r="L77" s="83"/>
+      <c r="M77" s="83"/>
+      <c r="N77" s="83"/>
+      <c r="O77" s="83"/>
+      <c r="P77" s="83"/>
+      <c r="Q77" s="83"/>
+      <c r="R77" s="83"/>
+      <c r="S77" s="83"/>
+      <c r="T77" s="83"/>
+      <c r="U77" s="83"/>
+      <c r="V77" s="83"/>
+      <c r="W77" s="83"/>
+      <c r="X77" s="83"/>
+      <c r="Y77" s="83"/>
+      <c r="Z77" s="83"/>
+      <c r="AA77" s="83"/>
+      <c r="AB77" s="83"/>
+      <c r="AC77" s="83"/>
+      <c r="AD77" s="83"/>
+      <c r="AE77" s="83"/>
+    </row>
+    <row r="78" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A78" s="83"/>
+      <c r="B78" s="83"/>
+      <c r="C78" s="83"/>
+      <c r="D78" s="83"/>
+      <c r="E78" s="83"/>
+      <c r="F78" s="83"/>
+      <c r="G78" s="83"/>
+      <c r="H78" s="83"/>
+      <c r="I78" s="83"/>
+      <c r="J78" s="83"/>
+      <c r="K78" s="83"/>
+      <c r="L78" s="83"/>
+      <c r="M78" s="83"/>
+      <c r="N78" s="83"/>
+      <c r="O78" s="83"/>
+      <c r="P78" s="83"/>
+      <c r="Q78" s="83"/>
+      <c r="R78" s="83"/>
+      <c r="S78" s="83"/>
+      <c r="T78" s="83"/>
+      <c r="U78" s="83"/>
+      <c r="V78" s="83"/>
+      <c r="W78" s="83"/>
+      <c r="X78" s="83"/>
+      <c r="Y78" s="83"/>
+      <c r="Z78" s="83"/>
+      <c r="AA78" s="83"/>
+      <c r="AB78" s="83"/>
+      <c r="AC78" s="83"/>
+      <c r="AD78" s="83"/>
+      <c r="AE78" s="83"/>
+    </row>
+    <row r="79" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A79" s="83"/>
+      <c r="B79" s="83"/>
+      <c r="C79" s="83"/>
+      <c r="D79" s="83"/>
+      <c r="E79" s="83"/>
+      <c r="F79" s="83"/>
+      <c r="G79" s="83"/>
+      <c r="H79" s="83"/>
+      <c r="I79" s="83"/>
+      <c r="J79" s="83"/>
+      <c r="K79" s="83"/>
+      <c r="L79" s="83"/>
+      <c r="M79" s="83"/>
+      <c r="N79" s="83"/>
+      <c r="O79" s="83"/>
+      <c r="P79" s="83"/>
+      <c r="Q79" s="83"/>
+      <c r="R79" s="83"/>
+      <c r="S79" s="83"/>
+      <c r="T79" s="83"/>
+      <c r="U79" s="83"/>
+      <c r="V79" s="83"/>
+      <c r="W79" s="83"/>
+      <c r="X79" s="83"/>
+      <c r="Y79" s="83"/>
+      <c r="Z79" s="83"/>
+      <c r="AA79" s="83"/>
+      <c r="AB79" s="83"/>
+      <c r="AC79" s="83"/>
+      <c r="AD79" s="83"/>
+      <c r="AE79" s="83"/>
+    </row>
+    <row r="80" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A80" s="83"/>
+      <c r="B80" s="83"/>
+      <c r="C80" s="83"/>
+      <c r="D80" s="83"/>
+      <c r="E80" s="83"/>
+      <c r="F80" s="83"/>
+      <c r="G80" s="83"/>
+      <c r="H80" s="83"/>
+      <c r="I80" s="83"/>
+      <c r="J80" s="83"/>
+      <c r="K80" s="83"/>
+      <c r="L80" s="83"/>
+      <c r="M80" s="83"/>
+      <c r="N80" s="83"/>
+      <c r="O80" s="83"/>
+      <c r="P80" s="83"/>
+      <c r="Q80" s="83"/>
+      <c r="R80" s="83"/>
+      <c r="S80" s="83"/>
+      <c r="T80" s="83"/>
+      <c r="U80" s="83"/>
+      <c r="V80" s="83"/>
+      <c r="W80" s="83"/>
+      <c r="X80" s="83"/>
+      <c r="Y80" s="83"/>
+      <c r="Z80" s="83"/>
+      <c r="AA80" s="83"/>
+      <c r="AB80" s="83"/>
+      <c r="AC80" s="83"/>
+      <c r="AD80" s="83"/>
+      <c r="AE80" s="83"/>
+    </row>
+    <row r="81" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A81" s="83"/>
+      <c r="B81" s="83"/>
+      <c r="C81" s="83"/>
+      <c r="D81" s="83"/>
+      <c r="E81" s="83"/>
+      <c r="F81" s="83"/>
+      <c r="G81" s="83"/>
+      <c r="H81" s="83"/>
+      <c r="I81" s="83"/>
+      <c r="J81" s="83"/>
+      <c r="K81" s="83"/>
+      <c r="L81" s="83"/>
+      <c r="M81" s="83"/>
+      <c r="N81" s="83"/>
+      <c r="O81" s="83"/>
+      <c r="P81" s="83"/>
+      <c r="Q81" s="83"/>
+      <c r="R81" s="83"/>
+      <c r="S81" s="83"/>
+      <c r="T81" s="83"/>
+      <c r="U81" s="83"/>
+      <c r="V81" s="83"/>
+      <c r="W81" s="83"/>
+      <c r="X81" s="83"/>
+      <c r="Y81" s="83"/>
+      <c r="Z81" s="83"/>
+      <c r="AA81" s="83"/>
+      <c r="AB81" s="83"/>
+      <c r="AC81" s="83"/>
+      <c r="AD81" s="83"/>
+      <c r="AE81" s="83"/>
+    </row>
+    <row r="82" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A82" s="83"/>
+      <c r="B82" s="83"/>
+      <c r="C82" s="83"/>
+      <c r="D82" s="83"/>
+      <c r="E82" s="83"/>
+      <c r="F82" s="83"/>
+      <c r="G82" s="83"/>
+      <c r="H82" s="83"/>
+      <c r="I82" s="83"/>
+      <c r="J82" s="83"/>
+      <c r="K82" s="83"/>
+      <c r="L82" s="83"/>
+      <c r="M82" s="83"/>
+      <c r="N82" s="83"/>
+      <c r="O82" s="83"/>
+      <c r="P82" s="83"/>
+      <c r="Q82" s="83"/>
+      <c r="R82" s="83"/>
+      <c r="S82" s="83"/>
+      <c r="T82" s="83"/>
+      <c r="U82" s="83"/>
+      <c r="V82" s="83"/>
+      <c r="W82" s="83"/>
+      <c r="X82" s="83"/>
+      <c r="Y82" s="83"/>
+      <c r="Z82" s="83"/>
+      <c r="AA82" s="83"/>
+      <c r="AB82" s="83"/>
+      <c r="AC82" s="83"/>
+      <c r="AD82" s="83"/>
+      <c r="AE82" s="83"/>
+    </row>
+    <row r="83" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A83" s="83"/>
+      <c r="B83" s="83"/>
+      <c r="C83" s="83"/>
+      <c r="D83" s="83"/>
+      <c r="E83" s="83"/>
+      <c r="F83" s="83"/>
+      <c r="G83" s="83"/>
+      <c r="H83" s="83"/>
+      <c r="I83" s="83"/>
+      <c r="J83" s="83"/>
+      <c r="K83" s="83"/>
+      <c r="L83" s="83"/>
+      <c r="M83" s="83"/>
+      <c r="N83" s="83"/>
+      <c r="O83" s="83"/>
+      <c r="P83" s="83"/>
+      <c r="Q83" s="83"/>
+      <c r="R83" s="83"/>
+      <c r="S83" s="83"/>
+      <c r="T83" s="83"/>
+      <c r="U83" s="83"/>
+      <c r="V83" s="83"/>
+      <c r="W83" s="83"/>
+      <c r="X83" s="83"/>
+      <c r="Y83" s="83"/>
+      <c r="Z83" s="83"/>
+      <c r="AA83" s="83"/>
+      <c r="AB83" s="83"/>
+      <c r="AC83" s="83"/>
+      <c r="AD83" s="83"/>
+      <c r="AE83" s="83"/>
+    </row>
+    <row r="84" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A84" s="83"/>
+      <c r="B84" s="83"/>
+      <c r="C84" s="83"/>
+      <c r="D84" s="83"/>
+      <c r="E84" s="83"/>
+      <c r="F84" s="83"/>
+      <c r="G84" s="83"/>
+      <c r="H84" s="83"/>
+      <c r="I84" s="83"/>
+      <c r="J84" s="83"/>
+      <c r="K84" s="83"/>
+      <c r="L84" s="83"/>
+      <c r="M84" s="83"/>
+      <c r="N84" s="83"/>
+      <c r="O84" s="83"/>
+      <c r="P84" s="83"/>
+      <c r="Q84" s="83"/>
+      <c r="R84" s="83"/>
+      <c r="S84" s="83"/>
+      <c r="T84" s="83"/>
+      <c r="U84" s="83"/>
+      <c r="V84" s="83"/>
+      <c r="W84" s="83"/>
+      <c r="X84" s="83"/>
+      <c r="Y84" s="83"/>
+      <c r="Z84" s="83"/>
+      <c r="AA84" s="83"/>
+      <c r="AB84" s="83"/>
+      <c r="AC84" s="83"/>
+      <c r="AD84" s="83"/>
+      <c r="AE84" s="83"/>
+    </row>
+    <row r="85" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A85" s="83"/>
+      <c r="B85" s="83"/>
+      <c r="C85" s="83"/>
+      <c r="D85" s="83"/>
+      <c r="E85" s="83"/>
+      <c r="F85" s="83"/>
+      <c r="G85" s="83"/>
+      <c r="H85" s="83"/>
+      <c r="I85" s="83"/>
+      <c r="J85" s="83"/>
+      <c r="K85" s="83"/>
+      <c r="L85" s="83"/>
+      <c r="M85" s="83"/>
+      <c r="N85" s="83"/>
+      <c r="O85" s="83"/>
+      <c r="P85" s="83"/>
+      <c r="Q85" s="83"/>
+      <c r="R85" s="83"/>
+      <c r="S85" s="83"/>
+      <c r="T85" s="83"/>
+      <c r="U85" s="83"/>
+      <c r="V85" s="83"/>
+      <c r="W85" s="83"/>
+      <c r="X85" s="83"/>
+      <c r="Y85" s="83"/>
+      <c r="Z85" s="83"/>
+      <c r="AA85" s="83"/>
+      <c r="AB85" s="83"/>
+      <c r="AC85" s="83"/>
+      <c r="AD85" s="83"/>
+      <c r="AE85" s="83"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
MM23 new excel done
</commit_message>
<xml_diff>
--- a/Manual/MM23_cleaned.xlsx
+++ b/Manual/MM23_cleaned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/onettperera/Desktop/ADS_Easter/Manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CDD7B3-AF62-0443-8D9E-AC0CF5295008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305A863A-1F84-F547-854F-4723095BA0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{B1576BF3-F55A-1D42-85D3-6C766BD046A7}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{B1576BF3-F55A-1D42-85D3-6C766BD046A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="134">
   <si>
     <t>aggregate number</t>
   </si>
@@ -434,6 +434,9 @@
   </si>
   <si>
     <t>Actual Rent</t>
+  </si>
+  <si>
+    <t>Energy</t>
   </si>
   <si>
     <t>Financial Year</t>
@@ -27594,12 +27597,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FA976F5-DA60-5F43-AF37-C024C9208180}">
-  <dimension ref="A1:VB25"/>
+  <dimension ref="A1:UL25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A1" s="83" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B1" s="83" t="s">
         <v>118</v>
@@ -27643,7 +27646,9 @@
       <c r="O1" s="83" t="s">
         <v>131</v>
       </c>
-      <c r="P1" s="83"/>
+      <c r="P1" s="83" t="s">
+        <v>132</v>
+      </c>
       <c r="Q1" s="83"/>
       <c r="R1" s="83"/>
       <c r="S1" s="83"/>
@@ -27723,7 +27728,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!Q$4:Q$461)</f>
         <v>100.72233333333334</v>
       </c>
-      <c r="P2" s="83"/>
+      <c r="P2" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!R$4:R$461)</f>
+        <v>98.998583333333329</v>
+      </c>
       <c r="Q2" s="83"/>
       <c r="R2" s="83"/>
       <c r="S2" s="83"/>
@@ -27803,7 +27811,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!Q$4:Q$461)</f>
         <v>102.063</v>
       </c>
-      <c r="P3" s="83"/>
+      <c r="P3" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A3,Monthly!R$4:R$461)</f>
+        <v>97.220999999999989</v>
+      </c>
       <c r="Q3" s="83"/>
       <c r="R3" s="83"/>
       <c r="S3" s="83"/>
@@ -27883,7 +27894,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!Q$4:Q$461)</f>
         <v>102.80433333333333</v>
       </c>
-      <c r="P4" s="83"/>
+      <c r="P4" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A4,Monthly!R$4:R$461)</f>
+        <v>102.45150000000001</v>
+      </c>
       <c r="Q4" s="83"/>
       <c r="R4" s="83"/>
       <c r="S4" s="83"/>
@@ -27963,7 +27977,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!Q$4:Q$461)</f>
         <v>103.36333333333334</v>
       </c>
-      <c r="P5" s="83"/>
+      <c r="P5" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A5,Monthly!R$4:R$461)</f>
+        <v>108.18466666666666</v>
+      </c>
       <c r="Q5" s="83"/>
       <c r="R5" s="83"/>
       <c r="S5" s="83"/>
@@ -28043,7 +28060,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!Q$4:Q$461)</f>
         <v>104.1439166666667</v>
       </c>
-      <c r="P6" s="83"/>
+      <c r="P6" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A6,Monthly!R$4:R$461)</f>
+        <v>112.86333333333333</v>
+      </c>
       <c r="Q6" s="83"/>
       <c r="R6" s="83"/>
       <c r="S6" s="83"/>
@@ -28123,7 +28143,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!Q$4:Q$461)</f>
         <v>105.88483333333335</v>
       </c>
-      <c r="P7" s="83"/>
+      <c r="P7" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A7,Monthly!R$4:R$461)</f>
+        <v>104.46749999999999</v>
+      </c>
       <c r="Q7" s="83"/>
       <c r="R7" s="83"/>
       <c r="S7" s="83"/>
@@ -28203,7 +28226,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!Q$4:Q$461)</f>
         <v>107.80974999999999</v>
       </c>
-      <c r="P8" s="83"/>
+      <c r="P8" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A8,Monthly!R$4:R$461)</f>
+        <v>117.88975000000001</v>
+      </c>
       <c r="Q8" s="83"/>
       <c r="R8" s="83"/>
       <c r="S8" s="83"/>
@@ -28283,7 +28309,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!Q$4:Q$461)</f>
         <v>112.18416666666667</v>
       </c>
-      <c r="P9" s="83"/>
+      <c r="P9" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A9,Monthly!R$4:R$461)</f>
+        <v>211.10791666666663</v>
+      </c>
       <c r="Q9" s="83"/>
       <c r="R9" s="83"/>
       <c r="S9" s="83"/>
@@ -28363,7 +28392,10 @@
         <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!Q$4:Q$461)</f>
         <v>119.24366666666664</v>
       </c>
-      <c r="P10" s="83"/>
+      <c r="P10" s="83">
+        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A10,Monthly!R$4:R$461)</f>
+        <v>200.73016666666669</v>
+      </c>
       <c r="Q10" s="83"/>
       <c r="R10" s="83"/>
       <c r="S10" s="83"/>
@@ -28402,22 +28434,6 @@
       <c r="P11" s="83"/>
       <c r="Q11" s="83"/>
       <c r="R11" s="83"/>
-      <c r="S11" s="83"/>
-      <c r="T11" s="83"/>
-      <c r="U11" s="83"/>
-      <c r="V11" s="83"/>
-      <c r="W11" s="83"/>
-      <c r="X11" s="83"/>
-      <c r="Y11" s="83"/>
-      <c r="Z11" s="83"/>
-      <c r="AA11" s="83"/>
-      <c r="AB11" s="83"/>
-      <c r="AC11" s="83"/>
-      <c r="AD11" s="83"/>
-      <c r="AE11" s="83"/>
-      <c r="AF11" s="83"/>
-      <c r="AG11" s="83"/>
-      <c r="AH11" s="83"/>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A12" s="83"/>
@@ -28438,22 +28454,6 @@
       <c r="P12" s="83"/>
       <c r="Q12" s="83"/>
       <c r="R12" s="83"/>
-      <c r="S12" s="83"/>
-      <c r="T12" s="83"/>
-      <c r="U12" s="83"/>
-      <c r="V12" s="83"/>
-      <c r="W12" s="83"/>
-      <c r="X12" s="83"/>
-      <c r="Y12" s="83"/>
-      <c r="Z12" s="83"/>
-      <c r="AA12" s="83"/>
-      <c r="AB12" s="83"/>
-      <c r="AC12" s="83"/>
-      <c r="AD12" s="83"/>
-      <c r="AE12" s="83"/>
-      <c r="AF12" s="83"/>
-      <c r="AG12" s="83"/>
-      <c r="AH12" s="83"/>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A13" s="83"/>
@@ -28474,22 +28474,6 @@
       <c r="P13" s="83"/>
       <c r="Q13" s="83"/>
       <c r="R13" s="83"/>
-      <c r="S13" s="83"/>
-      <c r="T13" s="83"/>
-      <c r="U13" s="83"/>
-      <c r="V13" s="83"/>
-      <c r="W13" s="83"/>
-      <c r="X13" s="83"/>
-      <c r="Y13" s="83"/>
-      <c r="Z13" s="83"/>
-      <c r="AA13" s="83"/>
-      <c r="AB13" s="83"/>
-      <c r="AC13" s="83"/>
-      <c r="AD13" s="83"/>
-      <c r="AE13" s="83"/>
-      <c r="AF13" s="83"/>
-      <c r="AG13" s="83"/>
-      <c r="AH13" s="83"/>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A14" s="83"/>
@@ -28510,22 +28494,6 @@
       <c r="P14" s="83"/>
       <c r="Q14" s="83"/>
       <c r="R14" s="83"/>
-      <c r="S14" s="83"/>
-      <c r="T14" s="83"/>
-      <c r="U14" s="83"/>
-      <c r="V14" s="83"/>
-      <c r="W14" s="83"/>
-      <c r="X14" s="83"/>
-      <c r="Y14" s="83"/>
-      <c r="Z14" s="83"/>
-      <c r="AA14" s="83"/>
-      <c r="AB14" s="83"/>
-      <c r="AC14" s="83"/>
-      <c r="AD14" s="83"/>
-      <c r="AE14" s="83"/>
-      <c r="AF14" s="83"/>
-      <c r="AG14" s="83"/>
-      <c r="AH14" s="83"/>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A15" s="83"/>
@@ -28546,22 +28514,6 @@
       <c r="P15" s="83"/>
       <c r="Q15" s="83"/>
       <c r="R15" s="83"/>
-      <c r="S15" s="83"/>
-      <c r="T15" s="83"/>
-      <c r="U15" s="83"/>
-      <c r="V15" s="83"/>
-      <c r="W15" s="83"/>
-      <c r="X15" s="83"/>
-      <c r="Y15" s="83"/>
-      <c r="Z15" s="83"/>
-      <c r="AA15" s="83"/>
-      <c r="AB15" s="83"/>
-      <c r="AC15" s="83"/>
-      <c r="AD15" s="83"/>
-      <c r="AE15" s="83"/>
-      <c r="AF15" s="83"/>
-      <c r="AG15" s="83"/>
-      <c r="AH15" s="83"/>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A16" s="83"/>
@@ -28582,24 +28534,8 @@
       <c r="P16" s="83"/>
       <c r="Q16" s="83"/>
       <c r="R16" s="83"/>
-      <c r="S16" s="83"/>
-      <c r="T16" s="83"/>
-      <c r="U16" s="83"/>
-      <c r="V16" s="83"/>
-      <c r="W16" s="83"/>
-      <c r="X16" s="83"/>
-      <c r="Y16" s="83"/>
-      <c r="Z16" s="83"/>
-      <c r="AA16" s="83"/>
-      <c r="AB16" s="83"/>
-      <c r="AC16" s="83"/>
-      <c r="AD16" s="83"/>
-      <c r="AE16" s="83"/>
-      <c r="AF16" s="83"/>
-      <c r="AG16" s="83"/>
-      <c r="AH16" s="83"/>
-    </row>
-    <row r="17" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A17" s="83"/>
       <c r="B17" s="83"/>
       <c r="C17" s="83"/>
@@ -28618,24 +28554,8 @@
       <c r="P17" s="83"/>
       <c r="Q17" s="83"/>
       <c r="R17" s="83"/>
-      <c r="S17" s="83"/>
-      <c r="T17" s="83"/>
-      <c r="U17" s="83"/>
-      <c r="V17" s="83"/>
-      <c r="W17" s="83"/>
-      <c r="X17" s="83"/>
-      <c r="Y17" s="83"/>
-      <c r="Z17" s="83"/>
-      <c r="AA17" s="83"/>
-      <c r="AB17" s="83"/>
-      <c r="AC17" s="83"/>
-      <c r="AD17" s="83"/>
-      <c r="AE17" s="83"/>
-      <c r="AF17" s="83"/>
-      <c r="AG17" s="83"/>
-      <c r="AH17" s="83"/>
-    </row>
-    <row r="18" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A18" s="83"/>
       <c r="B18" s="83"/>
       <c r="C18" s="83"/>
@@ -28654,24 +28574,8 @@
       <c r="P18" s="83"/>
       <c r="Q18" s="83"/>
       <c r="R18" s="83"/>
-      <c r="S18" s="83"/>
-      <c r="T18" s="83"/>
-      <c r="U18" s="83"/>
-      <c r="V18" s="83"/>
-      <c r="W18" s="83"/>
-      <c r="X18" s="83"/>
-      <c r="Y18" s="83"/>
-      <c r="Z18" s="83"/>
-      <c r="AA18" s="83"/>
-      <c r="AB18" s="83"/>
-      <c r="AC18" s="83"/>
-      <c r="AD18" s="83"/>
-      <c r="AE18" s="83"/>
-      <c r="AF18" s="83"/>
-      <c r="AG18" s="83"/>
-      <c r="AH18" s="83"/>
-    </row>
-    <row r="19" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A19" s="83"/>
       <c r="B19" s="83"/>
       <c r="C19" s="83"/>
@@ -28690,24 +28594,8 @@
       <c r="P19" s="83"/>
       <c r="Q19" s="83"/>
       <c r="R19" s="83"/>
-      <c r="S19" s="83"/>
-      <c r="T19" s="83"/>
-      <c r="U19" s="83"/>
-      <c r="V19" s="83"/>
-      <c r="W19" s="83"/>
-      <c r="X19" s="83"/>
-      <c r="Y19" s="83"/>
-      <c r="Z19" s="83"/>
-      <c r="AA19" s="83"/>
-      <c r="AB19" s="83"/>
-      <c r="AC19" s="83"/>
-      <c r="AD19" s="83"/>
-      <c r="AE19" s="83"/>
-      <c r="AF19" s="83"/>
-      <c r="AG19" s="83"/>
-      <c r="AH19" s="83"/>
-    </row>
-    <row r="20" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A20" s="83"/>
       <c r="B20" s="83"/>
       <c r="C20" s="83"/>
@@ -28726,24 +28614,8 @@
       <c r="P20" s="83"/>
       <c r="Q20" s="83"/>
       <c r="R20" s="83"/>
-      <c r="S20" s="83"/>
-      <c r="T20" s="83"/>
-      <c r="U20" s="83"/>
-      <c r="V20" s="83"/>
-      <c r="W20" s="83"/>
-      <c r="X20" s="83"/>
-      <c r="Y20" s="83"/>
-      <c r="Z20" s="83"/>
-      <c r="AA20" s="83"/>
-      <c r="AB20" s="83"/>
-      <c r="AC20" s="83"/>
-      <c r="AD20" s="83"/>
-      <c r="AE20" s="83"/>
-      <c r="AF20" s="83"/>
-      <c r="AG20" s="83"/>
-      <c r="AH20" s="83"/>
-    </row>
-    <row r="21" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A21" s="83"/>
       <c r="B21" s="83"/>
       <c r="C21" s="83"/>
@@ -28762,24 +28634,8 @@
       <c r="P21" s="83"/>
       <c r="Q21" s="83"/>
       <c r="R21" s="83"/>
-      <c r="S21" s="83"/>
-      <c r="T21" s="83"/>
-      <c r="U21" s="83"/>
-      <c r="V21" s="83"/>
-      <c r="W21" s="83"/>
-      <c r="X21" s="83"/>
-      <c r="Y21" s="83"/>
-      <c r="Z21" s="83"/>
-      <c r="AA21" s="83"/>
-      <c r="AB21" s="83"/>
-      <c r="AC21" s="83"/>
-      <c r="AD21" s="83"/>
-      <c r="AE21" s="83"/>
-      <c r="AF21" s="83"/>
-      <c r="AG21" s="83"/>
-      <c r="AH21" s="83"/>
-    </row>
-    <row r="22" spans="1:574" ht="17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:558" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="83"/>
       <c r="B22" s="83"/>
       <c r="C22" s="83"/>
@@ -28798,28 +28654,9 @@
       <c r="P22" s="83"/>
       <c r="Q22" s="83"/>
       <c r="R22" s="83"/>
-      <c r="S22" s="83"/>
-      <c r="T22" s="83"/>
-      <c r="U22" s="83"/>
-      <c r="V22" s="83"/>
-      <c r="W22" s="83"/>
-      <c r="X22" s="83"/>
-      <c r="Y22" s="83"/>
-      <c r="Z22" s="83"/>
-      <c r="AA22" s="83"/>
-      <c r="AB22" s="83"/>
-      <c r="AC22" s="83"/>
-      <c r="AD22" s="83"/>
-      <c r="AE22" s="83"/>
-      <c r="AF22" s="83"/>
-      <c r="AG22" s="83"/>
-      <c r="AH22" s="83"/>
-      <c r="VB22" s="82">
-        <f>AVERAGEIF(Monthly!$B$4:$B$461,$A2,Monthly!D$4:D$461)</f>
-        <v>100.16549999999999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:574" x14ac:dyDescent="0.2">
+      <c r="UL22" s="82"/>
+    </row>
+    <row r="23" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A23" s="83"/>
       <c r="B23" s="83"/>
       <c r="C23" s="83"/>
@@ -28838,24 +28675,8 @@
       <c r="P23" s="83"/>
       <c r="Q23" s="83"/>
       <c r="R23" s="83"/>
-      <c r="S23" s="83"/>
-      <c r="T23" s="83"/>
-      <c r="U23" s="83"/>
-      <c r="V23" s="83"/>
-      <c r="W23" s="83"/>
-      <c r="X23" s="83"/>
-      <c r="Y23" s="83"/>
-      <c r="Z23" s="83"/>
-      <c r="AA23" s="83"/>
-      <c r="AB23" s="83"/>
-      <c r="AC23" s="83"/>
-      <c r="AD23" s="83"/>
-      <c r="AE23" s="83"/>
-      <c r="AF23" s="83"/>
-      <c r="AG23" s="83"/>
-      <c r="AH23" s="83"/>
-    </row>
-    <row r="24" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A24" s="83"/>
       <c r="B24" s="83"/>
       <c r="C24" s="83"/>
@@ -28874,24 +28695,8 @@
       <c r="P24" s="83"/>
       <c r="Q24" s="83"/>
       <c r="R24" s="83"/>
-      <c r="S24" s="83"/>
-      <c r="T24" s="83"/>
-      <c r="U24" s="83"/>
-      <c r="V24" s="83"/>
-      <c r="W24" s="83"/>
-      <c r="X24" s="83"/>
-      <c r="Y24" s="83"/>
-      <c r="Z24" s="83"/>
-      <c r="AA24" s="83"/>
-      <c r="AB24" s="83"/>
-      <c r="AC24" s="83"/>
-      <c r="AD24" s="83"/>
-      <c r="AE24" s="83"/>
-      <c r="AF24" s="83"/>
-      <c r="AG24" s="83"/>
-      <c r="AH24" s="83"/>
-    </row>
-    <row r="25" spans="1:574" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:558" x14ac:dyDescent="0.2">
       <c r="A25" s="83"/>
       <c r="B25" s="83"/>
       <c r="C25" s="83"/>
@@ -28910,22 +28715,6 @@
       <c r="P25" s="83"/>
       <c r="Q25" s="83"/>
       <c r="R25" s="83"/>
-      <c r="S25" s="83"/>
-      <c r="T25" s="83"/>
-      <c r="U25" s="83"/>
-      <c r="V25" s="83"/>
-      <c r="W25" s="83"/>
-      <c r="X25" s="83"/>
-      <c r="Y25" s="83"/>
-      <c r="Z25" s="83"/>
-      <c r="AA25" s="83"/>
-      <c r="AB25" s="83"/>
-      <c r="AC25" s="83"/>
-      <c r="AD25" s="83"/>
-      <c r="AE25" s="83"/>
-      <c r="AF25" s="83"/>
-      <c r="AG25" s="83"/>
-      <c r="AH25" s="83"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -28934,12 +28723,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21DB90F7-3BE6-A64F-8333-62671F03D732}">
-  <dimension ref="A1:AE85"/>
+  <dimension ref="A1:AE84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="83" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B1" s="83" t="s">
         <v>118</v>
@@ -28983,26 +28772,13 @@
       <c r="O1" s="83" t="s">
         <v>131</v>
       </c>
-      <c r="P1" s="83"/>
-      <c r="Q1" s="83"/>
-      <c r="R1" s="83"/>
-      <c r="S1" s="83"/>
-      <c r="T1" s="83"/>
-      <c r="U1" s="83"/>
-      <c r="V1" s="83"/>
-      <c r="W1" s="83"/>
-      <c r="X1" s="83"/>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="83"/>
-      <c r="AA1" s="83"/>
-      <c r="AB1" s="83"/>
-      <c r="AC1" s="83"/>
-      <c r="AD1" s="83"/>
-      <c r="AE1" s="83"/>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P1" s="83" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="83">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="B2" s="83">
         <f>('Financial Year Averages'!B3-'Financial Year Averages'!B2)/'Financial Year Averages'!B2*100</f>
@@ -29060,26 +28836,14 @@
         <f>('Financial Year Averages'!O3-'Financial Year Averages'!O2)/'Financial Year Averages'!O2*100</f>
         <v>1.3310520341400587</v>
       </c>
-      <c r="P2" s="83"/>
-      <c r="Q2" s="83"/>
-      <c r="R2" s="83"/>
-      <c r="S2" s="83"/>
-      <c r="T2" s="83"/>
-      <c r="U2" s="83"/>
-      <c r="V2" s="83"/>
-      <c r="W2" s="83"/>
-      <c r="X2" s="83"/>
-      <c r="Y2" s="83"/>
-      <c r="Z2" s="83"/>
-      <c r="AA2" s="83"/>
-      <c r="AB2" s="83"/>
-      <c r="AC2" s="83"/>
-      <c r="AD2" s="83"/>
-      <c r="AE2" s="83"/>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P2" s="83">
+        <f>('Financial Year Averages'!P3-'Financial Year Averages'!P2)/'Financial Year Averages'!P2*100</f>
+        <v>-1.7955644146423033</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="83">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B3" s="83">
         <f>('Financial Year Averages'!B4-'Financial Year Averages'!B3)/'Financial Year Averages'!B3*100</f>
@@ -29137,26 +28901,14 @@
         <f>('Financial Year Averages'!O4-'Financial Year Averages'!O3)/'Financial Year Averages'!O3*100</f>
         <v>0.72634875844657687</v>
       </c>
-      <c r="P3" s="83"/>
-      <c r="Q3" s="83"/>
-      <c r="R3" s="83"/>
-      <c r="S3" s="83"/>
-      <c r="T3" s="83"/>
-      <c r="U3" s="83"/>
-      <c r="V3" s="83"/>
-      <c r="W3" s="83"/>
-      <c r="X3" s="83"/>
-      <c r="Y3" s="83"/>
-      <c r="Z3" s="83"/>
-      <c r="AA3" s="83"/>
-      <c r="AB3" s="83"/>
-      <c r="AC3" s="83"/>
-      <c r="AD3" s="83"/>
-      <c r="AE3" s="83"/>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P3" s="83">
+        <f>('Financial Year Averages'!P4-'Financial Year Averages'!P3)/'Financial Year Averages'!P3*100</f>
+        <v>5.3800104915604869</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="83">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B4" s="83">
         <f>('Financial Year Averages'!B5-'Financial Year Averages'!B4)/'Financial Year Averages'!B4*100</f>
@@ -29214,26 +28966,14 @@
         <f>('Financial Year Averages'!O5-'Financial Year Averages'!O4)/'Financial Year Averages'!O4*100</f>
         <v>0.54375139828737284</v>
       </c>
-      <c r="P4" s="83"/>
-      <c r="Q4" s="83"/>
-      <c r="R4" s="83"/>
-      <c r="S4" s="83"/>
-      <c r="T4" s="83"/>
-      <c r="U4" s="83"/>
-      <c r="V4" s="83"/>
-      <c r="W4" s="83"/>
-      <c r="X4" s="83"/>
-      <c r="Y4" s="83"/>
-      <c r="Z4" s="83"/>
-      <c r="AA4" s="83"/>
-      <c r="AB4" s="83"/>
-      <c r="AC4" s="83"/>
-      <c r="AD4" s="83"/>
-      <c r="AE4" s="83"/>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P4" s="83">
+        <f>('Financial Year Averages'!P5-'Financial Year Averages'!P4)/'Financial Year Averages'!P4*100</f>
+        <v>5.5959811878465882</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="83">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B5" s="83">
         <f>('Financial Year Averages'!B6-'Financial Year Averages'!B5)/'Financial Year Averages'!B5*100</f>
@@ -29291,26 +29031,14 @@
         <f>('Financial Year Averages'!O6-'Financial Year Averages'!O5)/'Financial Year Averages'!O5*100</f>
         <v>0.75518397884487132</v>
       </c>
-      <c r="P5" s="83"/>
-      <c r="Q5" s="83"/>
-      <c r="R5" s="83"/>
-      <c r="S5" s="83"/>
-      <c r="T5" s="83"/>
-      <c r="U5" s="83"/>
-      <c r="V5" s="83"/>
-      <c r="W5" s="83"/>
-      <c r="X5" s="83"/>
-      <c r="Y5" s="83"/>
-      <c r="Z5" s="83"/>
-      <c r="AA5" s="83"/>
-      <c r="AB5" s="83"/>
-      <c r="AC5" s="83"/>
-      <c r="AD5" s="83"/>
-      <c r="AE5" s="83"/>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P5" s="83">
+        <f>('Financial Year Averages'!P6-'Financial Year Averages'!P5)/'Financial Year Averages'!P5*100</f>
+        <v>4.3247040554114307</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="83">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B6" s="83">
         <f>('Financial Year Averages'!B7-'Financial Year Averages'!B6)/'Financial Year Averages'!B6*100</f>
@@ -29368,26 +29096,14 @@
         <f>('Financial Year Averages'!O7-'Financial Year Averages'!O6)/'Financial Year Averages'!O6*100</f>
         <v>1.6716450872870463</v>
       </c>
-      <c r="P6" s="83"/>
-      <c r="Q6" s="83"/>
-      <c r="R6" s="83"/>
-      <c r="S6" s="83"/>
-      <c r="T6" s="83"/>
-      <c r="U6" s="83"/>
-      <c r="V6" s="83"/>
-      <c r="W6" s="83"/>
-      <c r="X6" s="83"/>
-      <c r="Y6" s="83"/>
-      <c r="Z6" s="83"/>
-      <c r="AA6" s="83"/>
-      <c r="AB6" s="83"/>
-      <c r="AC6" s="83"/>
-      <c r="AD6" s="83"/>
-      <c r="AE6" s="83"/>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P6" s="83">
+        <f>('Financial Year Averages'!P7-'Financial Year Averages'!P6)/'Financial Year Averages'!P6*100</f>
+        <v>-7.438937948551354</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="83">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B7" s="83">
         <f>('Financial Year Averages'!B8-'Financial Year Averages'!B7)/'Financial Year Averages'!B7*100</f>
@@ -29445,26 +29161,14 @@
         <f>('Financial Year Averages'!O8-'Financial Year Averages'!O7)/'Financial Year Averages'!O7*100</f>
         <v>1.8179342650584014</v>
       </c>
-      <c r="P7" s="83"/>
-      <c r="Q7" s="83"/>
-      <c r="R7" s="83"/>
-      <c r="S7" s="83"/>
-      <c r="T7" s="83"/>
-      <c r="U7" s="83"/>
-      <c r="V7" s="83"/>
-      <c r="W7" s="83"/>
-      <c r="X7" s="83"/>
-      <c r="Y7" s="83"/>
-      <c r="Z7" s="83"/>
-      <c r="AA7" s="83"/>
-      <c r="AB7" s="83"/>
-      <c r="AC7" s="83"/>
-      <c r="AD7" s="83"/>
-      <c r="AE7" s="83"/>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P7" s="83">
+        <f>('Financial Year Averages'!P8-'Financial Year Averages'!P7)/'Financial Year Averages'!P7*100</f>
+        <v>12.848254241749846</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="83">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B8" s="83">
         <f>('Financial Year Averages'!B9-'Financial Year Averages'!B8)/'Financial Year Averages'!B8*100</f>
@@ -29522,26 +29226,14 @@
         <f>('Financial Year Averages'!O9-'Financial Year Averages'!O8)/'Financial Year Averages'!O8*100</f>
         <v>4.0575334481961756</v>
       </c>
-      <c r="P8" s="83"/>
-      <c r="Q8" s="83"/>
-      <c r="R8" s="83"/>
-      <c r="S8" s="83"/>
-      <c r="T8" s="83"/>
-      <c r="U8" s="83"/>
-      <c r="V8" s="83"/>
-      <c r="W8" s="83"/>
-      <c r="X8" s="83"/>
-      <c r="Y8" s="83"/>
-      <c r="Z8" s="83"/>
-      <c r="AA8" s="83"/>
-      <c r="AB8" s="83"/>
-      <c r="AC8" s="83"/>
-      <c r="AD8" s="83"/>
-      <c r="AE8" s="83"/>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P8" s="83">
+        <f>('Financial Year Averages'!P9-'Financial Year Averages'!P8)/'Financial Year Averages'!P8*100</f>
+        <v>79.072325343523602</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="83">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B9" s="83">
         <f>('Financial Year Averages'!B10-'Financial Year Averages'!B9)/'Financial Year Averages'!B9*100</f>
@@ -29599,101 +29291,29 @@
         <f>('Financial Year Averages'!O10-'Financial Year Averages'!O9)/'Financial Year Averages'!O9*100</f>
         <v>6.2927775012813489</v>
       </c>
-      <c r="P9" s="83"/>
-      <c r="Q9" s="83"/>
-      <c r="R9" s="83"/>
-      <c r="S9" s="83"/>
-      <c r="T9" s="83"/>
-      <c r="U9" s="83"/>
-      <c r="V9" s="83"/>
-      <c r="W9" s="83"/>
-      <c r="X9" s="83"/>
-      <c r="Y9" s="83"/>
-      <c r="Z9" s="83"/>
-      <c r="AA9" s="83"/>
-      <c r="AB9" s="83"/>
-      <c r="AC9" s="83"/>
-      <c r="AD9" s="83"/>
-      <c r="AE9" s="83"/>
-    </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A10" s="83">
-        <v>2023</v>
-      </c>
-      <c r="B10" s="83">
-        <f>('Financial Year Averages'!B11-'Financial Year Averages'!B10)/'Financial Year Averages'!B10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="C10" s="83">
-        <f>('Financial Year Averages'!C11-'Financial Year Averages'!C10)/'Financial Year Averages'!C10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="D10" s="83">
-        <f>('Financial Year Averages'!D11-'Financial Year Averages'!D10)/'Financial Year Averages'!D10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="E10" s="83">
-        <f>('Financial Year Averages'!E11-'Financial Year Averages'!E10)/'Financial Year Averages'!E10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="F10" s="83">
-        <f>('Financial Year Averages'!F11-'Financial Year Averages'!F10)/'Financial Year Averages'!F10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="G10" s="83">
-        <f>('Financial Year Averages'!G11-'Financial Year Averages'!G10)/'Financial Year Averages'!G10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="H10" s="83">
-        <f>('Financial Year Averages'!H11-'Financial Year Averages'!H10)/'Financial Year Averages'!H10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="I10" s="83">
-        <f>('Financial Year Averages'!I11-'Financial Year Averages'!I10)/'Financial Year Averages'!I10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="J10" s="83">
-        <f>('Financial Year Averages'!J11-'Financial Year Averages'!J10)/'Financial Year Averages'!J10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="K10" s="83">
-        <f>('Financial Year Averages'!K11-'Financial Year Averages'!K10)/'Financial Year Averages'!K10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="L10" s="83">
-        <f>('Financial Year Averages'!L11-'Financial Year Averages'!L10)/'Financial Year Averages'!L10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="M10" s="83">
-        <f>('Financial Year Averages'!M11-'Financial Year Averages'!M10)/'Financial Year Averages'!M10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="N10" s="83">
-        <f>('Financial Year Averages'!N11-'Financial Year Averages'!N10)/'Financial Year Averages'!N10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="O10" s="83">
-        <f>('Financial Year Averages'!O11-'Financial Year Averages'!O10)/'Financial Year Averages'!O10*100</f>
-        <v>-100</v>
-      </c>
-      <c r="P10" s="83"/>
-      <c r="Q10" s="83"/>
-      <c r="R10" s="83"/>
-      <c r="S10" s="83"/>
-      <c r="T10" s="83"/>
-      <c r="U10" s="83"/>
-      <c r="V10" s="83"/>
-      <c r="W10" s="83"/>
-      <c r="X10" s="83"/>
-      <c r="Y10" s="83"/>
-      <c r="Z10" s="83"/>
-      <c r="AA10" s="83"/>
-      <c r="AB10" s="83"/>
-      <c r="AC10" s="83"/>
-      <c r="AD10" s="83"/>
-      <c r="AE10" s="83"/>
-    </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="P9" s="83">
+        <f>('Financial Year Averages'!P10-'Financial Year Averages'!P9)/'Financial Year Averages'!P9*100</f>
+        <v>-4.9158507003724106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A10" s="83"/>
+      <c r="B10" s="83"/>
+      <c r="C10" s="83"/>
+      <c r="D10" s="83"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83"/>
+      <c r="G10" s="83"/>
+      <c r="H10" s="83"/>
+      <c r="I10" s="83"/>
+      <c r="J10" s="83"/>
+      <c r="K10" s="83"/>
+      <c r="L10" s="83"/>
+      <c r="M10" s="83"/>
+      <c r="N10" s="83"/>
+      <c r="O10" s="83"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="83"/>
       <c r="B11" s="83"/>
       <c r="C11" s="83"/>
@@ -29709,24 +29329,8 @@
       <c r="M11" s="83"/>
       <c r="N11" s="83"/>
       <c r="O11" s="83"/>
-      <c r="P11" s="83"/>
-      <c r="Q11" s="83"/>
-      <c r="R11" s="83"/>
-      <c r="S11" s="83"/>
-      <c r="T11" s="83"/>
-      <c r="U11" s="83"/>
-      <c r="V11" s="83"/>
-      <c r="W11" s="83"/>
-      <c r="X11" s="83"/>
-      <c r="Y11" s="83"/>
-      <c r="Z11" s="83"/>
-      <c r="AA11" s="83"/>
-      <c r="AB11" s="83"/>
-      <c r="AC11" s="83"/>
-      <c r="AD11" s="83"/>
-      <c r="AE11" s="83"/>
-    </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="83"/>
       <c r="B12" s="83"/>
       <c r="C12" s="83"/>
@@ -29742,24 +29346,8 @@
       <c r="M12" s="83"/>
       <c r="N12" s="83"/>
       <c r="O12" s="83"/>
-      <c r="P12" s="83"/>
-      <c r="Q12" s="83"/>
-      <c r="R12" s="83"/>
-      <c r="S12" s="83"/>
-      <c r="T12" s="83"/>
-      <c r="U12" s="83"/>
-      <c r="V12" s="83"/>
-      <c r="W12" s="83"/>
-      <c r="X12" s="83"/>
-      <c r="Y12" s="83"/>
-      <c r="Z12" s="83"/>
-      <c r="AA12" s="83"/>
-      <c r="AB12" s="83"/>
-      <c r="AC12" s="83"/>
-      <c r="AD12" s="83"/>
-      <c r="AE12" s="83"/>
-    </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="83"/>
       <c r="B13" s="83"/>
       <c r="C13" s="83"/>
@@ -29775,24 +29363,8 @@
       <c r="M13" s="83"/>
       <c r="N13" s="83"/>
       <c r="O13" s="83"/>
-      <c r="P13" s="83"/>
-      <c r="Q13" s="83"/>
-      <c r="R13" s="83"/>
-      <c r="S13" s="83"/>
-      <c r="T13" s="83"/>
-      <c r="U13" s="83"/>
-      <c r="V13" s="83"/>
-      <c r="W13" s="83"/>
-      <c r="X13" s="83"/>
-      <c r="Y13" s="83"/>
-      <c r="Z13" s="83"/>
-      <c r="AA13" s="83"/>
-      <c r="AB13" s="83"/>
-      <c r="AC13" s="83"/>
-      <c r="AD13" s="83"/>
-      <c r="AE13" s="83"/>
-    </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="83"/>
       <c r="B14" s="83"/>
       <c r="C14" s="83"/>
@@ -29808,24 +29380,8 @@
       <c r="M14" s="83"/>
       <c r="N14" s="83"/>
       <c r="O14" s="83"/>
-      <c r="P14" s="83"/>
-      <c r="Q14" s="83"/>
-      <c r="R14" s="83"/>
-      <c r="S14" s="83"/>
-      <c r="T14" s="83"/>
-      <c r="U14" s="83"/>
-      <c r="V14" s="83"/>
-      <c r="W14" s="83"/>
-      <c r="X14" s="83"/>
-      <c r="Y14" s="83"/>
-      <c r="Z14" s="83"/>
-      <c r="AA14" s="83"/>
-      <c r="AB14" s="83"/>
-      <c r="AC14" s="83"/>
-      <c r="AD14" s="83"/>
-      <c r="AE14" s="83"/>
-    </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="83"/>
       <c r="B15" s="83"/>
       <c r="C15" s="83"/>
@@ -29841,24 +29397,8 @@
       <c r="M15" s="83"/>
       <c r="N15" s="83"/>
       <c r="O15" s="83"/>
-      <c r="P15" s="83"/>
-      <c r="Q15" s="83"/>
-      <c r="R15" s="83"/>
-      <c r="S15" s="83"/>
-      <c r="T15" s="83"/>
-      <c r="U15" s="83"/>
-      <c r="V15" s="83"/>
-      <c r="W15" s="83"/>
-      <c r="X15" s="83"/>
-      <c r="Y15" s="83"/>
-      <c r="Z15" s="83"/>
-      <c r="AA15" s="83"/>
-      <c r="AB15" s="83"/>
-      <c r="AC15" s="83"/>
-      <c r="AD15" s="83"/>
-      <c r="AE15" s="83"/>
-    </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="83"/>
       <c r="B16" s="83"/>
       <c r="C16" s="83"/>
@@ -29874,24 +29414,8 @@
       <c r="M16" s="83"/>
       <c r="N16" s="83"/>
       <c r="O16" s="83"/>
-      <c r="P16" s="83"/>
-      <c r="Q16" s="83"/>
-      <c r="R16" s="83"/>
-      <c r="S16" s="83"/>
-      <c r="T16" s="83"/>
-      <c r="U16" s="83"/>
-      <c r="V16" s="83"/>
-      <c r="W16" s="83"/>
-      <c r="X16" s="83"/>
-      <c r="Y16" s="83"/>
-      <c r="Z16" s="83"/>
-      <c r="AA16" s="83"/>
-      <c r="AB16" s="83"/>
-      <c r="AC16" s="83"/>
-      <c r="AD16" s="83"/>
-      <c r="AE16" s="83"/>
-    </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="83"/>
       <c r="B17" s="83"/>
       <c r="C17" s="83"/>
@@ -29907,24 +29431,8 @@
       <c r="M17" s="83"/>
       <c r="N17" s="83"/>
       <c r="O17" s="83"/>
-      <c r="P17" s="83"/>
-      <c r="Q17" s="83"/>
-      <c r="R17" s="83"/>
-      <c r="S17" s="83"/>
-      <c r="T17" s="83"/>
-      <c r="U17" s="83"/>
-      <c r="V17" s="83"/>
-      <c r="W17" s="83"/>
-      <c r="X17" s="83"/>
-      <c r="Y17" s="83"/>
-      <c r="Z17" s="83"/>
-      <c r="AA17" s="83"/>
-      <c r="AB17" s="83"/>
-      <c r="AC17" s="83"/>
-      <c r="AD17" s="83"/>
-      <c r="AE17" s="83"/>
-    </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="83"/>
       <c r="B18" s="83"/>
       <c r="C18" s="83"/>
@@ -29940,24 +29448,8 @@
       <c r="M18" s="83"/>
       <c r="N18" s="83"/>
       <c r="O18" s="83"/>
-      <c r="P18" s="83"/>
-      <c r="Q18" s="83"/>
-      <c r="R18" s="83"/>
-      <c r="S18" s="83"/>
-      <c r="T18" s="83"/>
-      <c r="U18" s="83"/>
-      <c r="V18" s="83"/>
-      <c r="W18" s="83"/>
-      <c r="X18" s="83"/>
-      <c r="Y18" s="83"/>
-      <c r="Z18" s="83"/>
-      <c r="AA18" s="83"/>
-      <c r="AB18" s="83"/>
-      <c r="AC18" s="83"/>
-      <c r="AD18" s="83"/>
-      <c r="AE18" s="83"/>
-    </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="83"/>
       <c r="B19" s="83"/>
       <c r="C19" s="83"/>
@@ -29973,24 +29465,8 @@
       <c r="M19" s="83"/>
       <c r="N19" s="83"/>
       <c r="O19" s="83"/>
-      <c r="P19" s="83"/>
-      <c r="Q19" s="83"/>
-      <c r="R19" s="83"/>
-      <c r="S19" s="83"/>
-      <c r="T19" s="83"/>
-      <c r="U19" s="83"/>
-      <c r="V19" s="83"/>
-      <c r="W19" s="83"/>
-      <c r="X19" s="83"/>
-      <c r="Y19" s="83"/>
-      <c r="Z19" s="83"/>
-      <c r="AA19" s="83"/>
-      <c r="AB19" s="83"/>
-      <c r="AC19" s="83"/>
-      <c r="AD19" s="83"/>
-      <c r="AE19" s="83"/>
-    </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="83"/>
       <c r="B20" s="83"/>
       <c r="C20" s="83"/>
@@ -30006,24 +29482,8 @@
       <c r="M20" s="83"/>
       <c r="N20" s="83"/>
       <c r="O20" s="83"/>
-      <c r="P20" s="83"/>
-      <c r="Q20" s="83"/>
-      <c r="R20" s="83"/>
-      <c r="S20" s="83"/>
-      <c r="T20" s="83"/>
-      <c r="U20" s="83"/>
-      <c r="V20" s="83"/>
-      <c r="W20" s="83"/>
-      <c r="X20" s="83"/>
-      <c r="Y20" s="83"/>
-      <c r="Z20" s="83"/>
-      <c r="AA20" s="83"/>
-      <c r="AB20" s="83"/>
-      <c r="AC20" s="83"/>
-      <c r="AD20" s="83"/>
-      <c r="AE20" s="83"/>
-    </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="83"/>
       <c r="B21" s="83"/>
       <c r="C21" s="83"/>
@@ -30039,24 +29499,8 @@
       <c r="M21" s="83"/>
       <c r="N21" s="83"/>
       <c r="O21" s="83"/>
-      <c r="P21" s="83"/>
-      <c r="Q21" s="83"/>
-      <c r="R21" s="83"/>
-      <c r="S21" s="83"/>
-      <c r="T21" s="83"/>
-      <c r="U21" s="83"/>
-      <c r="V21" s="83"/>
-      <c r="W21" s="83"/>
-      <c r="X21" s="83"/>
-      <c r="Y21" s="83"/>
-      <c r="Z21" s="83"/>
-      <c r="AA21" s="83"/>
-      <c r="AB21" s="83"/>
-      <c r="AC21" s="83"/>
-      <c r="AD21" s="83"/>
-      <c r="AE21" s="83"/>
-    </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="83"/>
       <c r="B22" s="83"/>
       <c r="C22" s="83"/>
@@ -30072,24 +29516,8 @@
       <c r="M22" s="83"/>
       <c r="N22" s="83"/>
       <c r="O22" s="83"/>
-      <c r="P22" s="83"/>
-      <c r="Q22" s="83"/>
-      <c r="R22" s="83"/>
-      <c r="S22" s="83"/>
-      <c r="T22" s="83"/>
-      <c r="U22" s="83"/>
-      <c r="V22" s="83"/>
-      <c r="W22" s="83"/>
-      <c r="X22" s="83"/>
-      <c r="Y22" s="83"/>
-      <c r="Z22" s="83"/>
-      <c r="AA22" s="83"/>
-      <c r="AB22" s="83"/>
-      <c r="AC22" s="83"/>
-      <c r="AD22" s="83"/>
-      <c r="AE22" s="83"/>
-    </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="83"/>
       <c r="B23" s="83"/>
       <c r="C23" s="83"/>
@@ -30105,24 +29533,8 @@
       <c r="M23" s="83"/>
       <c r="N23" s="83"/>
       <c r="O23" s="83"/>
-      <c r="P23" s="83"/>
-      <c r="Q23" s="83"/>
-      <c r="R23" s="83"/>
-      <c r="S23" s="83"/>
-      <c r="T23" s="83"/>
-      <c r="U23" s="83"/>
-      <c r="V23" s="83"/>
-      <c r="W23" s="83"/>
-      <c r="X23" s="83"/>
-      <c r="Y23" s="83"/>
-      <c r="Z23" s="83"/>
-      <c r="AA23" s="83"/>
-      <c r="AB23" s="83"/>
-      <c r="AC23" s="83"/>
-      <c r="AD23" s="83"/>
-      <c r="AE23" s="83"/>
-    </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="83"/>
       <c r="B24" s="83"/>
       <c r="C24" s="83"/>
@@ -30138,24 +29550,8 @@
       <c r="M24" s="83"/>
       <c r="N24" s="83"/>
       <c r="O24" s="83"/>
-      <c r="P24" s="83"/>
-      <c r="Q24" s="83"/>
-      <c r="R24" s="83"/>
-      <c r="S24" s="83"/>
-      <c r="T24" s="83"/>
-      <c r="U24" s="83"/>
-      <c r="V24" s="83"/>
-      <c r="W24" s="83"/>
-      <c r="X24" s="83"/>
-      <c r="Y24" s="83"/>
-      <c r="Z24" s="83"/>
-      <c r="AA24" s="83"/>
-      <c r="AB24" s="83"/>
-      <c r="AC24" s="83"/>
-      <c r="AD24" s="83"/>
-      <c r="AE24" s="83"/>
-    </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="83"/>
       <c r="B25" s="83"/>
       <c r="C25" s="83"/>
@@ -30171,24 +29567,8 @@
       <c r="M25" s="83"/>
       <c r="N25" s="83"/>
       <c r="O25" s="83"/>
-      <c r="P25" s="83"/>
-      <c r="Q25" s="83"/>
-      <c r="R25" s="83"/>
-      <c r="S25" s="83"/>
-      <c r="T25" s="83"/>
-      <c r="U25" s="83"/>
-      <c r="V25" s="83"/>
-      <c r="W25" s="83"/>
-      <c r="X25" s="83"/>
-      <c r="Y25" s="83"/>
-      <c r="Z25" s="83"/>
-      <c r="AA25" s="83"/>
-      <c r="AB25" s="83"/>
-      <c r="AC25" s="83"/>
-      <c r="AD25" s="83"/>
-      <c r="AE25" s="83"/>
-    </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="83"/>
       <c r="B26" s="83"/>
       <c r="C26" s="83"/>
@@ -30204,24 +29584,8 @@
       <c r="M26" s="83"/>
       <c r="N26" s="83"/>
       <c r="O26" s="83"/>
-      <c r="P26" s="83"/>
-      <c r="Q26" s="83"/>
-      <c r="R26" s="83"/>
-      <c r="S26" s="83"/>
-      <c r="T26" s="83"/>
-      <c r="U26" s="83"/>
-      <c r="V26" s="83"/>
-      <c r="W26" s="83"/>
-      <c r="X26" s="83"/>
-      <c r="Y26" s="83"/>
-      <c r="Z26" s="83"/>
-      <c r="AA26" s="83"/>
-      <c r="AB26" s="83"/>
-      <c r="AC26" s="83"/>
-      <c r="AD26" s="83"/>
-      <c r="AE26" s="83"/>
-    </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="83"/>
       <c r="B27" s="83"/>
       <c r="C27" s="83"/>
@@ -30237,24 +29601,8 @@
       <c r="M27" s="83"/>
       <c r="N27" s="83"/>
       <c r="O27" s="83"/>
-      <c r="P27" s="83"/>
-      <c r="Q27" s="83"/>
-      <c r="R27" s="83"/>
-      <c r="S27" s="83"/>
-      <c r="T27" s="83"/>
-      <c r="U27" s="83"/>
-      <c r="V27" s="83"/>
-      <c r="W27" s="83"/>
-      <c r="X27" s="83"/>
-      <c r="Y27" s="83"/>
-      <c r="Z27" s="83"/>
-      <c r="AA27" s="83"/>
-      <c r="AB27" s="83"/>
-      <c r="AC27" s="83"/>
-      <c r="AD27" s="83"/>
-      <c r="AE27" s="83"/>
-    </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="83"/>
       <c r="B28" s="83"/>
       <c r="C28" s="83"/>
@@ -30270,24 +29618,8 @@
       <c r="M28" s="83"/>
       <c r="N28" s="83"/>
       <c r="O28" s="83"/>
-      <c r="P28" s="83"/>
-      <c r="Q28" s="83"/>
-      <c r="R28" s="83"/>
-      <c r="S28" s="83"/>
-      <c r="T28" s="83"/>
-      <c r="U28" s="83"/>
-      <c r="V28" s="83"/>
-      <c r="W28" s="83"/>
-      <c r="X28" s="83"/>
-      <c r="Y28" s="83"/>
-      <c r="Z28" s="83"/>
-      <c r="AA28" s="83"/>
-      <c r="AB28" s="83"/>
-      <c r="AC28" s="83"/>
-      <c r="AD28" s="83"/>
-      <c r="AE28" s="83"/>
-    </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="83"/>
       <c r="B29" s="83"/>
       <c r="C29" s="83"/>
@@ -30303,24 +29635,8 @@
       <c r="M29" s="83"/>
       <c r="N29" s="83"/>
       <c r="O29" s="83"/>
-      <c r="P29" s="83"/>
-      <c r="Q29" s="83"/>
-      <c r="R29" s="83"/>
-      <c r="S29" s="83"/>
-      <c r="T29" s="83"/>
-      <c r="U29" s="83"/>
-      <c r="V29" s="83"/>
-      <c r="W29" s="83"/>
-      <c r="X29" s="83"/>
-      <c r="Y29" s="83"/>
-      <c r="Z29" s="83"/>
-      <c r="AA29" s="83"/>
-      <c r="AB29" s="83"/>
-      <c r="AC29" s="83"/>
-      <c r="AD29" s="83"/>
-      <c r="AE29" s="83"/>
-    </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="83"/>
       <c r="B30" s="83"/>
       <c r="C30" s="83"/>
@@ -30336,24 +29652,8 @@
       <c r="M30" s="83"/>
       <c r="N30" s="83"/>
       <c r="O30" s="83"/>
-      <c r="P30" s="83"/>
-      <c r="Q30" s="83"/>
-      <c r="R30" s="83"/>
-      <c r="S30" s="83"/>
-      <c r="T30" s="83"/>
-      <c r="U30" s="83"/>
-      <c r="V30" s="83"/>
-      <c r="W30" s="83"/>
-      <c r="X30" s="83"/>
-      <c r="Y30" s="83"/>
-      <c r="Z30" s="83"/>
-      <c r="AA30" s="83"/>
-      <c r="AB30" s="83"/>
-      <c r="AC30" s="83"/>
-      <c r="AD30" s="83"/>
-      <c r="AE30" s="83"/>
-    </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="83"/>
       <c r="B31" s="83"/>
       <c r="C31" s="83"/>
@@ -30369,24 +29669,8 @@
       <c r="M31" s="83"/>
       <c r="N31" s="83"/>
       <c r="O31" s="83"/>
-      <c r="P31" s="83"/>
-      <c r="Q31" s="83"/>
-      <c r="R31" s="83"/>
-      <c r="S31" s="83"/>
-      <c r="T31" s="83"/>
-      <c r="U31" s="83"/>
-      <c r="V31" s="83"/>
-      <c r="W31" s="83"/>
-      <c r="X31" s="83"/>
-      <c r="Y31" s="83"/>
-      <c r="Z31" s="83"/>
-      <c r="AA31" s="83"/>
-      <c r="AB31" s="83"/>
-      <c r="AC31" s="83"/>
-      <c r="AD31" s="83"/>
-      <c r="AE31" s="83"/>
-    </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="83"/>
       <c r="B32" s="83"/>
       <c r="C32" s="83"/>
@@ -30402,22 +29686,6 @@
       <c r="M32" s="83"/>
       <c r="N32" s="83"/>
       <c r="O32" s="83"/>
-      <c r="P32" s="83"/>
-      <c r="Q32" s="83"/>
-      <c r="R32" s="83"/>
-      <c r="S32" s="83"/>
-      <c r="T32" s="83"/>
-      <c r="U32" s="83"/>
-      <c r="V32" s="83"/>
-      <c r="W32" s="83"/>
-      <c r="X32" s="83"/>
-      <c r="Y32" s="83"/>
-      <c r="Z32" s="83"/>
-      <c r="AA32" s="83"/>
-      <c r="AB32" s="83"/>
-      <c r="AC32" s="83"/>
-      <c r="AD32" s="83"/>
-      <c r="AE32" s="83"/>
     </row>
     <row r="33" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A33" s="83"/>
@@ -30435,22 +29703,6 @@
       <c r="M33" s="83"/>
       <c r="N33" s="83"/>
       <c r="O33" s="83"/>
-      <c r="P33" s="83"/>
-      <c r="Q33" s="83"/>
-      <c r="R33" s="83"/>
-      <c r="S33" s="83"/>
-      <c r="T33" s="83"/>
-      <c r="U33" s="83"/>
-      <c r="V33" s="83"/>
-      <c r="W33" s="83"/>
-      <c r="X33" s="83"/>
-      <c r="Y33" s="83"/>
-      <c r="Z33" s="83"/>
-      <c r="AA33" s="83"/>
-      <c r="AB33" s="83"/>
-      <c r="AC33" s="83"/>
-      <c r="AD33" s="83"/>
-      <c r="AE33" s="83"/>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A34" s="83"/>
@@ -30468,22 +29720,6 @@
       <c r="M34" s="83"/>
       <c r="N34" s="83"/>
       <c r="O34" s="83"/>
-      <c r="P34" s="83"/>
-      <c r="Q34" s="83"/>
-      <c r="R34" s="83"/>
-      <c r="S34" s="83"/>
-      <c r="T34" s="83"/>
-      <c r="U34" s="83"/>
-      <c r="V34" s="83"/>
-      <c r="W34" s="83"/>
-      <c r="X34" s="83"/>
-      <c r="Y34" s="83"/>
-      <c r="Z34" s="83"/>
-      <c r="AA34" s="83"/>
-      <c r="AB34" s="83"/>
-      <c r="AC34" s="83"/>
-      <c r="AD34" s="83"/>
-      <c r="AE34" s="83"/>
     </row>
     <row r="35" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A35" s="83"/>
@@ -30501,22 +29737,6 @@
       <c r="M35" s="83"/>
       <c r="N35" s="83"/>
       <c r="O35" s="83"/>
-      <c r="P35" s="83"/>
-      <c r="Q35" s="83"/>
-      <c r="R35" s="83"/>
-      <c r="S35" s="83"/>
-      <c r="T35" s="83"/>
-      <c r="U35" s="83"/>
-      <c r="V35" s="83"/>
-      <c r="W35" s="83"/>
-      <c r="X35" s="83"/>
-      <c r="Y35" s="83"/>
-      <c r="Z35" s="83"/>
-      <c r="AA35" s="83"/>
-      <c r="AB35" s="83"/>
-      <c r="AC35" s="83"/>
-      <c r="AD35" s="83"/>
-      <c r="AE35" s="83"/>
     </row>
     <row r="36" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A36" s="83"/>
@@ -30534,22 +29754,6 @@
       <c r="M36" s="83"/>
       <c r="N36" s="83"/>
       <c r="O36" s="83"/>
-      <c r="P36" s="83"/>
-      <c r="Q36" s="83"/>
-      <c r="R36" s="83"/>
-      <c r="S36" s="83"/>
-      <c r="T36" s="83"/>
-      <c r="U36" s="83"/>
-      <c r="V36" s="83"/>
-      <c r="W36" s="83"/>
-      <c r="X36" s="83"/>
-      <c r="Y36" s="83"/>
-      <c r="Z36" s="83"/>
-      <c r="AA36" s="83"/>
-      <c r="AB36" s="83"/>
-      <c r="AC36" s="83"/>
-      <c r="AD36" s="83"/>
-      <c r="AE36" s="83"/>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A37" s="83"/>
@@ -30567,22 +29771,6 @@
       <c r="M37" s="83"/>
       <c r="N37" s="83"/>
       <c r="O37" s="83"/>
-      <c r="P37" s="83"/>
-      <c r="Q37" s="83"/>
-      <c r="R37" s="83"/>
-      <c r="S37" s="83"/>
-      <c r="T37" s="83"/>
-      <c r="U37" s="83"/>
-      <c r="V37" s="83"/>
-      <c r="W37" s="83"/>
-      <c r="X37" s="83"/>
-      <c r="Y37" s="83"/>
-      <c r="Z37" s="83"/>
-      <c r="AA37" s="83"/>
-      <c r="AB37" s="83"/>
-      <c r="AC37" s="83"/>
-      <c r="AD37" s="83"/>
-      <c r="AE37" s="83"/>
     </row>
     <row r="38" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A38" s="83"/>
@@ -30600,22 +29788,6 @@
       <c r="M38" s="83"/>
       <c r="N38" s="83"/>
       <c r="O38" s="83"/>
-      <c r="P38" s="83"/>
-      <c r="Q38" s="83"/>
-      <c r="R38" s="83"/>
-      <c r="S38" s="83"/>
-      <c r="T38" s="83"/>
-      <c r="U38" s="83"/>
-      <c r="V38" s="83"/>
-      <c r="W38" s="83"/>
-      <c r="X38" s="83"/>
-      <c r="Y38" s="83"/>
-      <c r="Z38" s="83"/>
-      <c r="AA38" s="83"/>
-      <c r="AB38" s="83"/>
-      <c r="AC38" s="83"/>
-      <c r="AD38" s="83"/>
-      <c r="AE38" s="83"/>
     </row>
     <row r="39" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A39" s="83"/>
@@ -30633,22 +29805,6 @@
       <c r="M39" s="83"/>
       <c r="N39" s="83"/>
       <c r="O39" s="83"/>
-      <c r="P39" s="83"/>
-      <c r="Q39" s="83"/>
-      <c r="R39" s="83"/>
-      <c r="S39" s="83"/>
-      <c r="T39" s="83"/>
-      <c r="U39" s="83"/>
-      <c r="V39" s="83"/>
-      <c r="W39" s="83"/>
-      <c r="X39" s="83"/>
-      <c r="Y39" s="83"/>
-      <c r="Z39" s="83"/>
-      <c r="AA39" s="83"/>
-      <c r="AB39" s="83"/>
-      <c r="AC39" s="83"/>
-      <c r="AD39" s="83"/>
-      <c r="AE39" s="83"/>
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A40" s="83"/>
@@ -30666,22 +29822,6 @@
       <c r="M40" s="83"/>
       <c r="N40" s="83"/>
       <c r="O40" s="83"/>
-      <c r="P40" s="83"/>
-      <c r="Q40" s="83"/>
-      <c r="R40" s="83"/>
-      <c r="S40" s="83"/>
-      <c r="T40" s="83"/>
-      <c r="U40" s="83"/>
-      <c r="V40" s="83"/>
-      <c r="W40" s="83"/>
-      <c r="X40" s="83"/>
-      <c r="Y40" s="83"/>
-      <c r="Z40" s="83"/>
-      <c r="AA40" s="83"/>
-      <c r="AB40" s="83"/>
-      <c r="AC40" s="83"/>
-      <c r="AD40" s="83"/>
-      <c r="AE40" s="83"/>
     </row>
     <row r="41" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A41" s="83"/>
@@ -32135,39 +31275,6 @@
       <c r="AD84" s="83"/>
       <c r="AE84" s="83"/>
     </row>
-    <row r="85" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A85" s="83"/>
-      <c r="B85" s="83"/>
-      <c r="C85" s="83"/>
-      <c r="D85" s="83"/>
-      <c r="E85" s="83"/>
-      <c r="F85" s="83"/>
-      <c r="G85" s="83"/>
-      <c r="H85" s="83"/>
-      <c r="I85" s="83"/>
-      <c r="J85" s="83"/>
-      <c r="K85" s="83"/>
-      <c r="L85" s="83"/>
-      <c r="M85" s="83"/>
-      <c r="N85" s="83"/>
-      <c r="O85" s="83"/>
-      <c r="P85" s="83"/>
-      <c r="Q85" s="83"/>
-      <c r="R85" s="83"/>
-      <c r="S85" s="83"/>
-      <c r="T85" s="83"/>
-      <c r="U85" s="83"/>
-      <c r="V85" s="83"/>
-      <c r="W85" s="83"/>
-      <c r="X85" s="83"/>
-      <c r="Y85" s="83"/>
-      <c r="Z85" s="83"/>
-      <c r="AA85" s="83"/>
-      <c r="AB85" s="83"/>
-      <c r="AC85" s="83"/>
-      <c r="AD85" s="83"/>
-      <c r="AE85" s="83"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>